<commit_message>
Update draw scoring to 2 points in base .xlsx
</commit_message>
<xml_diff>
--- a/WorldCup2026_Sweepstake.xlsx
+++ b/WorldCup2026_Sweepstake.xlsx
@@ -706,9 +706,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -716,9 +714,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -747,9 +743,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
@@ -799,9 +793,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-    </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
@@ -830,9 +822,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-    </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
@@ -861,9 +851,7 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr"/>
-    </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
@@ -913,9 +901,7 @@
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr"/>
-    </row>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
@@ -1007,9 +993,7 @@
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr"/>
-    </row>
+    <row r="49"/>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
@@ -1052,9 +1036,7 @@
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="inlineStr"/>
-    </row>
+    <row r="56"/>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
@@ -1090,9 +1072,7 @@
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="inlineStr"/>
-    </row>
+    <row r="62"/>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
@@ -1154,7 +1134,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -3136,11 +3115,11 @@
         </is>
       </c>
       <c r="H5" s="19">
-        <f>IF(AND(E5&lt;&gt;"",F5&lt;&gt;""),IF(E5&gt;F5,3,IF(E5=F5,1,0)),"")</f>
+        <f>IF(AND(E5&lt;&gt;"",F5&lt;&gt;""),IF(E5&gt;F5,3,IF(E5=F5,2,0)),"")</f>
         <v/>
       </c>
       <c r="I5" s="19">
-        <f>IF(AND(E5&lt;&gt;"",F5&lt;&gt;""),IF(F5&gt;E5,3,IF(E5=F5,1,0)),"")</f>
+        <f>IF(AND(E5&lt;&gt;"",F5&lt;&gt;""),IF(F5&gt;E5,3,IF(E5=F5,2,0)),"")</f>
         <v/>
       </c>
       <c r="J5" s="19">
@@ -3179,11 +3158,11 @@
         </is>
       </c>
       <c r="H6" s="19">
-        <f>IF(AND(E6&lt;&gt;"",F6&lt;&gt;""),IF(E6&gt;F6,3,IF(E6=F6,1,0)),"")</f>
+        <f>IF(AND(E6&lt;&gt;"",F6&lt;&gt;""),IF(E6&gt;F6,3,IF(E6=F6,2,0)),"")</f>
         <v/>
       </c>
       <c r="I6" s="19">
-        <f>IF(AND(E6&lt;&gt;"",F6&lt;&gt;""),IF(F6&gt;E6,3,IF(E6=F6,1,0)),"")</f>
+        <f>IF(AND(E6&lt;&gt;"",F6&lt;&gt;""),IF(F6&gt;E6,3,IF(E6=F6,2,0)),"")</f>
         <v/>
       </c>
       <c r="J6" s="19">
@@ -3222,11 +3201,11 @@
         </is>
       </c>
       <c r="H7" s="21">
-        <f>IF(AND(E7&lt;&gt;"",F7&lt;&gt;""),IF(E7&gt;F7,3,IF(E7=F7,1,0)),"")</f>
+        <f>IF(AND(E7&lt;&gt;"",F7&lt;&gt;""),IF(E7&gt;F7,3,IF(E7=F7,2,0)),"")</f>
         <v/>
       </c>
       <c r="I7" s="21">
-        <f>IF(AND(E7&lt;&gt;"",F7&lt;&gt;""),IF(F7&gt;E7,3,IF(E7=F7,1,0)),"")</f>
+        <f>IF(AND(E7&lt;&gt;"",F7&lt;&gt;""),IF(F7&gt;E7,3,IF(E7=F7,2,0)),"")</f>
         <v/>
       </c>
       <c r="J7" s="21">
@@ -3265,11 +3244,11 @@
         </is>
       </c>
       <c r="H8" s="23">
-        <f>IF(AND(E8&lt;&gt;"",F8&lt;&gt;""),IF(E8&gt;F8,3,IF(E8=F8,1,0)),"")</f>
+        <f>IF(AND(E8&lt;&gt;"",F8&lt;&gt;""),IF(E8&gt;F8,3,IF(E8=F8,2,0)),"")</f>
         <v/>
       </c>
       <c r="I8" s="23">
-        <f>IF(AND(E8&lt;&gt;"",F8&lt;&gt;""),IF(F8&gt;E8,3,IF(E8=F8,1,0)),"")</f>
+        <f>IF(AND(E8&lt;&gt;"",F8&lt;&gt;""),IF(F8&gt;E8,3,IF(E8=F8,2,0)),"")</f>
         <v/>
       </c>
       <c r="J8" s="23">
@@ -3308,11 +3287,11 @@
         </is>
       </c>
       <c r="H9" s="25">
-        <f>IF(AND(E9&lt;&gt;"",F9&lt;&gt;""),IF(E9&gt;F9,3,IF(E9=F9,1,0)),"")</f>
+        <f>IF(AND(E9&lt;&gt;"",F9&lt;&gt;""),IF(E9&gt;F9,3,IF(E9=F9,2,0)),"")</f>
         <v/>
       </c>
       <c r="I9" s="25">
-        <f>IF(AND(E9&lt;&gt;"",F9&lt;&gt;""),IF(F9&gt;E9,3,IF(E9=F9,1,0)),"")</f>
+        <f>IF(AND(E9&lt;&gt;"",F9&lt;&gt;""),IF(F9&gt;E9,3,IF(E9=F9,2,0)),"")</f>
         <v/>
       </c>
       <c r="J9" s="25">
@@ -3351,11 +3330,11 @@
         </is>
       </c>
       <c r="H10" s="23">
-        <f>IF(AND(E10&lt;&gt;"",F10&lt;&gt;""),IF(E10&gt;F10,3,IF(E10=F10,1,0)),"")</f>
+        <f>IF(AND(E10&lt;&gt;"",F10&lt;&gt;""),IF(E10&gt;F10,3,IF(E10=F10,2,0)),"")</f>
         <v/>
       </c>
       <c r="I10" s="23">
-        <f>IF(AND(E10&lt;&gt;"",F10&lt;&gt;""),IF(F10&gt;E10,3,IF(E10=F10,1,0)),"")</f>
+        <f>IF(AND(E10&lt;&gt;"",F10&lt;&gt;""),IF(F10&gt;E10,3,IF(E10=F10,2,0)),"")</f>
         <v/>
       </c>
       <c r="J10" s="23">
@@ -3394,11 +3373,11 @@
         </is>
       </c>
       <c r="H11" s="25">
-        <f>IF(AND(E11&lt;&gt;"",F11&lt;&gt;""),IF(E11&gt;F11,3,IF(E11=F11,1,0)),"")</f>
+        <f>IF(AND(E11&lt;&gt;"",F11&lt;&gt;""),IF(E11&gt;F11,3,IF(E11=F11,2,0)),"")</f>
         <v/>
       </c>
       <c r="I11" s="25">
-        <f>IF(AND(E11&lt;&gt;"",F11&lt;&gt;""),IF(F11&gt;E11,3,IF(E11=F11,1,0)),"")</f>
+        <f>IF(AND(E11&lt;&gt;"",F11&lt;&gt;""),IF(F11&gt;E11,3,IF(E11=F11,2,0)),"")</f>
         <v/>
       </c>
       <c r="J11" s="25">
@@ -3437,11 +3416,11 @@
         </is>
       </c>
       <c r="H12" s="21">
-        <f>IF(AND(E12&lt;&gt;"",F12&lt;&gt;""),IF(E12&gt;F12,3,IF(E12=F12,1,0)),"")</f>
+        <f>IF(AND(E12&lt;&gt;"",F12&lt;&gt;""),IF(E12&gt;F12,3,IF(E12=F12,2,0)),"")</f>
         <v/>
       </c>
       <c r="I12" s="21">
-        <f>IF(AND(E12&lt;&gt;"",F12&lt;&gt;""),IF(F12&gt;E12,3,IF(E12=F12,1,0)),"")</f>
+        <f>IF(AND(E12&lt;&gt;"",F12&lt;&gt;""),IF(F12&gt;E12,3,IF(E12=F12,2,0)),"")</f>
         <v/>
       </c>
       <c r="J12" s="21">
@@ -3480,11 +3459,11 @@
         </is>
       </c>
       <c r="H13" s="27">
-        <f>IF(AND(E13&lt;&gt;"",F13&lt;&gt;""),IF(E13&gt;F13,3,IF(E13=F13,1,0)),"")</f>
+        <f>IF(AND(E13&lt;&gt;"",F13&lt;&gt;""),IF(E13&gt;F13,3,IF(E13=F13,2,0)),"")</f>
         <v/>
       </c>
       <c r="I13" s="27">
-        <f>IF(AND(E13&lt;&gt;"",F13&lt;&gt;""),IF(F13&gt;E13,3,IF(E13=F13,1,0)),"")</f>
+        <f>IF(AND(E13&lt;&gt;"",F13&lt;&gt;""),IF(F13&gt;E13,3,IF(E13=F13,2,0)),"")</f>
         <v/>
       </c>
       <c r="J13" s="27">
@@ -3523,11 +3502,11 @@
         </is>
       </c>
       <c r="H14" s="27">
-        <f>IF(AND(E14&lt;&gt;"",F14&lt;&gt;""),IF(E14&gt;F14,3,IF(E14=F14,1,0)),"")</f>
+        <f>IF(AND(E14&lt;&gt;"",F14&lt;&gt;""),IF(E14&gt;F14,3,IF(E14=F14,2,0)),"")</f>
         <v/>
       </c>
       <c r="I14" s="27">
-        <f>IF(AND(E14&lt;&gt;"",F14&lt;&gt;""),IF(F14&gt;E14,3,IF(E14=F14,1,0)),"")</f>
+        <f>IF(AND(E14&lt;&gt;"",F14&lt;&gt;""),IF(F14&gt;E14,3,IF(E14=F14,2,0)),"")</f>
         <v/>
       </c>
       <c r="J14" s="27">
@@ -3566,11 +3545,11 @@
         </is>
       </c>
       <c r="H15" s="29">
-        <f>IF(AND(E15&lt;&gt;"",F15&lt;&gt;""),IF(E15&gt;F15,3,IF(E15=F15,1,0)),"")</f>
+        <f>IF(AND(E15&lt;&gt;"",F15&lt;&gt;""),IF(E15&gt;F15,3,IF(E15=F15,2,0)),"")</f>
         <v/>
       </c>
       <c r="I15" s="29">
-        <f>IF(AND(E15&lt;&gt;"",F15&lt;&gt;""),IF(F15&gt;E15,3,IF(E15=F15,1,0)),"")</f>
+        <f>IF(AND(E15&lt;&gt;"",F15&lt;&gt;""),IF(F15&gt;E15,3,IF(E15=F15,2,0)),"")</f>
         <v/>
       </c>
       <c r="J15" s="29">
@@ -3609,11 +3588,11 @@
         </is>
       </c>
       <c r="H16" s="29">
-        <f>IF(AND(E16&lt;&gt;"",F16&lt;&gt;""),IF(E16&gt;F16,3,IF(E16=F16,1,0)),"")</f>
+        <f>IF(AND(E16&lt;&gt;"",F16&lt;&gt;""),IF(E16&gt;F16,3,IF(E16=F16,2,0)),"")</f>
         <v/>
       </c>
       <c r="I16" s="29">
-        <f>IF(AND(E16&lt;&gt;"",F16&lt;&gt;""),IF(F16&gt;E16,3,IF(E16=F16,1,0)),"")</f>
+        <f>IF(AND(E16&lt;&gt;"",F16&lt;&gt;""),IF(F16&gt;E16,3,IF(E16=F16,2,0)),"")</f>
         <v/>
       </c>
       <c r="J16" s="29">
@@ -3652,11 +3631,11 @@
         </is>
       </c>
       <c r="H17" s="31">
-        <f>IF(AND(E17&lt;&gt;"",F17&lt;&gt;""),IF(E17&gt;F17,3,IF(E17=F17,1,0)),"")</f>
+        <f>IF(AND(E17&lt;&gt;"",F17&lt;&gt;""),IF(E17&gt;F17,3,IF(E17=F17,2,0)),"")</f>
         <v/>
       </c>
       <c r="I17" s="31">
-        <f>IF(AND(E17&lt;&gt;"",F17&lt;&gt;""),IF(F17&gt;E17,3,IF(E17=F17,1,0)),"")</f>
+        <f>IF(AND(E17&lt;&gt;"",F17&lt;&gt;""),IF(F17&gt;E17,3,IF(E17=F17,2,0)),"")</f>
         <v/>
       </c>
       <c r="J17" s="31">
@@ -3695,11 +3674,11 @@
         </is>
       </c>
       <c r="H18" s="31">
-        <f>IF(AND(E18&lt;&gt;"",F18&lt;&gt;""),IF(E18&gt;F18,3,IF(E18=F18,1,0)),"")</f>
+        <f>IF(AND(E18&lt;&gt;"",F18&lt;&gt;""),IF(E18&gt;F18,3,IF(E18=F18,2,0)),"")</f>
         <v/>
       </c>
       <c r="I18" s="31">
-        <f>IF(AND(E18&lt;&gt;"",F18&lt;&gt;""),IF(F18&gt;E18,3,IF(E18=F18,1,0)),"")</f>
+        <f>IF(AND(E18&lt;&gt;"",F18&lt;&gt;""),IF(F18&gt;E18,3,IF(E18=F18,2,0)),"")</f>
         <v/>
       </c>
       <c r="J18" s="31">
@@ -3738,11 +3717,11 @@
         </is>
       </c>
       <c r="H19" s="33">
-        <f>IF(AND(E19&lt;&gt;"",F19&lt;&gt;""),IF(E19&gt;F19,3,IF(E19=F19,1,0)),"")</f>
+        <f>IF(AND(E19&lt;&gt;"",F19&lt;&gt;""),IF(E19&gt;F19,3,IF(E19=F19,2,0)),"")</f>
         <v/>
       </c>
       <c r="I19" s="33">
-        <f>IF(AND(E19&lt;&gt;"",F19&lt;&gt;""),IF(F19&gt;E19,3,IF(E19=F19,1,0)),"")</f>
+        <f>IF(AND(E19&lt;&gt;"",F19&lt;&gt;""),IF(F19&gt;E19,3,IF(E19=F19,2,0)),"")</f>
         <v/>
       </c>
       <c r="J19" s="33">
@@ -3781,11 +3760,11 @@
         </is>
       </c>
       <c r="H20" s="33">
-        <f>IF(AND(E20&lt;&gt;"",F20&lt;&gt;""),IF(E20&gt;F20,3,IF(E20=F20,1,0)),"")</f>
+        <f>IF(AND(E20&lt;&gt;"",F20&lt;&gt;""),IF(E20&gt;F20,3,IF(E20=F20,2,0)),"")</f>
         <v/>
       </c>
       <c r="I20" s="33">
-        <f>IF(AND(E20&lt;&gt;"",F20&lt;&gt;""),IF(F20&gt;E20,3,IF(E20=F20,1,0)),"")</f>
+        <f>IF(AND(E20&lt;&gt;"",F20&lt;&gt;""),IF(F20&gt;E20,3,IF(E20=F20,2,0)),"")</f>
         <v/>
       </c>
       <c r="J20" s="33">
@@ -3824,11 +3803,11 @@
         </is>
       </c>
       <c r="H21" s="35">
-        <f>IF(AND(E21&lt;&gt;"",F21&lt;&gt;""),IF(E21&gt;F21,3,IF(E21=F21,1,0)),"")</f>
+        <f>IF(AND(E21&lt;&gt;"",F21&lt;&gt;""),IF(E21&gt;F21,3,IF(E21=F21,2,0)),"")</f>
         <v/>
       </c>
       <c r="I21" s="35">
-        <f>IF(AND(E21&lt;&gt;"",F21&lt;&gt;""),IF(F21&gt;E21,3,IF(E21=F21,1,0)),"")</f>
+        <f>IF(AND(E21&lt;&gt;"",F21&lt;&gt;""),IF(F21&gt;E21,3,IF(E21=F21,2,0)),"")</f>
         <v/>
       </c>
       <c r="J21" s="35">
@@ -3867,11 +3846,11 @@
         </is>
       </c>
       <c r="H22" s="35">
-        <f>IF(AND(E22&lt;&gt;"",F22&lt;&gt;""),IF(E22&gt;F22,3,IF(E22=F22,1,0)),"")</f>
+        <f>IF(AND(E22&lt;&gt;"",F22&lt;&gt;""),IF(E22&gt;F22,3,IF(E22=F22,2,0)),"")</f>
         <v/>
       </c>
       <c r="I22" s="35">
-        <f>IF(AND(E22&lt;&gt;"",F22&lt;&gt;""),IF(F22&gt;E22,3,IF(E22=F22,1,0)),"")</f>
+        <f>IF(AND(E22&lt;&gt;"",F22&lt;&gt;""),IF(F22&gt;E22,3,IF(E22=F22,2,0)),"")</f>
         <v/>
       </c>
       <c r="J22" s="35">
@@ -3910,11 +3889,11 @@
         </is>
       </c>
       <c r="H23" s="37">
-        <f>IF(AND(E23&lt;&gt;"",F23&lt;&gt;""),IF(E23&gt;F23,3,IF(E23=F23,1,0)),"")</f>
+        <f>IF(AND(E23&lt;&gt;"",F23&lt;&gt;""),IF(E23&gt;F23,3,IF(E23=F23,2,0)),"")</f>
         <v/>
       </c>
       <c r="I23" s="37">
-        <f>IF(AND(E23&lt;&gt;"",F23&lt;&gt;""),IF(F23&gt;E23,3,IF(E23=F23,1,0)),"")</f>
+        <f>IF(AND(E23&lt;&gt;"",F23&lt;&gt;""),IF(F23&gt;E23,3,IF(E23=F23,2,0)),"")</f>
         <v/>
       </c>
       <c r="J23" s="37">
@@ -3953,11 +3932,11 @@
         </is>
       </c>
       <c r="H24" s="37">
-        <f>IF(AND(E24&lt;&gt;"",F24&lt;&gt;""),IF(E24&gt;F24,3,IF(E24=F24,1,0)),"")</f>
+        <f>IF(AND(E24&lt;&gt;"",F24&lt;&gt;""),IF(E24&gt;F24,3,IF(E24=F24,2,0)),"")</f>
         <v/>
       </c>
       <c r="I24" s="37">
-        <f>IF(AND(E24&lt;&gt;"",F24&lt;&gt;""),IF(F24&gt;E24,3,IF(E24=F24,1,0)),"")</f>
+        <f>IF(AND(E24&lt;&gt;"",F24&lt;&gt;""),IF(F24&gt;E24,3,IF(E24=F24,2,0)),"")</f>
         <v/>
       </c>
       <c r="J24" s="37">
@@ -3996,11 +3975,11 @@
         </is>
       </c>
       <c r="H25" s="39">
-        <f>IF(AND(E25&lt;&gt;"",F25&lt;&gt;""),IF(E25&gt;F25,3,IF(E25=F25,1,0)),"")</f>
+        <f>IF(AND(E25&lt;&gt;"",F25&lt;&gt;""),IF(E25&gt;F25,3,IF(E25=F25,2,0)),"")</f>
         <v/>
       </c>
       <c r="I25" s="39">
-        <f>IF(AND(E25&lt;&gt;"",F25&lt;&gt;""),IF(F25&gt;E25,3,IF(E25=F25,1,0)),"")</f>
+        <f>IF(AND(E25&lt;&gt;"",F25&lt;&gt;""),IF(F25&gt;E25,3,IF(E25=F25,2,0)),"")</f>
         <v/>
       </c>
       <c r="J25" s="39">
@@ -4039,11 +4018,11 @@
         </is>
       </c>
       <c r="H26" s="39">
-        <f>IF(AND(E26&lt;&gt;"",F26&lt;&gt;""),IF(E26&gt;F26,3,IF(E26=F26,1,0)),"")</f>
+        <f>IF(AND(E26&lt;&gt;"",F26&lt;&gt;""),IF(E26&gt;F26,3,IF(E26=F26,2,0)),"")</f>
         <v/>
       </c>
       <c r="I26" s="39">
-        <f>IF(AND(E26&lt;&gt;"",F26&lt;&gt;""),IF(F26&gt;E26,3,IF(E26=F26,1,0)),"")</f>
+        <f>IF(AND(E26&lt;&gt;"",F26&lt;&gt;""),IF(F26&gt;E26,3,IF(E26=F26,2,0)),"")</f>
         <v/>
       </c>
       <c r="J26" s="39">
@@ -4082,11 +4061,11 @@
         </is>
       </c>
       <c r="H27" s="41">
-        <f>IF(AND(E27&lt;&gt;"",F27&lt;&gt;""),IF(E27&gt;F27,3,IF(E27=F27,1,0)),"")</f>
+        <f>IF(AND(E27&lt;&gt;"",F27&lt;&gt;""),IF(E27&gt;F27,3,IF(E27=F27,2,0)),"")</f>
         <v/>
       </c>
       <c r="I27" s="41">
-        <f>IF(AND(E27&lt;&gt;"",F27&lt;&gt;""),IF(F27&gt;E27,3,IF(E27=F27,1,0)),"")</f>
+        <f>IF(AND(E27&lt;&gt;"",F27&lt;&gt;""),IF(F27&gt;E27,3,IF(E27=F27,2,0)),"")</f>
         <v/>
       </c>
       <c r="J27" s="41">
@@ -4125,11 +4104,11 @@
         </is>
       </c>
       <c r="H28" s="41">
-        <f>IF(AND(E28&lt;&gt;"",F28&lt;&gt;""),IF(E28&gt;F28,3,IF(E28=F28,1,0)),"")</f>
+        <f>IF(AND(E28&lt;&gt;"",F28&lt;&gt;""),IF(E28&gt;F28,3,IF(E28=F28,2,0)),"")</f>
         <v/>
       </c>
       <c r="I28" s="41">
-        <f>IF(AND(E28&lt;&gt;"",F28&lt;&gt;""),IF(F28&gt;E28,3,IF(E28=F28,1,0)),"")</f>
+        <f>IF(AND(E28&lt;&gt;"",F28&lt;&gt;""),IF(F28&gt;E28,3,IF(E28=F28,2,0)),"")</f>
         <v/>
       </c>
       <c r="J28" s="41">
@@ -4168,11 +4147,11 @@
         </is>
       </c>
       <c r="H29" s="19">
-        <f>IF(AND(E29&lt;&gt;"",F29&lt;&gt;""),IF(E29&gt;F29,3,IF(E29=F29,1,0)),"")</f>
+        <f>IF(AND(E29&lt;&gt;"",F29&lt;&gt;""),IF(E29&gt;F29,3,IF(E29=F29,2,0)),"")</f>
         <v/>
       </c>
       <c r="I29" s="19">
-        <f>IF(AND(E29&lt;&gt;"",F29&lt;&gt;""),IF(F29&gt;E29,3,IF(E29=F29,1,0)),"")</f>
+        <f>IF(AND(E29&lt;&gt;"",F29&lt;&gt;""),IF(F29&gt;E29,3,IF(E29=F29,2,0)),"")</f>
         <v/>
       </c>
       <c r="J29" s="19">
@@ -4211,11 +4190,11 @@
         </is>
       </c>
       <c r="H30" s="21">
-        <f>IF(AND(E30&lt;&gt;"",F30&lt;&gt;""),IF(E30&gt;F30,3,IF(E30=F30,1,0)),"")</f>
+        <f>IF(AND(E30&lt;&gt;"",F30&lt;&gt;""),IF(E30&gt;F30,3,IF(E30=F30,2,0)),"")</f>
         <v/>
       </c>
       <c r="I30" s="21">
-        <f>IF(AND(E30&lt;&gt;"",F30&lt;&gt;""),IF(F30&gt;E30,3,IF(E30=F30,1,0)),"")</f>
+        <f>IF(AND(E30&lt;&gt;"",F30&lt;&gt;""),IF(F30&gt;E30,3,IF(E30=F30,2,0)),"")</f>
         <v/>
       </c>
       <c r="J30" s="21">
@@ -4254,11 +4233,11 @@
         </is>
       </c>
       <c r="H31" s="21">
-        <f>IF(AND(E31&lt;&gt;"",F31&lt;&gt;""),IF(E31&gt;F31,3,IF(E31=F31,1,0)),"")</f>
+        <f>IF(AND(E31&lt;&gt;"",F31&lt;&gt;""),IF(E31&gt;F31,3,IF(E31=F31,2,0)),"")</f>
         <v/>
       </c>
       <c r="I31" s="21">
-        <f>IF(AND(E31&lt;&gt;"",F31&lt;&gt;""),IF(F31&gt;E31,3,IF(E31=F31,1,0)),"")</f>
+        <f>IF(AND(E31&lt;&gt;"",F31&lt;&gt;""),IF(F31&gt;E31,3,IF(E31=F31,2,0)),"")</f>
         <v/>
       </c>
       <c r="J31" s="21">
@@ -4297,11 +4276,11 @@
         </is>
       </c>
       <c r="H32" s="19">
-        <f>IF(AND(E32&lt;&gt;"",F32&lt;&gt;""),IF(E32&gt;F32,3,IF(E32=F32,1,0)),"")</f>
+        <f>IF(AND(E32&lt;&gt;"",F32&lt;&gt;""),IF(E32&gt;F32,3,IF(E32=F32,2,0)),"")</f>
         <v/>
       </c>
       <c r="I32" s="19">
-        <f>IF(AND(E32&lt;&gt;"",F32&lt;&gt;""),IF(F32&gt;E32,3,IF(E32=F32,1,0)),"")</f>
+        <f>IF(AND(E32&lt;&gt;"",F32&lt;&gt;""),IF(F32&gt;E32,3,IF(E32=F32,2,0)),"")</f>
         <v/>
       </c>
       <c r="J32" s="19">
@@ -4340,11 +4319,11 @@
         </is>
       </c>
       <c r="H33" s="25">
-        <f>IF(AND(E33&lt;&gt;"",F33&lt;&gt;""),IF(E33&gt;F33,3,IF(E33=F33,1,0)),"")</f>
+        <f>IF(AND(E33&lt;&gt;"",F33&lt;&gt;""),IF(E33&gt;F33,3,IF(E33=F33,2,0)),"")</f>
         <v/>
       </c>
       <c r="I33" s="25">
-        <f>IF(AND(E33&lt;&gt;"",F33&lt;&gt;""),IF(F33&gt;E33,3,IF(E33=F33,1,0)),"")</f>
+        <f>IF(AND(E33&lt;&gt;"",F33&lt;&gt;""),IF(F33&gt;E33,3,IF(E33=F33,2,0)),"")</f>
         <v/>
       </c>
       <c r="J33" s="25">
@@ -4383,11 +4362,11 @@
         </is>
       </c>
       <c r="H34" s="25">
-        <f>IF(AND(E34&lt;&gt;"",F34&lt;&gt;""),IF(E34&gt;F34,3,IF(E34=F34,1,0)),"")</f>
+        <f>IF(AND(E34&lt;&gt;"",F34&lt;&gt;""),IF(E34&gt;F34,3,IF(E34=F34,2,0)),"")</f>
         <v/>
       </c>
       <c r="I34" s="25">
-        <f>IF(AND(E34&lt;&gt;"",F34&lt;&gt;""),IF(F34&gt;E34,3,IF(E34=F34,1,0)),"")</f>
+        <f>IF(AND(E34&lt;&gt;"",F34&lt;&gt;""),IF(F34&gt;E34,3,IF(E34=F34,2,0)),"")</f>
         <v/>
       </c>
       <c r="J34" s="25">
@@ -4426,11 +4405,11 @@
         </is>
       </c>
       <c r="H35" s="23">
-        <f>IF(AND(E35&lt;&gt;"",F35&lt;&gt;""),IF(E35&gt;F35,3,IF(E35=F35,1,0)),"")</f>
+        <f>IF(AND(E35&lt;&gt;"",F35&lt;&gt;""),IF(E35&gt;F35,3,IF(E35=F35,2,0)),"")</f>
         <v/>
       </c>
       <c r="I35" s="23">
-        <f>IF(AND(E35&lt;&gt;"",F35&lt;&gt;""),IF(F35&gt;E35,3,IF(E35=F35,1,0)),"")</f>
+        <f>IF(AND(E35&lt;&gt;"",F35&lt;&gt;""),IF(F35&gt;E35,3,IF(E35=F35,2,0)),"")</f>
         <v/>
       </c>
       <c r="J35" s="23">
@@ -4469,11 +4448,11 @@
         </is>
       </c>
       <c r="H36" s="23">
-        <f>IF(AND(E36&lt;&gt;"",F36&lt;&gt;""),IF(E36&gt;F36,3,IF(E36=F36,1,0)),"")</f>
+        <f>IF(AND(E36&lt;&gt;"",F36&lt;&gt;""),IF(E36&gt;F36,3,IF(E36=F36,2,0)),"")</f>
         <v/>
       </c>
       <c r="I36" s="23">
-        <f>IF(AND(E36&lt;&gt;"",F36&lt;&gt;""),IF(F36&gt;E36,3,IF(E36=F36,1,0)),"")</f>
+        <f>IF(AND(E36&lt;&gt;"",F36&lt;&gt;""),IF(F36&gt;E36,3,IF(E36=F36,2,0)),"")</f>
         <v/>
       </c>
       <c r="J36" s="23">
@@ -4512,11 +4491,11 @@
         </is>
       </c>
       <c r="H37" s="27">
-        <f>IF(AND(E37&lt;&gt;"",F37&lt;&gt;""),IF(E37&gt;F37,3,IF(E37=F37,1,0)),"")</f>
+        <f>IF(AND(E37&lt;&gt;"",F37&lt;&gt;""),IF(E37&gt;F37,3,IF(E37=F37,2,0)),"")</f>
         <v/>
       </c>
       <c r="I37" s="27">
-        <f>IF(AND(E37&lt;&gt;"",F37&lt;&gt;""),IF(F37&gt;E37,3,IF(E37=F37,1,0)),"")</f>
+        <f>IF(AND(E37&lt;&gt;"",F37&lt;&gt;""),IF(F37&gt;E37,3,IF(E37=F37,2,0)),"")</f>
         <v/>
       </c>
       <c r="J37" s="27">
@@ -4555,11 +4534,11 @@
         </is>
       </c>
       <c r="H38" s="27">
-        <f>IF(AND(E38&lt;&gt;"",F38&lt;&gt;""),IF(E38&gt;F38,3,IF(E38=F38,1,0)),"")</f>
+        <f>IF(AND(E38&lt;&gt;"",F38&lt;&gt;""),IF(E38&gt;F38,3,IF(E38=F38,2,0)),"")</f>
         <v/>
       </c>
       <c r="I38" s="27">
-        <f>IF(AND(E38&lt;&gt;"",F38&lt;&gt;""),IF(F38&gt;E38,3,IF(E38=F38,1,0)),"")</f>
+        <f>IF(AND(E38&lt;&gt;"",F38&lt;&gt;""),IF(F38&gt;E38,3,IF(E38=F38,2,0)),"")</f>
         <v/>
       </c>
       <c r="J38" s="27">
@@ -4598,11 +4577,11 @@
         </is>
       </c>
       <c r="H39" s="29">
-        <f>IF(AND(E39&lt;&gt;"",F39&lt;&gt;""),IF(E39&gt;F39,3,IF(E39=F39,1,0)),"")</f>
+        <f>IF(AND(E39&lt;&gt;"",F39&lt;&gt;""),IF(E39&gt;F39,3,IF(E39=F39,2,0)),"")</f>
         <v/>
       </c>
       <c r="I39" s="29">
-        <f>IF(AND(E39&lt;&gt;"",F39&lt;&gt;""),IF(F39&gt;E39,3,IF(E39=F39,1,0)),"")</f>
+        <f>IF(AND(E39&lt;&gt;"",F39&lt;&gt;""),IF(F39&gt;E39,3,IF(E39=F39,2,0)),"")</f>
         <v/>
       </c>
       <c r="J39" s="29">
@@ -4641,11 +4620,11 @@
         </is>
       </c>
       <c r="H40" s="29">
-        <f>IF(AND(E40&lt;&gt;"",F40&lt;&gt;""),IF(E40&gt;F40,3,IF(E40=F40,1,0)),"")</f>
+        <f>IF(AND(E40&lt;&gt;"",F40&lt;&gt;""),IF(E40&gt;F40,3,IF(E40=F40,2,0)),"")</f>
         <v/>
       </c>
       <c r="I40" s="29">
-        <f>IF(AND(E40&lt;&gt;"",F40&lt;&gt;""),IF(F40&gt;E40,3,IF(E40=F40,1,0)),"")</f>
+        <f>IF(AND(E40&lt;&gt;"",F40&lt;&gt;""),IF(F40&gt;E40,3,IF(E40=F40,2,0)),"")</f>
         <v/>
       </c>
       <c r="J40" s="29">
@@ -4684,11 +4663,11 @@
         </is>
       </c>
       <c r="H41" s="31">
-        <f>IF(AND(E41&lt;&gt;"",F41&lt;&gt;""),IF(E41&gt;F41,3,IF(E41=F41,1,0)),"")</f>
+        <f>IF(AND(E41&lt;&gt;"",F41&lt;&gt;""),IF(E41&gt;F41,3,IF(E41=F41,2,0)),"")</f>
         <v/>
       </c>
       <c r="I41" s="31">
-        <f>IF(AND(E41&lt;&gt;"",F41&lt;&gt;""),IF(F41&gt;E41,3,IF(E41=F41,1,0)),"")</f>
+        <f>IF(AND(E41&lt;&gt;"",F41&lt;&gt;""),IF(F41&gt;E41,3,IF(E41=F41,2,0)),"")</f>
         <v/>
       </c>
       <c r="J41" s="31">
@@ -4727,11 +4706,11 @@
         </is>
       </c>
       <c r="H42" s="31">
-        <f>IF(AND(E42&lt;&gt;"",F42&lt;&gt;""),IF(E42&gt;F42,3,IF(E42=F42,1,0)),"")</f>
+        <f>IF(AND(E42&lt;&gt;"",F42&lt;&gt;""),IF(E42&gt;F42,3,IF(E42=F42,2,0)),"")</f>
         <v/>
       </c>
       <c r="I42" s="31">
-        <f>IF(AND(E42&lt;&gt;"",F42&lt;&gt;""),IF(F42&gt;E42,3,IF(E42=F42,1,0)),"")</f>
+        <f>IF(AND(E42&lt;&gt;"",F42&lt;&gt;""),IF(F42&gt;E42,3,IF(E42=F42,2,0)),"")</f>
         <v/>
       </c>
       <c r="J42" s="31">
@@ -4770,11 +4749,11 @@
         </is>
       </c>
       <c r="H43" s="33">
-        <f>IF(AND(E43&lt;&gt;"",F43&lt;&gt;""),IF(E43&gt;F43,3,IF(E43=F43,1,0)),"")</f>
+        <f>IF(AND(E43&lt;&gt;"",F43&lt;&gt;""),IF(E43&gt;F43,3,IF(E43=F43,2,0)),"")</f>
         <v/>
       </c>
       <c r="I43" s="33">
-        <f>IF(AND(E43&lt;&gt;"",F43&lt;&gt;""),IF(F43&gt;E43,3,IF(E43=F43,1,0)),"")</f>
+        <f>IF(AND(E43&lt;&gt;"",F43&lt;&gt;""),IF(F43&gt;E43,3,IF(E43=F43,2,0)),"")</f>
         <v/>
       </c>
       <c r="J43" s="33">
@@ -4813,11 +4792,11 @@
         </is>
       </c>
       <c r="H44" s="33">
-        <f>IF(AND(E44&lt;&gt;"",F44&lt;&gt;""),IF(E44&gt;F44,3,IF(E44=F44,1,0)),"")</f>
+        <f>IF(AND(E44&lt;&gt;"",F44&lt;&gt;""),IF(E44&gt;F44,3,IF(E44=F44,2,0)),"")</f>
         <v/>
       </c>
       <c r="I44" s="33">
-        <f>IF(AND(E44&lt;&gt;"",F44&lt;&gt;""),IF(F44&gt;E44,3,IF(E44=F44,1,0)),"")</f>
+        <f>IF(AND(E44&lt;&gt;"",F44&lt;&gt;""),IF(F44&gt;E44,3,IF(E44=F44,2,0)),"")</f>
         <v/>
       </c>
       <c r="J44" s="33">
@@ -4856,11 +4835,11 @@
         </is>
       </c>
       <c r="H45" s="35">
-        <f>IF(AND(E45&lt;&gt;"",F45&lt;&gt;""),IF(E45&gt;F45,3,IF(E45=F45,1,0)),"")</f>
+        <f>IF(AND(E45&lt;&gt;"",F45&lt;&gt;""),IF(E45&gt;F45,3,IF(E45=F45,2,0)),"")</f>
         <v/>
       </c>
       <c r="I45" s="35">
-        <f>IF(AND(E45&lt;&gt;"",F45&lt;&gt;""),IF(F45&gt;E45,3,IF(E45=F45,1,0)),"")</f>
+        <f>IF(AND(E45&lt;&gt;"",F45&lt;&gt;""),IF(F45&gt;E45,3,IF(E45=F45,2,0)),"")</f>
         <v/>
       </c>
       <c r="J45" s="35">
@@ -4899,11 +4878,11 @@
         </is>
       </c>
       <c r="H46" s="35">
-        <f>IF(AND(E46&lt;&gt;"",F46&lt;&gt;""),IF(E46&gt;F46,3,IF(E46=F46,1,0)),"")</f>
+        <f>IF(AND(E46&lt;&gt;"",F46&lt;&gt;""),IF(E46&gt;F46,3,IF(E46=F46,2,0)),"")</f>
         <v/>
       </c>
       <c r="I46" s="35">
-        <f>IF(AND(E46&lt;&gt;"",F46&lt;&gt;""),IF(F46&gt;E46,3,IF(E46=F46,1,0)),"")</f>
+        <f>IF(AND(E46&lt;&gt;"",F46&lt;&gt;""),IF(F46&gt;E46,3,IF(E46=F46,2,0)),"")</f>
         <v/>
       </c>
       <c r="J46" s="35">
@@ -4942,11 +4921,11 @@
         </is>
       </c>
       <c r="H47" s="37">
-        <f>IF(AND(E47&lt;&gt;"",F47&lt;&gt;""),IF(E47&gt;F47,3,IF(E47=F47,1,0)),"")</f>
+        <f>IF(AND(E47&lt;&gt;"",F47&lt;&gt;""),IF(E47&gt;F47,3,IF(E47=F47,2,0)),"")</f>
         <v/>
       </c>
       <c r="I47" s="37">
-        <f>IF(AND(E47&lt;&gt;"",F47&lt;&gt;""),IF(F47&gt;E47,3,IF(E47=F47,1,0)),"")</f>
+        <f>IF(AND(E47&lt;&gt;"",F47&lt;&gt;""),IF(F47&gt;E47,3,IF(E47=F47,2,0)),"")</f>
         <v/>
       </c>
       <c r="J47" s="37">
@@ -4985,11 +4964,11 @@
         </is>
       </c>
       <c r="H48" s="37">
-        <f>IF(AND(E48&lt;&gt;"",F48&lt;&gt;""),IF(E48&gt;F48,3,IF(E48=F48,1,0)),"")</f>
+        <f>IF(AND(E48&lt;&gt;"",F48&lt;&gt;""),IF(E48&gt;F48,3,IF(E48=F48,2,0)),"")</f>
         <v/>
       </c>
       <c r="I48" s="37">
-        <f>IF(AND(E48&lt;&gt;"",F48&lt;&gt;""),IF(F48&gt;E48,3,IF(E48=F48,1,0)),"")</f>
+        <f>IF(AND(E48&lt;&gt;"",F48&lt;&gt;""),IF(F48&gt;E48,3,IF(E48=F48,2,0)),"")</f>
         <v/>
       </c>
       <c r="J48" s="37">
@@ -5028,11 +5007,11 @@
         </is>
       </c>
       <c r="H49" s="39">
-        <f>IF(AND(E49&lt;&gt;"",F49&lt;&gt;""),IF(E49&gt;F49,3,IF(E49=F49,1,0)),"")</f>
+        <f>IF(AND(E49&lt;&gt;"",F49&lt;&gt;""),IF(E49&gt;F49,3,IF(E49=F49,2,0)),"")</f>
         <v/>
       </c>
       <c r="I49" s="39">
-        <f>IF(AND(E49&lt;&gt;"",F49&lt;&gt;""),IF(F49&gt;E49,3,IF(E49=F49,1,0)),"")</f>
+        <f>IF(AND(E49&lt;&gt;"",F49&lt;&gt;""),IF(F49&gt;E49,3,IF(E49=F49,2,0)),"")</f>
         <v/>
       </c>
       <c r="J49" s="39">
@@ -5071,11 +5050,11 @@
         </is>
       </c>
       <c r="H50" s="39">
-        <f>IF(AND(E50&lt;&gt;"",F50&lt;&gt;""),IF(E50&gt;F50,3,IF(E50=F50,1,0)),"")</f>
+        <f>IF(AND(E50&lt;&gt;"",F50&lt;&gt;""),IF(E50&gt;F50,3,IF(E50=F50,2,0)),"")</f>
         <v/>
       </c>
       <c r="I50" s="39">
-        <f>IF(AND(E50&lt;&gt;"",F50&lt;&gt;""),IF(F50&gt;E50,3,IF(E50=F50,1,0)),"")</f>
+        <f>IF(AND(E50&lt;&gt;"",F50&lt;&gt;""),IF(F50&gt;E50,3,IF(E50=F50,2,0)),"")</f>
         <v/>
       </c>
       <c r="J50" s="39">
@@ -5114,11 +5093,11 @@
         </is>
       </c>
       <c r="H51" s="41">
-        <f>IF(AND(E51&lt;&gt;"",F51&lt;&gt;""),IF(E51&gt;F51,3,IF(E51=F51,1,0)),"")</f>
+        <f>IF(AND(E51&lt;&gt;"",F51&lt;&gt;""),IF(E51&gt;F51,3,IF(E51=F51,2,0)),"")</f>
         <v/>
       </c>
       <c r="I51" s="41">
-        <f>IF(AND(E51&lt;&gt;"",F51&lt;&gt;""),IF(F51&gt;E51,3,IF(E51=F51,1,0)),"")</f>
+        <f>IF(AND(E51&lt;&gt;"",F51&lt;&gt;""),IF(F51&gt;E51,3,IF(E51=F51,2,0)),"")</f>
         <v/>
       </c>
       <c r="J51" s="41">
@@ -5157,11 +5136,11 @@
         </is>
       </c>
       <c r="H52" s="41">
-        <f>IF(AND(E52&lt;&gt;"",F52&lt;&gt;""),IF(E52&gt;F52,3,IF(E52=F52,1,0)),"")</f>
+        <f>IF(AND(E52&lt;&gt;"",F52&lt;&gt;""),IF(E52&gt;F52,3,IF(E52=F52,2,0)),"")</f>
         <v/>
       </c>
       <c r="I52" s="41">
-        <f>IF(AND(E52&lt;&gt;"",F52&lt;&gt;""),IF(F52&gt;E52,3,IF(E52=F52,1,0)),"")</f>
+        <f>IF(AND(E52&lt;&gt;"",F52&lt;&gt;""),IF(F52&gt;E52,3,IF(E52=F52,2,0)),"")</f>
         <v/>
       </c>
       <c r="J52" s="41">
@@ -5200,11 +5179,11 @@
         </is>
       </c>
       <c r="H53" s="25">
-        <f>IF(AND(E53&lt;&gt;"",F53&lt;&gt;""),IF(E53&gt;F53,3,IF(E53=F53,1,0)),"")</f>
+        <f>IF(AND(E53&lt;&gt;"",F53&lt;&gt;""),IF(E53&gt;F53,3,IF(E53=F53,2,0)),"")</f>
         <v/>
       </c>
       <c r="I53" s="25">
-        <f>IF(AND(E53&lt;&gt;"",F53&lt;&gt;""),IF(F53&gt;E53,3,IF(E53=F53,1,0)),"")</f>
+        <f>IF(AND(E53&lt;&gt;"",F53&lt;&gt;""),IF(F53&gt;E53,3,IF(E53=F53,2,0)),"")</f>
         <v/>
       </c>
       <c r="J53" s="25">
@@ -5243,11 +5222,11 @@
         </is>
       </c>
       <c r="H54" s="25">
-        <f>IF(AND(E54&lt;&gt;"",F54&lt;&gt;""),IF(E54&gt;F54,3,IF(E54=F54,1,0)),"")</f>
+        <f>IF(AND(E54&lt;&gt;"",F54&lt;&gt;""),IF(E54&gt;F54,3,IF(E54=F54,2,0)),"")</f>
         <v/>
       </c>
       <c r="I54" s="25">
-        <f>IF(AND(E54&lt;&gt;"",F54&lt;&gt;""),IF(F54&gt;E54,3,IF(E54=F54,1,0)),"")</f>
+        <f>IF(AND(E54&lt;&gt;"",F54&lt;&gt;""),IF(F54&gt;E54,3,IF(E54=F54,2,0)),"")</f>
         <v/>
       </c>
       <c r="J54" s="25">
@@ -5286,11 +5265,11 @@
         </is>
       </c>
       <c r="H55" s="21">
-        <f>IF(AND(E55&lt;&gt;"",F55&lt;&gt;""),IF(E55&gt;F55,3,IF(E55=F55,1,0)),"")</f>
+        <f>IF(AND(E55&lt;&gt;"",F55&lt;&gt;""),IF(E55&gt;F55,3,IF(E55=F55,2,0)),"")</f>
         <v/>
       </c>
       <c r="I55" s="21">
-        <f>IF(AND(E55&lt;&gt;"",F55&lt;&gt;""),IF(F55&gt;E55,3,IF(E55=F55,1,0)),"")</f>
+        <f>IF(AND(E55&lt;&gt;"",F55&lt;&gt;""),IF(F55&gt;E55,3,IF(E55=F55,2,0)),"")</f>
         <v/>
       </c>
       <c r="J55" s="21">
@@ -5329,11 +5308,11 @@
         </is>
       </c>
       <c r="H56" s="21">
-        <f>IF(AND(E56&lt;&gt;"",F56&lt;&gt;""),IF(E56&gt;F56,3,IF(E56=F56,1,0)),"")</f>
+        <f>IF(AND(E56&lt;&gt;"",F56&lt;&gt;""),IF(E56&gt;F56,3,IF(E56=F56,2,0)),"")</f>
         <v/>
       </c>
       <c r="I56" s="21">
-        <f>IF(AND(E56&lt;&gt;"",F56&lt;&gt;""),IF(F56&gt;E56,3,IF(E56=F56,1,0)),"")</f>
+        <f>IF(AND(E56&lt;&gt;"",F56&lt;&gt;""),IF(F56&gt;E56,3,IF(E56=F56,2,0)),"")</f>
         <v/>
       </c>
       <c r="J56" s="21">
@@ -5372,11 +5351,11 @@
         </is>
       </c>
       <c r="H57" s="19">
-        <f>IF(AND(E57&lt;&gt;"",F57&lt;&gt;""),IF(E57&gt;F57,3,IF(E57=F57,1,0)),"")</f>
+        <f>IF(AND(E57&lt;&gt;"",F57&lt;&gt;""),IF(E57&gt;F57,3,IF(E57=F57,2,0)),"")</f>
         <v/>
       </c>
       <c r="I57" s="19">
-        <f>IF(AND(E57&lt;&gt;"",F57&lt;&gt;""),IF(F57&gt;E57,3,IF(E57=F57,1,0)),"")</f>
+        <f>IF(AND(E57&lt;&gt;"",F57&lt;&gt;""),IF(F57&gt;E57,3,IF(E57=F57,2,0)),"")</f>
         <v/>
       </c>
       <c r="J57" s="19">
@@ -5415,11 +5394,11 @@
         </is>
       </c>
       <c r="H58" s="19">
-        <f>IF(AND(E58&lt;&gt;"",F58&lt;&gt;""),IF(E58&gt;F58,3,IF(E58=F58,1,0)),"")</f>
+        <f>IF(AND(E58&lt;&gt;"",F58&lt;&gt;""),IF(E58&gt;F58,3,IF(E58=F58,2,0)),"")</f>
         <v/>
       </c>
       <c r="I58" s="19">
-        <f>IF(AND(E58&lt;&gt;"",F58&lt;&gt;""),IF(F58&gt;E58,3,IF(E58=F58,1,0)),"")</f>
+        <f>IF(AND(E58&lt;&gt;"",F58&lt;&gt;""),IF(F58&gt;E58,3,IF(E58=F58,2,0)),"")</f>
         <v/>
       </c>
       <c r="J58" s="19">
@@ -5458,11 +5437,11 @@
         </is>
       </c>
       <c r="H59" s="27">
-        <f>IF(AND(E59&lt;&gt;"",F59&lt;&gt;""),IF(E59&gt;F59,3,IF(E59=F59,1,0)),"")</f>
+        <f>IF(AND(E59&lt;&gt;"",F59&lt;&gt;""),IF(E59&gt;F59,3,IF(E59=F59,2,0)),"")</f>
         <v/>
       </c>
       <c r="I59" s="27">
-        <f>IF(AND(E59&lt;&gt;"",F59&lt;&gt;""),IF(F59&gt;E59,3,IF(E59=F59,1,0)),"")</f>
+        <f>IF(AND(E59&lt;&gt;"",F59&lt;&gt;""),IF(F59&gt;E59,3,IF(E59=F59,2,0)),"")</f>
         <v/>
       </c>
       <c r="J59" s="27">
@@ -5501,11 +5480,11 @@
         </is>
       </c>
       <c r="H60" s="27">
-        <f>IF(AND(E60&lt;&gt;"",F60&lt;&gt;""),IF(E60&gt;F60,3,IF(E60=F60,1,0)),"")</f>
+        <f>IF(AND(E60&lt;&gt;"",F60&lt;&gt;""),IF(E60&gt;F60,3,IF(E60=F60,2,0)),"")</f>
         <v/>
       </c>
       <c r="I60" s="27">
-        <f>IF(AND(E60&lt;&gt;"",F60&lt;&gt;""),IF(F60&gt;E60,3,IF(E60=F60,1,0)),"")</f>
+        <f>IF(AND(E60&lt;&gt;"",F60&lt;&gt;""),IF(F60&gt;E60,3,IF(E60=F60,2,0)),"")</f>
         <v/>
       </c>
       <c r="J60" s="27">
@@ -5544,11 +5523,11 @@
         </is>
       </c>
       <c r="H61" s="29">
-        <f>IF(AND(E61&lt;&gt;"",F61&lt;&gt;""),IF(E61&gt;F61,3,IF(E61=F61,1,0)),"")</f>
+        <f>IF(AND(E61&lt;&gt;"",F61&lt;&gt;""),IF(E61&gt;F61,3,IF(E61=F61,2,0)),"")</f>
         <v/>
       </c>
       <c r="I61" s="29">
-        <f>IF(AND(E61&lt;&gt;"",F61&lt;&gt;""),IF(F61&gt;E61,3,IF(E61=F61,1,0)),"")</f>
+        <f>IF(AND(E61&lt;&gt;"",F61&lt;&gt;""),IF(F61&gt;E61,3,IF(E61=F61,2,0)),"")</f>
         <v/>
       </c>
       <c r="J61" s="29">
@@ -5587,11 +5566,11 @@
         </is>
       </c>
       <c r="H62" s="29">
-        <f>IF(AND(E62&lt;&gt;"",F62&lt;&gt;""),IF(E62&gt;F62,3,IF(E62=F62,1,0)),"")</f>
+        <f>IF(AND(E62&lt;&gt;"",F62&lt;&gt;""),IF(E62&gt;F62,3,IF(E62=F62,2,0)),"")</f>
         <v/>
       </c>
       <c r="I62" s="29">
-        <f>IF(AND(E62&lt;&gt;"",F62&lt;&gt;""),IF(F62&gt;E62,3,IF(E62=F62,1,0)),"")</f>
+        <f>IF(AND(E62&lt;&gt;"",F62&lt;&gt;""),IF(F62&gt;E62,3,IF(E62=F62,2,0)),"")</f>
         <v/>
       </c>
       <c r="J62" s="29">
@@ -5630,11 +5609,11 @@
         </is>
       </c>
       <c r="H63" s="23">
-        <f>IF(AND(E63&lt;&gt;"",F63&lt;&gt;""),IF(E63&gt;F63,3,IF(E63=F63,1,0)),"")</f>
+        <f>IF(AND(E63&lt;&gt;"",F63&lt;&gt;""),IF(E63&gt;F63,3,IF(E63=F63,2,0)),"")</f>
         <v/>
       </c>
       <c r="I63" s="23">
-        <f>IF(AND(E63&lt;&gt;"",F63&lt;&gt;""),IF(F63&gt;E63,3,IF(E63=F63,1,0)),"")</f>
+        <f>IF(AND(E63&lt;&gt;"",F63&lt;&gt;""),IF(F63&gt;E63,3,IF(E63=F63,2,0)),"")</f>
         <v/>
       </c>
       <c r="J63" s="23">
@@ -5673,11 +5652,11 @@
         </is>
       </c>
       <c r="H64" s="23">
-        <f>IF(AND(E64&lt;&gt;"",F64&lt;&gt;""),IF(E64&gt;F64,3,IF(E64=F64,1,0)),"")</f>
+        <f>IF(AND(E64&lt;&gt;"",F64&lt;&gt;""),IF(E64&gt;F64,3,IF(E64=F64,2,0)),"")</f>
         <v/>
       </c>
       <c r="I64" s="23">
-        <f>IF(AND(E64&lt;&gt;"",F64&lt;&gt;""),IF(F64&gt;E64,3,IF(E64=F64,1,0)),"")</f>
+        <f>IF(AND(E64&lt;&gt;"",F64&lt;&gt;""),IF(F64&gt;E64,3,IF(E64=F64,2,0)),"")</f>
         <v/>
       </c>
       <c r="J64" s="23">
@@ -5716,11 +5695,11 @@
         </is>
       </c>
       <c r="H65" s="35">
-        <f>IF(AND(E65&lt;&gt;"",F65&lt;&gt;""),IF(E65&gt;F65,3,IF(E65=F65,1,0)),"")</f>
+        <f>IF(AND(E65&lt;&gt;"",F65&lt;&gt;""),IF(E65&gt;F65,3,IF(E65=F65,2,0)),"")</f>
         <v/>
       </c>
       <c r="I65" s="35">
-        <f>IF(AND(E65&lt;&gt;"",F65&lt;&gt;""),IF(F65&gt;E65,3,IF(E65=F65,1,0)),"")</f>
+        <f>IF(AND(E65&lt;&gt;"",F65&lt;&gt;""),IF(F65&gt;E65,3,IF(E65=F65,2,0)),"")</f>
         <v/>
       </c>
       <c r="J65" s="35">
@@ -5759,11 +5738,11 @@
         </is>
       </c>
       <c r="H66" s="35">
-        <f>IF(AND(E66&lt;&gt;"",F66&lt;&gt;""),IF(E66&gt;F66,3,IF(E66=F66,1,0)),"")</f>
+        <f>IF(AND(E66&lt;&gt;"",F66&lt;&gt;""),IF(E66&gt;F66,3,IF(E66=F66,2,0)),"")</f>
         <v/>
       </c>
       <c r="I66" s="35">
-        <f>IF(AND(E66&lt;&gt;"",F66&lt;&gt;""),IF(F66&gt;E66,3,IF(E66=F66,1,0)),"")</f>
+        <f>IF(AND(E66&lt;&gt;"",F66&lt;&gt;""),IF(F66&gt;E66,3,IF(E66=F66,2,0)),"")</f>
         <v/>
       </c>
       <c r="J66" s="35">
@@ -5802,11 +5781,11 @@
         </is>
       </c>
       <c r="H67" s="33">
-        <f>IF(AND(E67&lt;&gt;"",F67&lt;&gt;""),IF(E67&gt;F67,3,IF(E67=F67,1,0)),"")</f>
+        <f>IF(AND(E67&lt;&gt;"",F67&lt;&gt;""),IF(E67&gt;F67,3,IF(E67=F67,2,0)),"")</f>
         <v/>
       </c>
       <c r="I67" s="33">
-        <f>IF(AND(E67&lt;&gt;"",F67&lt;&gt;""),IF(F67&gt;E67,3,IF(E67=F67,1,0)),"")</f>
+        <f>IF(AND(E67&lt;&gt;"",F67&lt;&gt;""),IF(F67&gt;E67,3,IF(E67=F67,2,0)),"")</f>
         <v/>
       </c>
       <c r="J67" s="33">
@@ -5845,11 +5824,11 @@
         </is>
       </c>
       <c r="H68" s="33">
-        <f>IF(AND(E68&lt;&gt;"",F68&lt;&gt;""),IF(E68&gt;F68,3,IF(E68=F68,1,0)),"")</f>
+        <f>IF(AND(E68&lt;&gt;"",F68&lt;&gt;""),IF(E68&gt;F68,3,IF(E68=F68,2,0)),"")</f>
         <v/>
       </c>
       <c r="I68" s="33">
-        <f>IF(AND(E68&lt;&gt;"",F68&lt;&gt;""),IF(F68&gt;E68,3,IF(E68=F68,1,0)),"")</f>
+        <f>IF(AND(E68&lt;&gt;"",F68&lt;&gt;""),IF(F68&gt;E68,3,IF(E68=F68,2,0)),"")</f>
         <v/>
       </c>
       <c r="J68" s="33">
@@ -5888,11 +5867,11 @@
         </is>
       </c>
       <c r="H69" s="31">
-        <f>IF(AND(E69&lt;&gt;"",F69&lt;&gt;""),IF(E69&gt;F69,3,IF(E69=F69,1,0)),"")</f>
+        <f>IF(AND(E69&lt;&gt;"",F69&lt;&gt;""),IF(E69&gt;F69,3,IF(E69=F69,2,0)),"")</f>
         <v/>
       </c>
       <c r="I69" s="31">
-        <f>IF(AND(E69&lt;&gt;"",F69&lt;&gt;""),IF(F69&gt;E69,3,IF(E69=F69,1,0)),"")</f>
+        <f>IF(AND(E69&lt;&gt;"",F69&lt;&gt;""),IF(F69&gt;E69,3,IF(E69=F69,2,0)),"")</f>
         <v/>
       </c>
       <c r="J69" s="31">
@@ -5931,11 +5910,11 @@
         </is>
       </c>
       <c r="H70" s="31">
-        <f>IF(AND(E70&lt;&gt;"",F70&lt;&gt;""),IF(E70&gt;F70,3,IF(E70=F70,1,0)),"")</f>
+        <f>IF(AND(E70&lt;&gt;"",F70&lt;&gt;""),IF(E70&gt;F70,3,IF(E70=F70,2,0)),"")</f>
         <v/>
       </c>
       <c r="I70" s="31">
-        <f>IF(AND(E70&lt;&gt;"",F70&lt;&gt;""),IF(F70&gt;E70,3,IF(E70=F70,1,0)),"")</f>
+        <f>IF(AND(E70&lt;&gt;"",F70&lt;&gt;""),IF(F70&gt;E70,3,IF(E70=F70,2,0)),"")</f>
         <v/>
       </c>
       <c r="J70" s="31">
@@ -5974,11 +5953,11 @@
         </is>
       </c>
       <c r="H71" s="39">
-        <f>IF(AND(E71&lt;&gt;"",F71&lt;&gt;""),IF(E71&gt;F71,3,IF(E71=F71,1,0)),"")</f>
+        <f>IF(AND(E71&lt;&gt;"",F71&lt;&gt;""),IF(E71&gt;F71,3,IF(E71=F71,2,0)),"")</f>
         <v/>
       </c>
       <c r="I71" s="39">
-        <f>IF(AND(E71&lt;&gt;"",F71&lt;&gt;""),IF(F71&gt;E71,3,IF(E71=F71,1,0)),"")</f>
+        <f>IF(AND(E71&lt;&gt;"",F71&lt;&gt;""),IF(F71&gt;E71,3,IF(E71=F71,2,0)),"")</f>
         <v/>
       </c>
       <c r="J71" s="39">
@@ -6017,11 +5996,11 @@
         </is>
       </c>
       <c r="H72" s="39">
-        <f>IF(AND(E72&lt;&gt;"",F72&lt;&gt;""),IF(E72&gt;F72,3,IF(E72=F72,1,0)),"")</f>
+        <f>IF(AND(E72&lt;&gt;"",F72&lt;&gt;""),IF(E72&gt;F72,3,IF(E72=F72,2,0)),"")</f>
         <v/>
       </c>
       <c r="I72" s="39">
-        <f>IF(AND(E72&lt;&gt;"",F72&lt;&gt;""),IF(F72&gt;E72,3,IF(E72=F72,1,0)),"")</f>
+        <f>IF(AND(E72&lt;&gt;"",F72&lt;&gt;""),IF(F72&gt;E72,3,IF(E72=F72,2,0)),"")</f>
         <v/>
       </c>
       <c r="J72" s="39">
@@ -6060,11 +6039,11 @@
         </is>
       </c>
       <c r="H73" s="37">
-        <f>IF(AND(E73&lt;&gt;"",F73&lt;&gt;""),IF(E73&gt;F73,3,IF(E73=F73,1,0)),"")</f>
+        <f>IF(AND(E73&lt;&gt;"",F73&lt;&gt;""),IF(E73&gt;F73,3,IF(E73=F73,2,0)),"")</f>
         <v/>
       </c>
       <c r="I73" s="37">
-        <f>IF(AND(E73&lt;&gt;"",F73&lt;&gt;""),IF(F73&gt;E73,3,IF(E73=F73,1,0)),"")</f>
+        <f>IF(AND(E73&lt;&gt;"",F73&lt;&gt;""),IF(F73&gt;E73,3,IF(E73=F73,2,0)),"")</f>
         <v/>
       </c>
       <c r="J73" s="37">
@@ -6103,11 +6082,11 @@
         </is>
       </c>
       <c r="H74" s="37">
-        <f>IF(AND(E74&lt;&gt;"",F74&lt;&gt;""),IF(E74&gt;F74,3,IF(E74=F74,1,0)),"")</f>
+        <f>IF(AND(E74&lt;&gt;"",F74&lt;&gt;""),IF(E74&gt;F74,3,IF(E74=F74,2,0)),"")</f>
         <v/>
       </c>
       <c r="I74" s="37">
-        <f>IF(AND(E74&lt;&gt;"",F74&lt;&gt;""),IF(F74&gt;E74,3,IF(E74=F74,1,0)),"")</f>
+        <f>IF(AND(E74&lt;&gt;"",F74&lt;&gt;""),IF(F74&gt;E74,3,IF(E74=F74,2,0)),"")</f>
         <v/>
       </c>
       <c r="J74" s="37">
@@ -6146,11 +6125,11 @@
         </is>
       </c>
       <c r="H75" s="41">
-        <f>IF(AND(E75&lt;&gt;"",F75&lt;&gt;""),IF(E75&gt;F75,3,IF(E75=F75,1,0)),"")</f>
+        <f>IF(AND(E75&lt;&gt;"",F75&lt;&gt;""),IF(E75&gt;F75,3,IF(E75=F75,2,0)),"")</f>
         <v/>
       </c>
       <c r="I75" s="41">
-        <f>IF(AND(E75&lt;&gt;"",F75&lt;&gt;""),IF(F75&gt;E75,3,IF(E75=F75,1,0)),"")</f>
+        <f>IF(AND(E75&lt;&gt;"",F75&lt;&gt;""),IF(F75&gt;E75,3,IF(E75=F75,2,0)),"")</f>
         <v/>
       </c>
       <c r="J75" s="41">
@@ -6189,11 +6168,11 @@
         </is>
       </c>
       <c r="H76" s="41">
-        <f>IF(AND(E76&lt;&gt;"",F76&lt;&gt;""),IF(E76&gt;F76,3,IF(E76=F76,1,0)),"")</f>
+        <f>IF(AND(E76&lt;&gt;"",F76&lt;&gt;""),IF(E76&gt;F76,3,IF(E76=F76,2,0)),"")</f>
         <v/>
       </c>
       <c r="I76" s="41">
-        <f>IF(AND(E76&lt;&gt;"",F76&lt;&gt;""),IF(F76&gt;E76,3,IF(E76=F76,1,0)),"")</f>
+        <f>IF(AND(E76&lt;&gt;"",F76&lt;&gt;""),IF(F76&gt;E76,3,IF(E76=F76,2,0)),"")</f>
         <v/>
       </c>
       <c r="J76" s="41">
@@ -6232,11 +6211,11 @@
         </is>
       </c>
       <c r="H77" s="43">
-        <f>IF(AND(E77&lt;&gt;"",F77&lt;&gt;""),IF(E77&gt;F77,3,IF(E77=F77,1,0)),"")</f>
+        <f>IF(AND(E77&lt;&gt;"",F77&lt;&gt;""),IF(E77&gt;F77,3,IF(E77=F77,2,0)),"")</f>
         <v/>
       </c>
       <c r="I77" s="43">
-        <f>IF(AND(E77&lt;&gt;"",F77&lt;&gt;""),IF(F77&gt;E77,3,IF(E77=F77,1,0)),"")</f>
+        <f>IF(AND(E77&lt;&gt;"",F77&lt;&gt;""),IF(F77&gt;E77,3,IF(E77=F77,2,0)),"")</f>
         <v/>
       </c>
       <c r="J77" s="43">
@@ -6275,11 +6254,11 @@
         </is>
       </c>
       <c r="H78" s="43">
-        <f>IF(AND(E78&lt;&gt;"",F78&lt;&gt;""),IF(E78&gt;F78,3,IF(E78=F78,1,0)),"")</f>
+        <f>IF(AND(E78&lt;&gt;"",F78&lt;&gt;""),IF(E78&gt;F78,3,IF(E78=F78,2,0)),"")</f>
         <v/>
       </c>
       <c r="I78" s="43">
-        <f>IF(AND(E78&lt;&gt;"",F78&lt;&gt;""),IF(F78&gt;E78,3,IF(E78=F78,1,0)),"")</f>
+        <f>IF(AND(E78&lt;&gt;"",F78&lt;&gt;""),IF(F78&gt;E78,3,IF(E78=F78,2,0)),"")</f>
         <v/>
       </c>
       <c r="J78" s="43">
@@ -6318,11 +6297,11 @@
         </is>
       </c>
       <c r="H79" s="43">
-        <f>IF(AND(E79&lt;&gt;"",F79&lt;&gt;""),IF(E79&gt;F79,3,IF(E79=F79,1,0)),"")</f>
+        <f>IF(AND(E79&lt;&gt;"",F79&lt;&gt;""),IF(E79&gt;F79,3,IF(E79=F79,2,0)),"")</f>
         <v/>
       </c>
       <c r="I79" s="43">
-        <f>IF(AND(E79&lt;&gt;"",F79&lt;&gt;""),IF(F79&gt;E79,3,IF(E79=F79,1,0)),"")</f>
+        <f>IF(AND(E79&lt;&gt;"",F79&lt;&gt;""),IF(F79&gt;E79,3,IF(E79=F79,2,0)),"")</f>
         <v/>
       </c>
       <c r="J79" s="43">
@@ -6361,11 +6340,11 @@
         </is>
       </c>
       <c r="H80" s="43">
-        <f>IF(AND(E80&lt;&gt;"",F80&lt;&gt;""),IF(E80&gt;F80,3,IF(E80=F80,1,0)),"")</f>
+        <f>IF(AND(E80&lt;&gt;"",F80&lt;&gt;""),IF(E80&gt;F80,3,IF(E80=F80,2,0)),"")</f>
         <v/>
       </c>
       <c r="I80" s="43">
-        <f>IF(AND(E80&lt;&gt;"",F80&lt;&gt;""),IF(F80&gt;E80,3,IF(E80=F80,1,0)),"")</f>
+        <f>IF(AND(E80&lt;&gt;"",F80&lt;&gt;""),IF(F80&gt;E80,3,IF(E80=F80,2,0)),"")</f>
         <v/>
       </c>
       <c r="J80" s="43">
@@ -6404,11 +6383,11 @@
         </is>
       </c>
       <c r="H81" s="43">
-        <f>IF(AND(E81&lt;&gt;"",F81&lt;&gt;""),IF(E81&gt;F81,3,IF(E81=F81,1,0)),"")</f>
+        <f>IF(AND(E81&lt;&gt;"",F81&lt;&gt;""),IF(E81&gt;F81,3,IF(E81=F81,2,0)),"")</f>
         <v/>
       </c>
       <c r="I81" s="43">
-        <f>IF(AND(E81&lt;&gt;"",F81&lt;&gt;""),IF(F81&gt;E81,3,IF(E81=F81,1,0)),"")</f>
+        <f>IF(AND(E81&lt;&gt;"",F81&lt;&gt;""),IF(F81&gt;E81,3,IF(E81=F81,2,0)),"")</f>
         <v/>
       </c>
       <c r="J81" s="43">
@@ -6447,11 +6426,11 @@
         </is>
       </c>
       <c r="H82" s="43">
-        <f>IF(AND(E82&lt;&gt;"",F82&lt;&gt;""),IF(E82&gt;F82,3,IF(E82=F82,1,0)),"")</f>
+        <f>IF(AND(E82&lt;&gt;"",F82&lt;&gt;""),IF(E82&gt;F82,3,IF(E82=F82,2,0)),"")</f>
         <v/>
       </c>
       <c r="I82" s="43">
-        <f>IF(AND(E82&lt;&gt;"",F82&lt;&gt;""),IF(F82&gt;E82,3,IF(E82=F82,1,0)),"")</f>
+        <f>IF(AND(E82&lt;&gt;"",F82&lt;&gt;""),IF(F82&gt;E82,3,IF(E82=F82,2,0)),"")</f>
         <v/>
       </c>
       <c r="J82" s="43">
@@ -6490,11 +6469,11 @@
         </is>
       </c>
       <c r="H83" s="43">
-        <f>IF(AND(E83&lt;&gt;"",F83&lt;&gt;""),IF(E83&gt;F83,3,IF(E83=F83,1,0)),"")</f>
+        <f>IF(AND(E83&lt;&gt;"",F83&lt;&gt;""),IF(E83&gt;F83,3,IF(E83=F83,2,0)),"")</f>
         <v/>
       </c>
       <c r="I83" s="43">
-        <f>IF(AND(E83&lt;&gt;"",F83&lt;&gt;""),IF(F83&gt;E83,3,IF(E83=F83,1,0)),"")</f>
+        <f>IF(AND(E83&lt;&gt;"",F83&lt;&gt;""),IF(F83&gt;E83,3,IF(E83=F83,2,0)),"")</f>
         <v/>
       </c>
       <c r="J83" s="43">
@@ -6533,11 +6512,11 @@
         </is>
       </c>
       <c r="H84" s="43">
-        <f>IF(AND(E84&lt;&gt;"",F84&lt;&gt;""),IF(E84&gt;F84,3,IF(E84=F84,1,0)),"")</f>
+        <f>IF(AND(E84&lt;&gt;"",F84&lt;&gt;""),IF(E84&gt;F84,3,IF(E84=F84,2,0)),"")</f>
         <v/>
       </c>
       <c r="I84" s="43">
-        <f>IF(AND(E84&lt;&gt;"",F84&lt;&gt;""),IF(F84&gt;E84,3,IF(E84=F84,1,0)),"")</f>
+        <f>IF(AND(E84&lt;&gt;"",F84&lt;&gt;""),IF(F84&gt;E84,3,IF(E84=F84,2,0)),"")</f>
         <v/>
       </c>
       <c r="J84" s="43">
@@ -6576,11 +6555,11 @@
         </is>
       </c>
       <c r="H85" s="43">
-        <f>IF(AND(E85&lt;&gt;"",F85&lt;&gt;""),IF(E85&gt;F85,3,IF(E85=F85,1,0)),"")</f>
+        <f>IF(AND(E85&lt;&gt;"",F85&lt;&gt;""),IF(E85&gt;F85,3,IF(E85=F85,2,0)),"")</f>
         <v/>
       </c>
       <c r="I85" s="43">
-        <f>IF(AND(E85&lt;&gt;"",F85&lt;&gt;""),IF(F85&gt;E85,3,IF(E85=F85,1,0)),"")</f>
+        <f>IF(AND(E85&lt;&gt;"",F85&lt;&gt;""),IF(F85&gt;E85,3,IF(E85=F85,2,0)),"")</f>
         <v/>
       </c>
       <c r="J85" s="43">
@@ -6619,11 +6598,11 @@
         </is>
       </c>
       <c r="H86" s="43">
-        <f>IF(AND(E86&lt;&gt;"",F86&lt;&gt;""),IF(E86&gt;F86,3,IF(E86=F86,1,0)),"")</f>
+        <f>IF(AND(E86&lt;&gt;"",F86&lt;&gt;""),IF(E86&gt;F86,3,IF(E86=F86,2,0)),"")</f>
         <v/>
       </c>
       <c r="I86" s="43">
-        <f>IF(AND(E86&lt;&gt;"",F86&lt;&gt;""),IF(F86&gt;E86,3,IF(E86=F86,1,0)),"")</f>
+        <f>IF(AND(E86&lt;&gt;"",F86&lt;&gt;""),IF(F86&gt;E86,3,IF(E86=F86,2,0)),"")</f>
         <v/>
       </c>
       <c r="J86" s="43">
@@ -6662,11 +6641,11 @@
         </is>
       </c>
       <c r="H87" s="43">
-        <f>IF(AND(E87&lt;&gt;"",F87&lt;&gt;""),IF(E87&gt;F87,3,IF(E87=F87,1,0)),"")</f>
+        <f>IF(AND(E87&lt;&gt;"",F87&lt;&gt;""),IF(E87&gt;F87,3,IF(E87=F87,2,0)),"")</f>
         <v/>
       </c>
       <c r="I87" s="43">
-        <f>IF(AND(E87&lt;&gt;"",F87&lt;&gt;""),IF(F87&gt;E87,3,IF(E87=F87,1,0)),"")</f>
+        <f>IF(AND(E87&lt;&gt;"",F87&lt;&gt;""),IF(F87&gt;E87,3,IF(E87=F87,2,0)),"")</f>
         <v/>
       </c>
       <c r="J87" s="43">
@@ -6705,11 +6684,11 @@
         </is>
       </c>
       <c r="H88" s="43">
-        <f>IF(AND(E88&lt;&gt;"",F88&lt;&gt;""),IF(E88&gt;F88,3,IF(E88=F88,1,0)),"")</f>
+        <f>IF(AND(E88&lt;&gt;"",F88&lt;&gt;""),IF(E88&gt;F88,3,IF(E88=F88,2,0)),"")</f>
         <v/>
       </c>
       <c r="I88" s="43">
-        <f>IF(AND(E88&lt;&gt;"",F88&lt;&gt;""),IF(F88&gt;E88,3,IF(E88=F88,1,0)),"")</f>
+        <f>IF(AND(E88&lt;&gt;"",F88&lt;&gt;""),IF(F88&gt;E88,3,IF(E88=F88,2,0)),"")</f>
         <v/>
       </c>
       <c r="J88" s="43">
@@ -6748,11 +6727,11 @@
         </is>
       </c>
       <c r="H89" s="43">
-        <f>IF(AND(E89&lt;&gt;"",F89&lt;&gt;""),IF(E89&gt;F89,3,IF(E89=F89,1,0)),"")</f>
+        <f>IF(AND(E89&lt;&gt;"",F89&lt;&gt;""),IF(E89&gt;F89,3,IF(E89=F89,2,0)),"")</f>
         <v/>
       </c>
       <c r="I89" s="43">
-        <f>IF(AND(E89&lt;&gt;"",F89&lt;&gt;""),IF(F89&gt;E89,3,IF(E89=F89,1,0)),"")</f>
+        <f>IF(AND(E89&lt;&gt;"",F89&lt;&gt;""),IF(F89&gt;E89,3,IF(E89=F89,2,0)),"")</f>
         <v/>
       </c>
       <c r="J89" s="43">
@@ -6791,11 +6770,11 @@
         </is>
       </c>
       <c r="H90" s="43">
-        <f>IF(AND(E90&lt;&gt;"",F90&lt;&gt;""),IF(E90&gt;F90,3,IF(E90=F90,1,0)),"")</f>
+        <f>IF(AND(E90&lt;&gt;"",F90&lt;&gt;""),IF(E90&gt;F90,3,IF(E90=F90,2,0)),"")</f>
         <v/>
       </c>
       <c r="I90" s="43">
-        <f>IF(AND(E90&lt;&gt;"",F90&lt;&gt;""),IF(F90&gt;E90,3,IF(E90=F90,1,0)),"")</f>
+        <f>IF(AND(E90&lt;&gt;"",F90&lt;&gt;""),IF(F90&gt;E90,3,IF(E90=F90,2,0)),"")</f>
         <v/>
       </c>
       <c r="J90" s="43">
@@ -6834,11 +6813,11 @@
         </is>
       </c>
       <c r="H91" s="43">
-        <f>IF(AND(E91&lt;&gt;"",F91&lt;&gt;""),IF(E91&gt;F91,3,IF(E91=F91,1,0)),"")</f>
+        <f>IF(AND(E91&lt;&gt;"",F91&lt;&gt;""),IF(E91&gt;F91,3,IF(E91=F91,2,0)),"")</f>
         <v/>
       </c>
       <c r="I91" s="43">
-        <f>IF(AND(E91&lt;&gt;"",F91&lt;&gt;""),IF(F91&gt;E91,3,IF(E91=F91,1,0)),"")</f>
+        <f>IF(AND(E91&lt;&gt;"",F91&lt;&gt;""),IF(F91&gt;E91,3,IF(E91=F91,2,0)),"")</f>
         <v/>
       </c>
       <c r="J91" s="43">
@@ -6877,11 +6856,11 @@
         </is>
       </c>
       <c r="H92" s="43">
-        <f>IF(AND(E92&lt;&gt;"",F92&lt;&gt;""),IF(E92&gt;F92,3,IF(E92=F92,1,0)),"")</f>
+        <f>IF(AND(E92&lt;&gt;"",F92&lt;&gt;""),IF(E92&gt;F92,3,IF(E92=F92,2,0)),"")</f>
         <v/>
       </c>
       <c r="I92" s="43">
-        <f>IF(AND(E92&lt;&gt;"",F92&lt;&gt;""),IF(F92&gt;E92,3,IF(E92=F92,1,0)),"")</f>
+        <f>IF(AND(E92&lt;&gt;"",F92&lt;&gt;""),IF(F92&gt;E92,3,IF(E92=F92,2,0)),"")</f>
         <v/>
       </c>
       <c r="J92" s="43">
@@ -6920,11 +6899,11 @@
         </is>
       </c>
       <c r="H93" s="43">
-        <f>IF(AND(E93&lt;&gt;"",F93&lt;&gt;""),IF(E93&gt;F93,3,IF(E93=F93,1,0)),"")</f>
+        <f>IF(AND(E93&lt;&gt;"",F93&lt;&gt;""),IF(E93&gt;F93,3,IF(E93=F93,2,0)),"")</f>
         <v/>
       </c>
       <c r="I93" s="43">
-        <f>IF(AND(E93&lt;&gt;"",F93&lt;&gt;""),IF(F93&gt;E93,3,IF(E93=F93,1,0)),"")</f>
+        <f>IF(AND(E93&lt;&gt;"",F93&lt;&gt;""),IF(F93&gt;E93,3,IF(E93=F93,2,0)),"")</f>
         <v/>
       </c>
       <c r="J93" s="43">
@@ -6963,11 +6942,11 @@
         </is>
       </c>
       <c r="H94" s="43">
-        <f>IF(AND(E94&lt;&gt;"",F94&lt;&gt;""),IF(E94&gt;F94,3,IF(E94=F94,1,0)),"")</f>
+        <f>IF(AND(E94&lt;&gt;"",F94&lt;&gt;""),IF(E94&gt;F94,3,IF(E94=F94,2,0)),"")</f>
         <v/>
       </c>
       <c r="I94" s="43">
-        <f>IF(AND(E94&lt;&gt;"",F94&lt;&gt;""),IF(F94&gt;E94,3,IF(E94=F94,1,0)),"")</f>
+        <f>IF(AND(E94&lt;&gt;"",F94&lt;&gt;""),IF(F94&gt;E94,3,IF(E94=F94,2,0)),"")</f>
         <v/>
       </c>
       <c r="J94" s="43">
@@ -7006,11 +6985,11 @@
         </is>
       </c>
       <c r="H95" s="43">
-        <f>IF(AND(E95&lt;&gt;"",F95&lt;&gt;""),IF(E95&gt;F95,3,IF(E95=F95,1,0)),"")</f>
+        <f>IF(AND(E95&lt;&gt;"",F95&lt;&gt;""),IF(E95&gt;F95,3,IF(E95=F95,2,0)),"")</f>
         <v/>
       </c>
       <c r="I95" s="43">
-        <f>IF(AND(E95&lt;&gt;"",F95&lt;&gt;""),IF(F95&gt;E95,3,IF(E95=F95,1,0)),"")</f>
+        <f>IF(AND(E95&lt;&gt;"",F95&lt;&gt;""),IF(F95&gt;E95,3,IF(E95=F95,2,0)),"")</f>
         <v/>
       </c>
       <c r="J95" s="43">
@@ -7049,11 +7028,11 @@
         </is>
       </c>
       <c r="H96" s="43">
-        <f>IF(AND(E96&lt;&gt;"",F96&lt;&gt;""),IF(E96&gt;F96,3,IF(E96=F96,1,0)),"")</f>
+        <f>IF(AND(E96&lt;&gt;"",F96&lt;&gt;""),IF(E96&gt;F96,3,IF(E96=F96,2,0)),"")</f>
         <v/>
       </c>
       <c r="I96" s="43">
-        <f>IF(AND(E96&lt;&gt;"",F96&lt;&gt;""),IF(F96&gt;E96,3,IF(E96=F96,1,0)),"")</f>
+        <f>IF(AND(E96&lt;&gt;"",F96&lt;&gt;""),IF(F96&gt;E96,3,IF(E96=F96,2,0)),"")</f>
         <v/>
       </c>
       <c r="J96" s="43">
@@ -7092,11 +7071,11 @@
         </is>
       </c>
       <c r="H97" s="43">
-        <f>IF(AND(E97&lt;&gt;"",F97&lt;&gt;""),IF(E97&gt;F97,3,IF(E97=F97,1,0)),"")</f>
+        <f>IF(AND(E97&lt;&gt;"",F97&lt;&gt;""),IF(E97&gt;F97,3,IF(E97=F97,2,0)),"")</f>
         <v/>
       </c>
       <c r="I97" s="43">
-        <f>IF(AND(E97&lt;&gt;"",F97&lt;&gt;""),IF(F97&gt;E97,3,IF(E97=F97,1,0)),"")</f>
+        <f>IF(AND(E97&lt;&gt;"",F97&lt;&gt;""),IF(F97&gt;E97,3,IF(E97=F97,2,0)),"")</f>
         <v/>
       </c>
       <c r="J97" s="43">
@@ -7135,11 +7114,11 @@
         </is>
       </c>
       <c r="H98" s="43">
-        <f>IF(AND(E98&lt;&gt;"",F98&lt;&gt;""),IF(E98&gt;F98,3,IF(E98=F98,1,0)),"")</f>
+        <f>IF(AND(E98&lt;&gt;"",F98&lt;&gt;""),IF(E98&gt;F98,3,IF(E98=F98,2,0)),"")</f>
         <v/>
       </c>
       <c r="I98" s="43">
-        <f>IF(AND(E98&lt;&gt;"",F98&lt;&gt;""),IF(F98&gt;E98,3,IF(E98=F98,1,0)),"")</f>
+        <f>IF(AND(E98&lt;&gt;"",F98&lt;&gt;""),IF(F98&gt;E98,3,IF(E98=F98,2,0)),"")</f>
         <v/>
       </c>
       <c r="J98" s="43">
@@ -7178,11 +7157,11 @@
         </is>
       </c>
       <c r="H99" s="43">
-        <f>IF(AND(E99&lt;&gt;"",F99&lt;&gt;""),IF(E99&gt;F99,3,IF(E99=F99,1,0)),"")</f>
+        <f>IF(AND(E99&lt;&gt;"",F99&lt;&gt;""),IF(E99&gt;F99,3,IF(E99=F99,2,0)),"")</f>
         <v/>
       </c>
       <c r="I99" s="43">
-        <f>IF(AND(E99&lt;&gt;"",F99&lt;&gt;""),IF(F99&gt;E99,3,IF(E99=F99,1,0)),"")</f>
+        <f>IF(AND(E99&lt;&gt;"",F99&lt;&gt;""),IF(F99&gt;E99,3,IF(E99=F99,2,0)),"")</f>
         <v/>
       </c>
       <c r="J99" s="43">
@@ -7221,11 +7200,11 @@
         </is>
       </c>
       <c r="H100" s="43">
-        <f>IF(AND(E100&lt;&gt;"",F100&lt;&gt;""),IF(E100&gt;F100,3,IF(E100=F100,1,0)),"")</f>
+        <f>IF(AND(E100&lt;&gt;"",F100&lt;&gt;""),IF(E100&gt;F100,3,IF(E100=F100,2,0)),"")</f>
         <v/>
       </c>
       <c r="I100" s="43">
-        <f>IF(AND(E100&lt;&gt;"",F100&lt;&gt;""),IF(F100&gt;E100,3,IF(E100=F100,1,0)),"")</f>
+        <f>IF(AND(E100&lt;&gt;"",F100&lt;&gt;""),IF(F100&gt;E100,3,IF(E100=F100,2,0)),"")</f>
         <v/>
       </c>
       <c r="J100" s="43">
@@ -7264,11 +7243,11 @@
         </is>
       </c>
       <c r="H101" s="43">
-        <f>IF(AND(E101&lt;&gt;"",F101&lt;&gt;""),IF(E101&gt;F101,3,IF(E101=F101,1,0)),"")</f>
+        <f>IF(AND(E101&lt;&gt;"",F101&lt;&gt;""),IF(E101&gt;F101,3,IF(E101=F101,2,0)),"")</f>
         <v/>
       </c>
       <c r="I101" s="43">
-        <f>IF(AND(E101&lt;&gt;"",F101&lt;&gt;""),IF(F101&gt;E101,3,IF(E101=F101,1,0)),"")</f>
+        <f>IF(AND(E101&lt;&gt;"",F101&lt;&gt;""),IF(F101&gt;E101,3,IF(E101=F101,2,0)),"")</f>
         <v/>
       </c>
       <c r="J101" s="43">
@@ -7307,11 +7286,11 @@
         </is>
       </c>
       <c r="H102" s="43">
-        <f>IF(AND(E102&lt;&gt;"",F102&lt;&gt;""),IF(E102&gt;F102,3,IF(E102=F102,1,0)),"")</f>
+        <f>IF(AND(E102&lt;&gt;"",F102&lt;&gt;""),IF(E102&gt;F102,3,IF(E102=F102,2,0)),"")</f>
         <v/>
       </c>
       <c r="I102" s="43">
-        <f>IF(AND(E102&lt;&gt;"",F102&lt;&gt;""),IF(F102&gt;E102,3,IF(E102=F102,1,0)),"")</f>
+        <f>IF(AND(E102&lt;&gt;"",F102&lt;&gt;""),IF(F102&gt;E102,3,IF(E102=F102,2,0)),"")</f>
         <v/>
       </c>
       <c r="J102" s="43">
@@ -7350,11 +7329,11 @@
         </is>
       </c>
       <c r="H103" s="43">
-        <f>IF(AND(E103&lt;&gt;"",F103&lt;&gt;""),IF(E103&gt;F103,3,IF(E103=F103,1,0)),"")</f>
+        <f>IF(AND(E103&lt;&gt;"",F103&lt;&gt;""),IF(E103&gt;F103,3,IF(E103=F103,2,0)),"")</f>
         <v/>
       </c>
       <c r="I103" s="43">
-        <f>IF(AND(E103&lt;&gt;"",F103&lt;&gt;""),IF(F103&gt;E103,3,IF(E103=F103,1,0)),"")</f>
+        <f>IF(AND(E103&lt;&gt;"",F103&lt;&gt;""),IF(F103&gt;E103,3,IF(E103=F103,2,0)),"")</f>
         <v/>
       </c>
       <c r="J103" s="43">
@@ -7393,11 +7372,11 @@
         </is>
       </c>
       <c r="H104" s="43">
-        <f>IF(AND(E104&lt;&gt;"",F104&lt;&gt;""),IF(E104&gt;F104,3,IF(E104=F104,1,0)),"")</f>
+        <f>IF(AND(E104&lt;&gt;"",F104&lt;&gt;""),IF(E104&gt;F104,3,IF(E104=F104,2,0)),"")</f>
         <v/>
       </c>
       <c r="I104" s="43">
-        <f>IF(AND(E104&lt;&gt;"",F104&lt;&gt;""),IF(F104&gt;E104,3,IF(E104=F104,1,0)),"")</f>
+        <f>IF(AND(E104&lt;&gt;"",F104&lt;&gt;""),IF(F104&gt;E104,3,IF(E104=F104,2,0)),"")</f>
         <v/>
       </c>
       <c r="J104" s="43">
@@ -7436,11 +7415,11 @@
         </is>
       </c>
       <c r="H105" s="43">
-        <f>IF(AND(E105&lt;&gt;"",F105&lt;&gt;""),IF(E105&gt;F105,3,IF(E105=F105,1,0)),"")</f>
+        <f>IF(AND(E105&lt;&gt;"",F105&lt;&gt;""),IF(E105&gt;F105,3,IF(E105=F105,2,0)),"")</f>
         <v/>
       </c>
       <c r="I105" s="43">
-        <f>IF(AND(E105&lt;&gt;"",F105&lt;&gt;""),IF(F105&gt;E105,3,IF(E105=F105,1,0)),"")</f>
+        <f>IF(AND(E105&lt;&gt;"",F105&lt;&gt;""),IF(F105&gt;E105,3,IF(E105=F105,2,0)),"")</f>
         <v/>
       </c>
       <c r="J105" s="43">
@@ -7479,11 +7458,11 @@
         </is>
       </c>
       <c r="H106" s="43">
-        <f>IF(AND(E106&lt;&gt;"",F106&lt;&gt;""),IF(E106&gt;F106,3,IF(E106=F106,1,0)),"")</f>
+        <f>IF(AND(E106&lt;&gt;"",F106&lt;&gt;""),IF(E106&gt;F106,3,IF(E106=F106,2,0)),"")</f>
         <v/>
       </c>
       <c r="I106" s="43">
-        <f>IF(AND(E106&lt;&gt;"",F106&lt;&gt;""),IF(F106&gt;E106,3,IF(E106=F106,1,0)),"")</f>
+        <f>IF(AND(E106&lt;&gt;"",F106&lt;&gt;""),IF(F106&gt;E106,3,IF(E106=F106,2,0)),"")</f>
         <v/>
       </c>
       <c r="J106" s="43">
@@ -7522,11 +7501,11 @@
         </is>
       </c>
       <c r="H107" s="43">
-        <f>IF(AND(E107&lt;&gt;"",F107&lt;&gt;""),IF(E107&gt;F107,3,IF(E107=F107,1,0)),"")</f>
+        <f>IF(AND(E107&lt;&gt;"",F107&lt;&gt;""),IF(E107&gt;F107,3,IF(E107=F107,2,0)),"")</f>
         <v/>
       </c>
       <c r="I107" s="43">
-        <f>IF(AND(E107&lt;&gt;"",F107&lt;&gt;""),IF(F107&gt;E107,3,IF(E107=F107,1,0)),"")</f>
+        <f>IF(AND(E107&lt;&gt;"",F107&lt;&gt;""),IF(F107&gt;E107,3,IF(E107=F107,2,0)),"")</f>
         <v/>
       </c>
       <c r="J107" s="43">
@@ -7565,11 +7544,11 @@
         </is>
       </c>
       <c r="H108" s="43">
-        <f>IF(AND(E108&lt;&gt;"",F108&lt;&gt;""),IF(E108&gt;F108,3,IF(E108=F108,1,0)),"")</f>
+        <f>IF(AND(E108&lt;&gt;"",F108&lt;&gt;""),IF(E108&gt;F108,3,IF(E108=F108,2,0)),"")</f>
         <v/>
       </c>
       <c r="I108" s="43">
-        <f>IF(AND(E108&lt;&gt;"",F108&lt;&gt;""),IF(F108&gt;E108,3,IF(E108=F108,1,0)),"")</f>
+        <f>IF(AND(E108&lt;&gt;"",F108&lt;&gt;""),IF(F108&gt;E108,3,IF(E108=F108,2,0)),"")</f>
         <v/>
       </c>
       <c r="J108" s="43">

</xml_diff>

<commit_message>
Fix Golden Boot: ranking now handles ties sequentially + multiple rows per match
</commit_message>
<xml_diff>
--- a/WorldCup2026_Sweepstake.xlsx
+++ b/WorldCup2026_Sweepstake.xlsx
@@ -706,7 +706,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -714,7 +713,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -743,7 +741,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
@@ -793,7 +790,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
@@ -822,7 +818,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
@@ -851,7 +846,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
@@ -901,7 +895,6 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
@@ -993,7 +986,6 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
@@ -1036,7 +1028,6 @@
         </is>
       </c>
     </row>
-    <row r="56"/>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
@@ -1072,7 +1063,6 @@
         </is>
       </c>
     </row>
-    <row r="62"/>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
@@ -15386,7 +15376,7 @@
       </c>
       <c r="D4" s="52" t="inlineStr">
         <is>
-          <t>Enter one row per scorer per match</t>
+          <t>Enter one row per goal scorer per match (multiple scorers per match OK)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -15550,7 +15540,7 @@
         <v/>
       </c>
       <c r="S6">
-        <f>IF(OR(B6="",COUNTIF($B$6:$B6,B6)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B6,$B$6:$B$305)=1)*($R$6:$R$305&gt;R6)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B6="",COUNTIF($B$6:$B6,B6)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R6)+(($R$6:$R$305=R6)*(ROW($B$6:$B$305)&lt;ROW(B6)))))+1)</f>
         <v/>
       </c>
       <c r="T6">
@@ -15618,7 +15608,7 @@
         <v/>
       </c>
       <c r="S7">
-        <f>IF(OR(B7="",COUNTIF($B$6:$B7,B7)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B7,$B$6:$B$305)=1)*($R$6:$R$305&gt;R7)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B7="",COUNTIF($B$6:$B7,B7)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R7)+(($R$6:$R$305=R7)*(ROW($B$6:$B$305)&lt;ROW(B7)))))+1)</f>
         <v/>
       </c>
       <c r="T7">
@@ -15686,7 +15676,7 @@
         <v/>
       </c>
       <c r="S8">
-        <f>IF(OR(B8="",COUNTIF($B$6:$B8,B8)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B8,$B$6:$B$305)=1)*($R$6:$R$305&gt;R8)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B8="",COUNTIF($B$6:$B8,B8)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R8)+(($R$6:$R$305=R8)*(ROW($B$6:$B$305)&lt;ROW(B8)))))+1)</f>
         <v/>
       </c>
       <c r="T8">
@@ -15754,7 +15744,7 @@
         <v/>
       </c>
       <c r="S9">
-        <f>IF(OR(B9="",COUNTIF($B$6:$B9,B9)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B9,$B$6:$B$305)=1)*($R$6:$R$305&gt;R9)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B9="",COUNTIF($B$6:$B9,B9)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R9)+(($R$6:$R$305=R9)*(ROW($B$6:$B$305)&lt;ROW(B9)))))+1)</f>
         <v/>
       </c>
       <c r="T9">
@@ -15822,7 +15812,7 @@
         <v/>
       </c>
       <c r="S10">
-        <f>IF(OR(B10="",COUNTIF($B$6:$B10,B10)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B10,$B$6:$B$305)=1)*($R$6:$R$305&gt;R10)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B10="",COUNTIF($B$6:$B10,B10)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R10)+(($R$6:$R$305=R10)*(ROW($B$6:$B$305)&lt;ROW(B10)))))+1)</f>
         <v/>
       </c>
       <c r="T10">
@@ -15890,7 +15880,7 @@
         <v/>
       </c>
       <c r="S11">
-        <f>IF(OR(B11="",COUNTIF($B$6:$B11,B11)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B11,$B$6:$B$305)=1)*($R$6:$R$305&gt;R11)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B11="",COUNTIF($B$6:$B11,B11)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R11)+(($R$6:$R$305=R11)*(ROW($B$6:$B$305)&lt;ROW(B11)))))+1)</f>
         <v/>
       </c>
       <c r="T11">
@@ -15958,7 +15948,7 @@
         <v/>
       </c>
       <c r="S12">
-        <f>IF(OR(B12="",COUNTIF($B$6:$B12,B12)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B12,$B$6:$B$305)=1)*($R$6:$R$305&gt;R12)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B12="",COUNTIF($B$6:$B12,B12)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R12)+(($R$6:$R$305=R12)*(ROW($B$6:$B$305)&lt;ROW(B12)))))+1)</f>
         <v/>
       </c>
       <c r="T12">
@@ -16026,7 +16016,7 @@
         <v/>
       </c>
       <c r="S13">
-        <f>IF(OR(B13="",COUNTIF($B$6:$B13,B13)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B13,$B$6:$B$305)=1)*($R$6:$R$305&gt;R13)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B13="",COUNTIF($B$6:$B13,B13)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R13)+(($R$6:$R$305=R13)*(ROW($B$6:$B$305)&lt;ROW(B13)))))+1)</f>
         <v/>
       </c>
       <c r="T13">
@@ -16094,7 +16084,7 @@
         <v/>
       </c>
       <c r="S14">
-        <f>IF(OR(B14="",COUNTIF($B$6:$B14,B14)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B14,$B$6:$B$305)=1)*($R$6:$R$305&gt;R14)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B14="",COUNTIF($B$6:$B14,B14)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R14)+(($R$6:$R$305=R14)*(ROW($B$6:$B$305)&lt;ROW(B14)))))+1)</f>
         <v/>
       </c>
       <c r="T14">
@@ -16162,7 +16152,7 @@
         <v/>
       </c>
       <c r="S15">
-        <f>IF(OR(B15="",COUNTIF($B$6:$B15,B15)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B15,$B$6:$B$305)=1)*($R$6:$R$305&gt;R15)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B15="",COUNTIF($B$6:$B15,B15)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R15)+(($R$6:$R$305=R15)*(ROW($B$6:$B$305)&lt;ROW(B15)))))+1)</f>
         <v/>
       </c>
       <c r="T15">
@@ -16230,7 +16220,7 @@
         <v/>
       </c>
       <c r="S16">
-        <f>IF(OR(B16="",COUNTIF($B$6:$B16,B16)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B16,$B$6:$B$305)=1)*($R$6:$R$305&gt;R16)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B16="",COUNTIF($B$6:$B16,B16)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R16)+(($R$6:$R$305=R16)*(ROW($B$6:$B$305)&lt;ROW(B16)))))+1)</f>
         <v/>
       </c>
       <c r="T16">
@@ -16298,7 +16288,7 @@
         <v/>
       </c>
       <c r="S17">
-        <f>IF(OR(B17="",COUNTIF($B$6:$B17,B17)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B17,$B$6:$B$305)=1)*($R$6:$R$305&gt;R17)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B17="",COUNTIF($B$6:$B17,B17)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R17)+(($R$6:$R$305=R17)*(ROW($B$6:$B$305)&lt;ROW(B17)))))+1)</f>
         <v/>
       </c>
       <c r="T17">
@@ -16366,7 +16356,7 @@
         <v/>
       </c>
       <c r="S18">
-        <f>IF(OR(B18="",COUNTIF($B$6:$B18,B18)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B18,$B$6:$B$305)=1)*($R$6:$R$305&gt;R18)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B18="",COUNTIF($B$6:$B18,B18)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R18)+(($R$6:$R$305=R18)*(ROW($B$6:$B$305)&lt;ROW(B18)))))+1)</f>
         <v/>
       </c>
       <c r="T18">
@@ -16434,7 +16424,7 @@
         <v/>
       </c>
       <c r="S19">
-        <f>IF(OR(B19="",COUNTIF($B$6:$B19,B19)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B19,$B$6:$B$305)=1)*($R$6:$R$305&gt;R19)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B19="",COUNTIF($B$6:$B19,B19)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R19)+(($R$6:$R$305=R19)*(ROW($B$6:$B$305)&lt;ROW(B19)))))+1)</f>
         <v/>
       </c>
       <c r="T19">
@@ -16502,7 +16492,7 @@
         <v/>
       </c>
       <c r="S20">
-        <f>IF(OR(B20="",COUNTIF($B$6:$B20,B20)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B20,$B$6:$B$305)=1)*($R$6:$R$305&gt;R20)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B20="",COUNTIF($B$6:$B20,B20)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R20)+(($R$6:$R$305=R20)*(ROW($B$6:$B$305)&lt;ROW(B20)))))+1)</f>
         <v/>
       </c>
       <c r="T20">
@@ -16570,7 +16560,7 @@
         <v/>
       </c>
       <c r="S21">
-        <f>IF(OR(B21="",COUNTIF($B$6:$B21,B21)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B21,$B$6:$B$305)=1)*($R$6:$R$305&gt;R21)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B21="",COUNTIF($B$6:$B21,B21)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R21)+(($R$6:$R$305=R21)*(ROW($B$6:$B$305)&lt;ROW(B21)))))+1)</f>
         <v/>
       </c>
       <c r="T21">
@@ -16638,7 +16628,7 @@
         <v/>
       </c>
       <c r="S22">
-        <f>IF(OR(B22="",COUNTIF($B$6:$B22,B22)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B22,$B$6:$B$305)=1)*($R$6:$R$305&gt;R22)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B22="",COUNTIF($B$6:$B22,B22)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R22)+(($R$6:$R$305=R22)*(ROW($B$6:$B$305)&lt;ROW(B22)))))+1)</f>
         <v/>
       </c>
       <c r="T22">
@@ -16706,7 +16696,7 @@
         <v/>
       </c>
       <c r="S23">
-        <f>IF(OR(B23="",COUNTIF($B$6:$B23,B23)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B23,$B$6:$B$305)=1)*($R$6:$R$305&gt;R23)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B23="",COUNTIF($B$6:$B23,B23)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R23)+(($R$6:$R$305=R23)*(ROW($B$6:$B$305)&lt;ROW(B23)))))+1)</f>
         <v/>
       </c>
       <c r="T23">
@@ -16774,7 +16764,7 @@
         <v/>
       </c>
       <c r="S24">
-        <f>IF(OR(B24="",COUNTIF($B$6:$B24,B24)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B24,$B$6:$B$305)=1)*($R$6:$R$305&gt;R24)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B24="",COUNTIF($B$6:$B24,B24)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R24)+(($R$6:$R$305=R24)*(ROW($B$6:$B$305)&lt;ROW(B24)))))+1)</f>
         <v/>
       </c>
       <c r="T24">
@@ -16842,7 +16832,7 @@
         <v/>
       </c>
       <c r="S25">
-        <f>IF(OR(B25="",COUNTIF($B$6:$B25,B25)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B25,$B$6:$B$305)=1)*($R$6:$R$305&gt;R25)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B25="",COUNTIF($B$6:$B25,B25)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R25)+(($R$6:$R$305=R25)*(ROW($B$6:$B$305)&lt;ROW(B25)))))+1)</f>
         <v/>
       </c>
       <c r="T25">
@@ -16910,7 +16900,7 @@
         <v/>
       </c>
       <c r="S26">
-        <f>IF(OR(B26="",COUNTIF($B$6:$B26,B26)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B26,$B$6:$B$305)=1)*($R$6:$R$305&gt;R26)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B26="",COUNTIF($B$6:$B26,B26)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R26)+(($R$6:$R$305=R26)*(ROW($B$6:$B$305)&lt;ROW(B26)))))+1)</f>
         <v/>
       </c>
       <c r="T26">
@@ -16978,7 +16968,7 @@
         <v/>
       </c>
       <c r="S27">
-        <f>IF(OR(B27="",COUNTIF($B$6:$B27,B27)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B27,$B$6:$B$305)=1)*($R$6:$R$305&gt;R27)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B27="",COUNTIF($B$6:$B27,B27)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R27)+(($R$6:$R$305=R27)*(ROW($B$6:$B$305)&lt;ROW(B27)))))+1)</f>
         <v/>
       </c>
       <c r="T27">
@@ -17046,7 +17036,7 @@
         <v/>
       </c>
       <c r="S28">
-        <f>IF(OR(B28="",COUNTIF($B$6:$B28,B28)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B28,$B$6:$B$305)=1)*($R$6:$R$305&gt;R28)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B28="",COUNTIF($B$6:$B28,B28)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R28)+(($R$6:$R$305=R28)*(ROW($B$6:$B$305)&lt;ROW(B28)))))+1)</f>
         <v/>
       </c>
       <c r="T28">
@@ -17114,7 +17104,7 @@
         <v/>
       </c>
       <c r="S29">
-        <f>IF(OR(B29="",COUNTIF($B$6:$B29,B29)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B29,$B$6:$B$305)=1)*($R$6:$R$305&gt;R29)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B29="",COUNTIF($B$6:$B29,B29)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R29)+(($R$6:$R$305=R29)*(ROW($B$6:$B$305)&lt;ROW(B29)))))+1)</f>
         <v/>
       </c>
       <c r="T29">
@@ -17182,7 +17172,7 @@
         <v/>
       </c>
       <c r="S30">
-        <f>IF(OR(B30="",COUNTIF($B$6:$B30,B30)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B30,$B$6:$B$305)=1)*($R$6:$R$305&gt;R30)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B30="",COUNTIF($B$6:$B30,B30)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R30)+(($R$6:$R$305=R30)*(ROW($B$6:$B$305)&lt;ROW(B30)))))+1)</f>
         <v/>
       </c>
       <c r="T30">
@@ -17250,7 +17240,7 @@
         <v/>
       </c>
       <c r="S31">
-        <f>IF(OR(B31="",COUNTIF($B$6:$B31,B31)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B31,$B$6:$B$305)=1)*($R$6:$R$305&gt;R31)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B31="",COUNTIF($B$6:$B31,B31)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R31)+(($R$6:$R$305=R31)*(ROW($B$6:$B$305)&lt;ROW(B31)))))+1)</f>
         <v/>
       </c>
       <c r="T31">
@@ -17318,7 +17308,7 @@
         <v/>
       </c>
       <c r="S32">
-        <f>IF(OR(B32="",COUNTIF($B$6:$B32,B32)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B32,$B$6:$B$305)=1)*($R$6:$R$305&gt;R32)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B32="",COUNTIF($B$6:$B32,B32)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R32)+(($R$6:$R$305=R32)*(ROW($B$6:$B$305)&lt;ROW(B32)))))+1)</f>
         <v/>
       </c>
       <c r="T32">
@@ -17386,7 +17376,7 @@
         <v/>
       </c>
       <c r="S33">
-        <f>IF(OR(B33="",COUNTIF($B$6:$B33,B33)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B33,$B$6:$B$305)=1)*($R$6:$R$305&gt;R33)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B33="",COUNTIF($B$6:$B33,B33)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R33)+(($R$6:$R$305=R33)*(ROW($B$6:$B$305)&lt;ROW(B33)))))+1)</f>
         <v/>
       </c>
       <c r="T33">
@@ -17454,7 +17444,7 @@
         <v/>
       </c>
       <c r="S34">
-        <f>IF(OR(B34="",COUNTIF($B$6:$B34,B34)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B34,$B$6:$B$305)=1)*($R$6:$R$305&gt;R34)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B34="",COUNTIF($B$6:$B34,B34)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R34)+(($R$6:$R$305=R34)*(ROW($B$6:$B$305)&lt;ROW(B34)))))+1)</f>
         <v/>
       </c>
       <c r="T34">
@@ -17522,7 +17512,7 @@
         <v/>
       </c>
       <c r="S35">
-        <f>IF(OR(B35="",COUNTIF($B$6:$B35,B35)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B35,$B$6:$B$305)=1)*($R$6:$R$305&gt;R35)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B35="",COUNTIF($B$6:$B35,B35)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R35)+(($R$6:$R$305=R35)*(ROW($B$6:$B$305)&lt;ROW(B35)))))+1)</f>
         <v/>
       </c>
       <c r="T35">
@@ -17575,7 +17565,7 @@
         <v/>
       </c>
       <c r="S36">
-        <f>IF(OR(B36="",COUNTIF($B$6:$B36,B36)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B36,$B$6:$B$305)=1)*($R$6:$R$305&gt;R36)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B36="",COUNTIF($B$6:$B36,B36)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R36)+(($R$6:$R$305=R36)*(ROW($B$6:$B$305)&lt;ROW(B36)))))+1)</f>
         <v/>
       </c>
       <c r="T36">
@@ -17628,7 +17618,7 @@
         <v/>
       </c>
       <c r="S37">
-        <f>IF(OR(B37="",COUNTIF($B$6:$B37,B37)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B37,$B$6:$B$305)=1)*($R$6:$R$305&gt;R37)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B37="",COUNTIF($B$6:$B37,B37)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R37)+(($R$6:$R$305=R37)*(ROW($B$6:$B$305)&lt;ROW(B37)))))+1)</f>
         <v/>
       </c>
       <c r="T37">
@@ -17681,7 +17671,7 @@
         <v/>
       </c>
       <c r="S38">
-        <f>IF(OR(B38="",COUNTIF($B$6:$B38,B38)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B38,$B$6:$B$305)=1)*($R$6:$R$305&gt;R38)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B38="",COUNTIF($B$6:$B38,B38)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R38)+(($R$6:$R$305=R38)*(ROW($B$6:$B$305)&lt;ROW(B38)))))+1)</f>
         <v/>
       </c>
       <c r="T38">
@@ -17734,7 +17724,7 @@
         <v/>
       </c>
       <c r="S39">
-        <f>IF(OR(B39="",COUNTIF($B$6:$B39,B39)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B39,$B$6:$B$305)=1)*($R$6:$R$305&gt;R39)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B39="",COUNTIF($B$6:$B39,B39)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R39)+(($R$6:$R$305=R39)*(ROW($B$6:$B$305)&lt;ROW(B39)))))+1)</f>
         <v/>
       </c>
       <c r="T39">
@@ -17787,7 +17777,7 @@
         <v/>
       </c>
       <c r="S40">
-        <f>IF(OR(B40="",COUNTIF($B$6:$B40,B40)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B40,$B$6:$B$305)=1)*($R$6:$R$305&gt;R40)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B40="",COUNTIF($B$6:$B40,B40)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R40)+(($R$6:$R$305=R40)*(ROW($B$6:$B$305)&lt;ROW(B40)))))+1)</f>
         <v/>
       </c>
       <c r="T40">
@@ -17840,7 +17830,7 @@
         <v/>
       </c>
       <c r="S41">
-        <f>IF(OR(B41="",COUNTIF($B$6:$B41,B41)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B41,$B$6:$B$305)=1)*($R$6:$R$305&gt;R41)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B41="",COUNTIF($B$6:$B41,B41)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R41)+(($R$6:$R$305=R41)*(ROW($B$6:$B$305)&lt;ROW(B41)))))+1)</f>
         <v/>
       </c>
       <c r="T41">
@@ -17893,7 +17883,7 @@
         <v/>
       </c>
       <c r="S42">
-        <f>IF(OR(B42="",COUNTIF($B$6:$B42,B42)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B42,$B$6:$B$305)=1)*($R$6:$R$305&gt;R42)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B42="",COUNTIF($B$6:$B42,B42)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R42)+(($R$6:$R$305=R42)*(ROW($B$6:$B$305)&lt;ROW(B42)))))+1)</f>
         <v/>
       </c>
       <c r="T42">
@@ -17946,7 +17936,7 @@
         <v/>
       </c>
       <c r="S43">
-        <f>IF(OR(B43="",COUNTIF($B$6:$B43,B43)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B43,$B$6:$B$305)=1)*($R$6:$R$305&gt;R43)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B43="",COUNTIF($B$6:$B43,B43)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R43)+(($R$6:$R$305=R43)*(ROW($B$6:$B$305)&lt;ROW(B43)))))+1)</f>
         <v/>
       </c>
       <c r="T43">
@@ -17999,7 +17989,7 @@
         <v/>
       </c>
       <c r="S44">
-        <f>IF(OR(B44="",COUNTIF($B$6:$B44,B44)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B44,$B$6:$B$305)=1)*($R$6:$R$305&gt;R44)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B44="",COUNTIF($B$6:$B44,B44)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R44)+(($R$6:$R$305=R44)*(ROW($B$6:$B$305)&lt;ROW(B44)))))+1)</f>
         <v/>
       </c>
       <c r="T44">
@@ -18052,7 +18042,7 @@
         <v/>
       </c>
       <c r="S45">
-        <f>IF(OR(B45="",COUNTIF($B$6:$B45,B45)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B45,$B$6:$B$305)=1)*($R$6:$R$305&gt;R45)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B45="",COUNTIF($B$6:$B45,B45)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R45)+(($R$6:$R$305=R45)*(ROW($B$6:$B$305)&lt;ROW(B45)))))+1)</f>
         <v/>
       </c>
       <c r="T45">
@@ -18105,7 +18095,7 @@
         <v/>
       </c>
       <c r="S46">
-        <f>IF(OR(B46="",COUNTIF($B$6:$B46,B46)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B46,$B$6:$B$305)=1)*($R$6:$R$305&gt;R46)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B46="",COUNTIF($B$6:$B46,B46)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R46)+(($R$6:$R$305=R46)*(ROW($B$6:$B$305)&lt;ROW(B46)))))+1)</f>
         <v/>
       </c>
       <c r="T46">
@@ -18158,7 +18148,7 @@
         <v/>
       </c>
       <c r="S47">
-        <f>IF(OR(B47="",COUNTIF($B$6:$B47,B47)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B47,$B$6:$B$305)=1)*($R$6:$R$305&gt;R47)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B47="",COUNTIF($B$6:$B47,B47)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R47)+(($R$6:$R$305=R47)*(ROW($B$6:$B$305)&lt;ROW(B47)))))+1)</f>
         <v/>
       </c>
       <c r="T47">
@@ -18211,7 +18201,7 @@
         <v/>
       </c>
       <c r="S48">
-        <f>IF(OR(B48="",COUNTIF($B$6:$B48,B48)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B48,$B$6:$B$305)=1)*($R$6:$R$305&gt;R48)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B48="",COUNTIF($B$6:$B48,B48)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R48)+(($R$6:$R$305=R48)*(ROW($B$6:$B$305)&lt;ROW(B48)))))+1)</f>
         <v/>
       </c>
       <c r="T48">
@@ -18264,7 +18254,7 @@
         <v/>
       </c>
       <c r="S49">
-        <f>IF(OR(B49="",COUNTIF($B$6:$B49,B49)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B49,$B$6:$B$305)=1)*($R$6:$R$305&gt;R49)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B49="",COUNTIF($B$6:$B49,B49)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R49)+(($R$6:$R$305=R49)*(ROW($B$6:$B$305)&lt;ROW(B49)))))+1)</f>
         <v/>
       </c>
       <c r="T49">
@@ -18317,7 +18307,7 @@
         <v/>
       </c>
       <c r="S50">
-        <f>IF(OR(B50="",COUNTIF($B$6:$B50,B50)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B50,$B$6:$B$305)=1)*($R$6:$R$305&gt;R50)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B50="",COUNTIF($B$6:$B50,B50)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R50)+(($R$6:$R$305=R50)*(ROW($B$6:$B$305)&lt;ROW(B50)))))+1)</f>
         <v/>
       </c>
       <c r="T50">
@@ -18370,7 +18360,7 @@
         <v/>
       </c>
       <c r="S51">
-        <f>IF(OR(B51="",COUNTIF($B$6:$B51,B51)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B51,$B$6:$B$305)=1)*($R$6:$R$305&gt;R51)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B51="",COUNTIF($B$6:$B51,B51)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R51)+(($R$6:$R$305=R51)*(ROW($B$6:$B$305)&lt;ROW(B51)))))+1)</f>
         <v/>
       </c>
       <c r="T51">
@@ -18423,7 +18413,7 @@
         <v/>
       </c>
       <c r="S52">
-        <f>IF(OR(B52="",COUNTIF($B$6:$B52,B52)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B52,$B$6:$B$305)=1)*($R$6:$R$305&gt;R52)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B52="",COUNTIF($B$6:$B52,B52)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R52)+(($R$6:$R$305=R52)*(ROW($B$6:$B$305)&lt;ROW(B52)))))+1)</f>
         <v/>
       </c>
       <c r="T52">
@@ -18476,7 +18466,7 @@
         <v/>
       </c>
       <c r="S53">
-        <f>IF(OR(B53="",COUNTIF($B$6:$B53,B53)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B53,$B$6:$B$305)=1)*($R$6:$R$305&gt;R53)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B53="",COUNTIF($B$6:$B53,B53)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R53)+(($R$6:$R$305=R53)*(ROW($B$6:$B$305)&lt;ROW(B53)))))+1)</f>
         <v/>
       </c>
       <c r="T53">
@@ -18529,7 +18519,7 @@
         <v/>
       </c>
       <c r="S54">
-        <f>IF(OR(B54="",COUNTIF($B$6:$B54,B54)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B54,$B$6:$B$305)=1)*($R$6:$R$305&gt;R54)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B54="",COUNTIF($B$6:$B54,B54)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R54)+(($R$6:$R$305=R54)*(ROW($B$6:$B$305)&lt;ROW(B54)))))+1)</f>
         <v/>
       </c>
       <c r="T54">
@@ -18582,7 +18572,7 @@
         <v/>
       </c>
       <c r="S55">
-        <f>IF(OR(B55="",COUNTIF($B$6:$B55,B55)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B55,$B$6:$B$305)=1)*($R$6:$R$305&gt;R55)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B55="",COUNTIF($B$6:$B55,B55)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R55)+(($R$6:$R$305=R55)*(ROW($B$6:$B$305)&lt;ROW(B55)))))+1)</f>
         <v/>
       </c>
       <c r="T55">
@@ -18620,7 +18610,7 @@
         <v/>
       </c>
       <c r="S56">
-        <f>IF(OR(B56="",COUNTIF($B$6:$B56,B56)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B56,$B$6:$B$305)=1)*($R$6:$R$305&gt;R56)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B56="",COUNTIF($B$6:$B56,B56)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R56)+(($R$6:$R$305=R56)*(ROW($B$6:$B$305)&lt;ROW(B56)))))+1)</f>
         <v/>
       </c>
       <c r="T56">
@@ -18658,7 +18648,7 @@
         <v/>
       </c>
       <c r="S57">
-        <f>IF(OR(B57="",COUNTIF($B$6:$B57,B57)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B57,$B$6:$B$305)=1)*($R$6:$R$305&gt;R57)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B57="",COUNTIF($B$6:$B57,B57)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R57)+(($R$6:$R$305=R57)*(ROW($B$6:$B$305)&lt;ROW(B57)))))+1)</f>
         <v/>
       </c>
       <c r="T57">
@@ -18696,7 +18686,7 @@
         <v/>
       </c>
       <c r="S58">
-        <f>IF(OR(B58="",COUNTIF($B$6:$B58,B58)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B58,$B$6:$B$305)=1)*($R$6:$R$305&gt;R58)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B58="",COUNTIF($B$6:$B58,B58)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R58)+(($R$6:$R$305=R58)*(ROW($B$6:$B$305)&lt;ROW(B58)))))+1)</f>
         <v/>
       </c>
       <c r="T58">
@@ -18734,7 +18724,7 @@
         <v/>
       </c>
       <c r="S59">
-        <f>IF(OR(B59="",COUNTIF($B$6:$B59,B59)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B59,$B$6:$B$305)=1)*($R$6:$R$305&gt;R59)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B59="",COUNTIF($B$6:$B59,B59)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R59)+(($R$6:$R$305=R59)*(ROW($B$6:$B$305)&lt;ROW(B59)))))+1)</f>
         <v/>
       </c>
       <c r="T59">
@@ -18772,7 +18762,7 @@
         <v/>
       </c>
       <c r="S60">
-        <f>IF(OR(B60="",COUNTIF($B$6:$B60,B60)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B60,$B$6:$B$305)=1)*($R$6:$R$305&gt;R60)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B60="",COUNTIF($B$6:$B60,B60)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R60)+(($R$6:$R$305=R60)*(ROW($B$6:$B$305)&lt;ROW(B60)))))+1)</f>
         <v/>
       </c>
       <c r="T60">
@@ -18810,7 +18800,7 @@
         <v/>
       </c>
       <c r="S61">
-        <f>IF(OR(B61="",COUNTIF($B$6:$B61,B61)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B61,$B$6:$B$305)=1)*($R$6:$R$305&gt;R61)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B61="",COUNTIF($B$6:$B61,B61)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R61)+(($R$6:$R$305=R61)*(ROW($B$6:$B$305)&lt;ROW(B61)))))+1)</f>
         <v/>
       </c>
       <c r="T61">
@@ -18848,7 +18838,7 @@
         <v/>
       </c>
       <c r="S62">
-        <f>IF(OR(B62="",COUNTIF($B$6:$B62,B62)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B62,$B$6:$B$305)=1)*($R$6:$R$305&gt;R62)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B62="",COUNTIF($B$6:$B62,B62)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R62)+(($R$6:$R$305=R62)*(ROW($B$6:$B$305)&lt;ROW(B62)))))+1)</f>
         <v/>
       </c>
       <c r="T62">
@@ -18886,7 +18876,7 @@
         <v/>
       </c>
       <c r="S63">
-        <f>IF(OR(B63="",COUNTIF($B$6:$B63,B63)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B63,$B$6:$B$305)=1)*($R$6:$R$305&gt;R63)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B63="",COUNTIF($B$6:$B63,B63)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R63)+(($R$6:$R$305=R63)*(ROW($B$6:$B$305)&lt;ROW(B63)))))+1)</f>
         <v/>
       </c>
       <c r="T63">
@@ -18924,7 +18914,7 @@
         <v/>
       </c>
       <c r="S64">
-        <f>IF(OR(B64="",COUNTIF($B$6:$B64,B64)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B64,$B$6:$B$305)=1)*($R$6:$R$305&gt;R64)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B64="",COUNTIF($B$6:$B64,B64)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R64)+(($R$6:$R$305=R64)*(ROW($B$6:$B$305)&lt;ROW(B64)))))+1)</f>
         <v/>
       </c>
       <c r="T64">
@@ -18962,7 +18952,7 @@
         <v/>
       </c>
       <c r="S65">
-        <f>IF(OR(B65="",COUNTIF($B$6:$B65,B65)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B65,$B$6:$B$305)=1)*($R$6:$R$305&gt;R65)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B65="",COUNTIF($B$6:$B65,B65)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R65)+(($R$6:$R$305=R65)*(ROW($B$6:$B$305)&lt;ROW(B65)))))+1)</f>
         <v/>
       </c>
       <c r="T65">
@@ -19000,7 +18990,7 @@
         <v/>
       </c>
       <c r="S66">
-        <f>IF(OR(B66="",COUNTIF($B$6:$B66,B66)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B66,$B$6:$B$305)=1)*($R$6:$R$305&gt;R66)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B66="",COUNTIF($B$6:$B66,B66)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R66)+(($R$6:$R$305=R66)*(ROW($B$6:$B$305)&lt;ROW(B66)))))+1)</f>
         <v/>
       </c>
       <c r="T66">
@@ -19038,7 +19028,7 @@
         <v/>
       </c>
       <c r="S67">
-        <f>IF(OR(B67="",COUNTIF($B$6:$B67,B67)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B67,$B$6:$B$305)=1)*($R$6:$R$305&gt;R67)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B67="",COUNTIF($B$6:$B67,B67)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R67)+(($R$6:$R$305=R67)*(ROW($B$6:$B$305)&lt;ROW(B67)))))+1)</f>
         <v/>
       </c>
       <c r="T67">
@@ -19076,7 +19066,7 @@
         <v/>
       </c>
       <c r="S68">
-        <f>IF(OR(B68="",COUNTIF($B$6:$B68,B68)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B68,$B$6:$B$305)=1)*($R$6:$R$305&gt;R68)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B68="",COUNTIF($B$6:$B68,B68)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R68)+(($R$6:$R$305=R68)*(ROW($B$6:$B$305)&lt;ROW(B68)))))+1)</f>
         <v/>
       </c>
       <c r="T68">
@@ -19114,7 +19104,7 @@
         <v/>
       </c>
       <c r="S69">
-        <f>IF(OR(B69="",COUNTIF($B$6:$B69,B69)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B69,$B$6:$B$305)=1)*($R$6:$R$305&gt;R69)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B69="",COUNTIF($B$6:$B69,B69)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R69)+(($R$6:$R$305=R69)*(ROW($B$6:$B$305)&lt;ROW(B69)))))+1)</f>
         <v/>
       </c>
       <c r="T69">
@@ -19152,7 +19142,7 @@
         <v/>
       </c>
       <c r="S70">
-        <f>IF(OR(B70="",COUNTIF($B$6:$B70,B70)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B70,$B$6:$B$305)=1)*($R$6:$R$305&gt;R70)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B70="",COUNTIF($B$6:$B70,B70)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R70)+(($R$6:$R$305=R70)*(ROW($B$6:$B$305)&lt;ROW(B70)))))+1)</f>
         <v/>
       </c>
       <c r="T70">
@@ -19190,7 +19180,7 @@
         <v/>
       </c>
       <c r="S71">
-        <f>IF(OR(B71="",COUNTIF($B$6:$B71,B71)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B71,$B$6:$B$305)=1)*($R$6:$R$305&gt;R71)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B71="",COUNTIF($B$6:$B71,B71)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R71)+(($R$6:$R$305=R71)*(ROW($B$6:$B$305)&lt;ROW(B71)))))+1)</f>
         <v/>
       </c>
       <c r="T71">
@@ -19228,7 +19218,7 @@
         <v/>
       </c>
       <c r="S72">
-        <f>IF(OR(B72="",COUNTIF($B$6:$B72,B72)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B72,$B$6:$B$305)=1)*($R$6:$R$305&gt;R72)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B72="",COUNTIF($B$6:$B72,B72)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R72)+(($R$6:$R$305=R72)*(ROW($B$6:$B$305)&lt;ROW(B72)))))+1)</f>
         <v/>
       </c>
       <c r="T72">
@@ -19266,7 +19256,7 @@
         <v/>
       </c>
       <c r="S73">
-        <f>IF(OR(B73="",COUNTIF($B$6:$B73,B73)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B73,$B$6:$B$305)=1)*($R$6:$R$305&gt;R73)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B73="",COUNTIF($B$6:$B73,B73)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R73)+(($R$6:$R$305=R73)*(ROW($B$6:$B$305)&lt;ROW(B73)))))+1)</f>
         <v/>
       </c>
       <c r="T73">
@@ -19304,7 +19294,7 @@
         <v/>
       </c>
       <c r="S74">
-        <f>IF(OR(B74="",COUNTIF($B$6:$B74,B74)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B74,$B$6:$B$305)=1)*($R$6:$R$305&gt;R74)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B74="",COUNTIF($B$6:$B74,B74)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R74)+(($R$6:$R$305=R74)*(ROW($B$6:$B$305)&lt;ROW(B74)))))+1)</f>
         <v/>
       </c>
       <c r="T74">
@@ -19342,7 +19332,7 @@
         <v/>
       </c>
       <c r="S75">
-        <f>IF(OR(B75="",COUNTIF($B$6:$B75,B75)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B75,$B$6:$B$305)=1)*($R$6:$R$305&gt;R75)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B75="",COUNTIF($B$6:$B75,B75)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R75)+(($R$6:$R$305=R75)*(ROW($B$6:$B$305)&lt;ROW(B75)))))+1)</f>
         <v/>
       </c>
       <c r="T75">
@@ -19380,7 +19370,7 @@
         <v/>
       </c>
       <c r="S76">
-        <f>IF(OR(B76="",COUNTIF($B$6:$B76,B76)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B76,$B$6:$B$305)=1)*($R$6:$R$305&gt;R76)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B76="",COUNTIF($B$6:$B76,B76)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R76)+(($R$6:$R$305=R76)*(ROW($B$6:$B$305)&lt;ROW(B76)))))+1)</f>
         <v/>
       </c>
       <c r="T76">
@@ -19418,7 +19408,7 @@
         <v/>
       </c>
       <c r="S77">
-        <f>IF(OR(B77="",COUNTIF($B$6:$B77,B77)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B77,$B$6:$B$305)=1)*($R$6:$R$305&gt;R77)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B77="",COUNTIF($B$6:$B77,B77)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R77)+(($R$6:$R$305=R77)*(ROW($B$6:$B$305)&lt;ROW(B77)))))+1)</f>
         <v/>
       </c>
       <c r="T77">
@@ -19456,7 +19446,7 @@
         <v/>
       </c>
       <c r="S78">
-        <f>IF(OR(B78="",COUNTIF($B$6:$B78,B78)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B78,$B$6:$B$305)=1)*($R$6:$R$305&gt;R78)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B78="",COUNTIF($B$6:$B78,B78)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R78)+(($R$6:$R$305=R78)*(ROW($B$6:$B$305)&lt;ROW(B78)))))+1)</f>
         <v/>
       </c>
       <c r="T78">
@@ -19494,7 +19484,7 @@
         <v/>
       </c>
       <c r="S79">
-        <f>IF(OR(B79="",COUNTIF($B$6:$B79,B79)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B79,$B$6:$B$305)=1)*($R$6:$R$305&gt;R79)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B79="",COUNTIF($B$6:$B79,B79)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R79)+(($R$6:$R$305=R79)*(ROW($B$6:$B$305)&lt;ROW(B79)))))+1)</f>
         <v/>
       </c>
       <c r="T79">
@@ -19532,7 +19522,7 @@
         <v/>
       </c>
       <c r="S80">
-        <f>IF(OR(B80="",COUNTIF($B$6:$B80,B80)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B80,$B$6:$B$305)=1)*($R$6:$R$305&gt;R80)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B80="",COUNTIF($B$6:$B80,B80)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R80)+(($R$6:$R$305=R80)*(ROW($B$6:$B$305)&lt;ROW(B80)))))+1)</f>
         <v/>
       </c>
       <c r="T80">
@@ -19570,7 +19560,7 @@
         <v/>
       </c>
       <c r="S81">
-        <f>IF(OR(B81="",COUNTIF($B$6:$B81,B81)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B81,$B$6:$B$305)=1)*($R$6:$R$305&gt;R81)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B81="",COUNTIF($B$6:$B81,B81)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R81)+(($R$6:$R$305=R81)*(ROW($B$6:$B$305)&lt;ROW(B81)))))+1)</f>
         <v/>
       </c>
       <c r="T81">
@@ -19608,7 +19598,7 @@
         <v/>
       </c>
       <c r="S82">
-        <f>IF(OR(B82="",COUNTIF($B$6:$B82,B82)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B82,$B$6:$B$305)=1)*($R$6:$R$305&gt;R82)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B82="",COUNTIF($B$6:$B82,B82)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R82)+(($R$6:$R$305=R82)*(ROW($B$6:$B$305)&lt;ROW(B82)))))+1)</f>
         <v/>
       </c>
       <c r="T82">
@@ -19646,7 +19636,7 @@
         <v/>
       </c>
       <c r="S83">
-        <f>IF(OR(B83="",COUNTIF($B$6:$B83,B83)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B83,$B$6:$B$305)=1)*($R$6:$R$305&gt;R83)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B83="",COUNTIF($B$6:$B83,B83)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R83)+(($R$6:$R$305=R83)*(ROW($B$6:$B$305)&lt;ROW(B83)))))+1)</f>
         <v/>
       </c>
       <c r="T83">
@@ -19684,7 +19674,7 @@
         <v/>
       </c>
       <c r="S84">
-        <f>IF(OR(B84="",COUNTIF($B$6:$B84,B84)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B84,$B$6:$B$305)=1)*($R$6:$R$305&gt;R84)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B84="",COUNTIF($B$6:$B84,B84)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R84)+(($R$6:$R$305=R84)*(ROW($B$6:$B$305)&lt;ROW(B84)))))+1)</f>
         <v/>
       </c>
       <c r="T84">
@@ -19722,7 +19712,7 @@
         <v/>
       </c>
       <c r="S85">
-        <f>IF(OR(B85="",COUNTIF($B$6:$B85,B85)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B85,$B$6:$B$305)=1)*($R$6:$R$305&gt;R85)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B85="",COUNTIF($B$6:$B85,B85)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R85)+(($R$6:$R$305=R85)*(ROW($B$6:$B$305)&lt;ROW(B85)))))+1)</f>
         <v/>
       </c>
       <c r="T85">
@@ -19760,7 +19750,7 @@
         <v/>
       </c>
       <c r="S86">
-        <f>IF(OR(B86="",COUNTIF($B$6:$B86,B86)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B86,$B$6:$B$305)=1)*($R$6:$R$305&gt;R86)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B86="",COUNTIF($B$6:$B86,B86)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R86)+(($R$6:$R$305=R86)*(ROW($B$6:$B$305)&lt;ROW(B86)))))+1)</f>
         <v/>
       </c>
       <c r="T86">
@@ -19798,7 +19788,7 @@
         <v/>
       </c>
       <c r="S87">
-        <f>IF(OR(B87="",COUNTIF($B$6:$B87,B87)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B87,$B$6:$B$305)=1)*($R$6:$R$305&gt;R87)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B87="",COUNTIF($B$6:$B87,B87)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R87)+(($R$6:$R$305=R87)*(ROW($B$6:$B$305)&lt;ROW(B87)))))+1)</f>
         <v/>
       </c>
       <c r="T87">
@@ -19836,7 +19826,7 @@
         <v/>
       </c>
       <c r="S88">
-        <f>IF(OR(B88="",COUNTIF($B$6:$B88,B88)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B88,$B$6:$B$305)=1)*($R$6:$R$305&gt;R88)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B88="",COUNTIF($B$6:$B88,B88)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R88)+(($R$6:$R$305=R88)*(ROW($B$6:$B$305)&lt;ROW(B88)))))+1)</f>
         <v/>
       </c>
       <c r="T88">
@@ -19874,7 +19864,7 @@
         <v/>
       </c>
       <c r="S89">
-        <f>IF(OR(B89="",COUNTIF($B$6:$B89,B89)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B89,$B$6:$B$305)=1)*($R$6:$R$305&gt;R89)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B89="",COUNTIF($B$6:$B89,B89)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R89)+(($R$6:$R$305=R89)*(ROW($B$6:$B$305)&lt;ROW(B89)))))+1)</f>
         <v/>
       </c>
       <c r="T89">
@@ -19912,7 +19902,7 @@
         <v/>
       </c>
       <c r="S90">
-        <f>IF(OR(B90="",COUNTIF($B$6:$B90,B90)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B90,$B$6:$B$305)=1)*($R$6:$R$305&gt;R90)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B90="",COUNTIF($B$6:$B90,B90)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R90)+(($R$6:$R$305=R90)*(ROW($B$6:$B$305)&lt;ROW(B90)))))+1)</f>
         <v/>
       </c>
       <c r="T90">
@@ -19950,7 +19940,7 @@
         <v/>
       </c>
       <c r="S91">
-        <f>IF(OR(B91="",COUNTIF($B$6:$B91,B91)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B91,$B$6:$B$305)=1)*($R$6:$R$305&gt;R91)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B91="",COUNTIF($B$6:$B91,B91)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R91)+(($R$6:$R$305=R91)*(ROW($B$6:$B$305)&lt;ROW(B91)))))+1)</f>
         <v/>
       </c>
       <c r="T91">
@@ -19988,7 +19978,7 @@
         <v/>
       </c>
       <c r="S92">
-        <f>IF(OR(B92="",COUNTIF($B$6:$B92,B92)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B92,$B$6:$B$305)=1)*($R$6:$R$305&gt;R92)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B92="",COUNTIF($B$6:$B92,B92)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R92)+(($R$6:$R$305=R92)*(ROW($B$6:$B$305)&lt;ROW(B92)))))+1)</f>
         <v/>
       </c>
       <c r="T92">
@@ -20026,7 +20016,7 @@
         <v/>
       </c>
       <c r="S93">
-        <f>IF(OR(B93="",COUNTIF($B$6:$B93,B93)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B93,$B$6:$B$305)=1)*($R$6:$R$305&gt;R93)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B93="",COUNTIF($B$6:$B93,B93)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R93)+(($R$6:$R$305=R93)*(ROW($B$6:$B$305)&lt;ROW(B93)))))+1)</f>
         <v/>
       </c>
       <c r="T93">
@@ -20064,7 +20054,7 @@
         <v/>
       </c>
       <c r="S94">
-        <f>IF(OR(B94="",COUNTIF($B$6:$B94,B94)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B94,$B$6:$B$305)=1)*($R$6:$R$305&gt;R94)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B94="",COUNTIF($B$6:$B94,B94)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R94)+(($R$6:$R$305=R94)*(ROW($B$6:$B$305)&lt;ROW(B94)))))+1)</f>
         <v/>
       </c>
       <c r="T94">
@@ -20102,7 +20092,7 @@
         <v/>
       </c>
       <c r="S95">
-        <f>IF(OR(B95="",COUNTIF($B$6:$B95,B95)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B95,$B$6:$B$305)=1)*($R$6:$R$305&gt;R95)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B95="",COUNTIF($B$6:$B95,B95)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R95)+(($R$6:$R$305=R95)*(ROW($B$6:$B$305)&lt;ROW(B95)))))+1)</f>
         <v/>
       </c>
       <c r="T95">
@@ -20140,7 +20130,7 @@
         <v/>
       </c>
       <c r="S96">
-        <f>IF(OR(B96="",COUNTIF($B$6:$B96,B96)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B96,$B$6:$B$305)=1)*($R$6:$R$305&gt;R96)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B96="",COUNTIF($B$6:$B96,B96)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R96)+(($R$6:$R$305=R96)*(ROW($B$6:$B$305)&lt;ROW(B96)))))+1)</f>
         <v/>
       </c>
       <c r="T96">
@@ -20178,7 +20168,7 @@
         <v/>
       </c>
       <c r="S97">
-        <f>IF(OR(B97="",COUNTIF($B$6:$B97,B97)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B97,$B$6:$B$305)=1)*($R$6:$R$305&gt;R97)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B97="",COUNTIF($B$6:$B97,B97)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R97)+(($R$6:$R$305=R97)*(ROW($B$6:$B$305)&lt;ROW(B97)))))+1)</f>
         <v/>
       </c>
       <c r="T97">
@@ -20216,7 +20206,7 @@
         <v/>
       </c>
       <c r="S98">
-        <f>IF(OR(B98="",COUNTIF($B$6:$B98,B98)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B98,$B$6:$B$305)=1)*($R$6:$R$305&gt;R98)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B98="",COUNTIF($B$6:$B98,B98)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R98)+(($R$6:$R$305=R98)*(ROW($B$6:$B$305)&lt;ROW(B98)))))+1)</f>
         <v/>
       </c>
       <c r="T98">
@@ -20254,7 +20244,7 @@
         <v/>
       </c>
       <c r="S99">
-        <f>IF(OR(B99="",COUNTIF($B$6:$B99,B99)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B99,$B$6:$B$305)=1)*($R$6:$R$305&gt;R99)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B99="",COUNTIF($B$6:$B99,B99)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R99)+(($R$6:$R$305=R99)*(ROW($B$6:$B$305)&lt;ROW(B99)))))+1)</f>
         <v/>
       </c>
       <c r="T99">
@@ -20292,7 +20282,7 @@
         <v/>
       </c>
       <c r="S100">
-        <f>IF(OR(B100="",COUNTIF($B$6:$B100,B100)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B100,$B$6:$B$305)=1)*($R$6:$R$305&gt;R100)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B100="",COUNTIF($B$6:$B100,B100)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R100)+(($R$6:$R$305=R100)*(ROW($B$6:$B$305)&lt;ROW(B100)))))+1)</f>
         <v/>
       </c>
       <c r="T100">
@@ -20330,7 +20320,7 @@
         <v/>
       </c>
       <c r="S101">
-        <f>IF(OR(B101="",COUNTIF($B$6:$B101,B101)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B101,$B$6:$B$305)=1)*($R$6:$R$305&gt;R101)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B101="",COUNTIF($B$6:$B101,B101)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R101)+(($R$6:$R$305=R101)*(ROW($B$6:$B$305)&lt;ROW(B101)))))+1)</f>
         <v/>
       </c>
       <c r="T101">
@@ -20368,7 +20358,7 @@
         <v/>
       </c>
       <c r="S102">
-        <f>IF(OR(B102="",COUNTIF($B$6:$B102,B102)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B102,$B$6:$B$305)=1)*($R$6:$R$305&gt;R102)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B102="",COUNTIF($B$6:$B102,B102)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R102)+(($R$6:$R$305=R102)*(ROW($B$6:$B$305)&lt;ROW(B102)))))+1)</f>
         <v/>
       </c>
       <c r="T102">
@@ -20406,7 +20396,7 @@
         <v/>
       </c>
       <c r="S103">
-        <f>IF(OR(B103="",COUNTIF($B$6:$B103,B103)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B103,$B$6:$B$305)=1)*($R$6:$R$305&gt;R103)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B103="",COUNTIF($B$6:$B103,B103)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R103)+(($R$6:$R$305=R103)*(ROW($B$6:$B$305)&lt;ROW(B103)))))+1)</f>
         <v/>
       </c>
       <c r="T103">
@@ -20444,7 +20434,7 @@
         <v/>
       </c>
       <c r="S104">
-        <f>IF(OR(B104="",COUNTIF($B$6:$B104,B104)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B104,$B$6:$B$305)=1)*($R$6:$R$305&gt;R104)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B104="",COUNTIF($B$6:$B104,B104)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R104)+(($R$6:$R$305=R104)*(ROW($B$6:$B$305)&lt;ROW(B104)))))+1)</f>
         <v/>
       </c>
       <c r="T104">
@@ -20482,7 +20472,7 @@
         <v/>
       </c>
       <c r="S105">
-        <f>IF(OR(B105="",COUNTIF($B$6:$B105,B105)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B105,$B$6:$B$305)=1)*($R$6:$R$305&gt;R105)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B105="",COUNTIF($B$6:$B105,B105)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R105)+(($R$6:$R$305=R105)*(ROW($B$6:$B$305)&lt;ROW(B105)))))+1)</f>
         <v/>
       </c>
       <c r="T105">
@@ -20520,7 +20510,7 @@
         <v/>
       </c>
       <c r="S106">
-        <f>IF(OR(B106="",COUNTIF($B$6:$B106,B106)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B106,$B$6:$B$305)=1)*($R$6:$R$305&gt;R106)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B106="",COUNTIF($B$6:$B106,B106)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R106)+(($R$6:$R$305=R106)*(ROW($B$6:$B$305)&lt;ROW(B106)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20542,7 +20532,7 @@
         <v/>
       </c>
       <c r="S107">
-        <f>IF(OR(B107="",COUNTIF($B$6:$B107,B107)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B107,$B$6:$B$305)=1)*($R$6:$R$305&gt;R107)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B107="",COUNTIF($B$6:$B107,B107)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R107)+(($R$6:$R$305=R107)*(ROW($B$6:$B$305)&lt;ROW(B107)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20564,7 +20554,7 @@
         <v/>
       </c>
       <c r="S108">
-        <f>IF(OR(B108="",COUNTIF($B$6:$B108,B108)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B108,$B$6:$B$305)=1)*($R$6:$R$305&gt;R108)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B108="",COUNTIF($B$6:$B108,B108)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R108)+(($R$6:$R$305=R108)*(ROW($B$6:$B$305)&lt;ROW(B108)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20586,7 +20576,7 @@
         <v/>
       </c>
       <c r="S109">
-        <f>IF(OR(B109="",COUNTIF($B$6:$B109,B109)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B109,$B$6:$B$305)=1)*($R$6:$R$305&gt;R109)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B109="",COUNTIF($B$6:$B109,B109)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R109)+(($R$6:$R$305=R109)*(ROW($B$6:$B$305)&lt;ROW(B109)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20608,7 +20598,7 @@
         <v/>
       </c>
       <c r="S110">
-        <f>IF(OR(B110="",COUNTIF($B$6:$B110,B110)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B110,$B$6:$B$305)=1)*($R$6:$R$305&gt;R110)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B110="",COUNTIF($B$6:$B110,B110)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R110)+(($R$6:$R$305=R110)*(ROW($B$6:$B$305)&lt;ROW(B110)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20630,7 +20620,7 @@
         <v/>
       </c>
       <c r="S111">
-        <f>IF(OR(B111="",COUNTIF($B$6:$B111,B111)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B111,$B$6:$B$305)=1)*($R$6:$R$305&gt;R111)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B111="",COUNTIF($B$6:$B111,B111)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R111)+(($R$6:$R$305=R111)*(ROW($B$6:$B$305)&lt;ROW(B111)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20652,7 +20642,7 @@
         <v/>
       </c>
       <c r="S112">
-        <f>IF(OR(B112="",COUNTIF($B$6:$B112,B112)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B112,$B$6:$B$305)=1)*($R$6:$R$305&gt;R112)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B112="",COUNTIF($B$6:$B112,B112)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R112)+(($R$6:$R$305=R112)*(ROW($B$6:$B$305)&lt;ROW(B112)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20674,7 +20664,7 @@
         <v/>
       </c>
       <c r="S113">
-        <f>IF(OR(B113="",COUNTIF($B$6:$B113,B113)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B113,$B$6:$B$305)=1)*($R$6:$R$305&gt;R113)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B113="",COUNTIF($B$6:$B113,B113)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R113)+(($R$6:$R$305=R113)*(ROW($B$6:$B$305)&lt;ROW(B113)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20696,7 +20686,7 @@
         <v/>
       </c>
       <c r="S114">
-        <f>IF(OR(B114="",COUNTIF($B$6:$B114,B114)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B114,$B$6:$B$305)=1)*($R$6:$R$305&gt;R114)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B114="",COUNTIF($B$6:$B114,B114)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R114)+(($R$6:$R$305=R114)*(ROW($B$6:$B$305)&lt;ROW(B114)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20718,7 +20708,7 @@
         <v/>
       </c>
       <c r="S115">
-        <f>IF(OR(B115="",COUNTIF($B$6:$B115,B115)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B115,$B$6:$B$305)=1)*($R$6:$R$305&gt;R115)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B115="",COUNTIF($B$6:$B115,B115)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R115)+(($R$6:$R$305=R115)*(ROW($B$6:$B$305)&lt;ROW(B115)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20740,7 +20730,7 @@
         <v/>
       </c>
       <c r="S116">
-        <f>IF(OR(B116="",COUNTIF($B$6:$B116,B116)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B116,$B$6:$B$305)=1)*($R$6:$R$305&gt;R116)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B116="",COUNTIF($B$6:$B116,B116)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R116)+(($R$6:$R$305=R116)*(ROW($B$6:$B$305)&lt;ROW(B116)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20762,7 +20752,7 @@
         <v/>
       </c>
       <c r="S117">
-        <f>IF(OR(B117="",COUNTIF($B$6:$B117,B117)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B117,$B$6:$B$305)=1)*($R$6:$R$305&gt;R117)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B117="",COUNTIF($B$6:$B117,B117)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R117)+(($R$6:$R$305=R117)*(ROW($B$6:$B$305)&lt;ROW(B117)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20784,7 +20774,7 @@
         <v/>
       </c>
       <c r="S118">
-        <f>IF(OR(B118="",COUNTIF($B$6:$B118,B118)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B118,$B$6:$B$305)=1)*($R$6:$R$305&gt;R118)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B118="",COUNTIF($B$6:$B118,B118)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R118)+(($R$6:$R$305=R118)*(ROW($B$6:$B$305)&lt;ROW(B118)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20806,7 +20796,7 @@
         <v/>
       </c>
       <c r="S119">
-        <f>IF(OR(B119="",COUNTIF($B$6:$B119,B119)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B119,$B$6:$B$305)=1)*($R$6:$R$305&gt;R119)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B119="",COUNTIF($B$6:$B119,B119)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R119)+(($R$6:$R$305=R119)*(ROW($B$6:$B$305)&lt;ROW(B119)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20828,7 +20818,7 @@
         <v/>
       </c>
       <c r="S120">
-        <f>IF(OR(B120="",COUNTIF($B$6:$B120,B120)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B120,$B$6:$B$305)=1)*($R$6:$R$305&gt;R120)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B120="",COUNTIF($B$6:$B120,B120)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R120)+(($R$6:$R$305=R120)*(ROW($B$6:$B$305)&lt;ROW(B120)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20850,7 +20840,7 @@
         <v/>
       </c>
       <c r="S121">
-        <f>IF(OR(B121="",COUNTIF($B$6:$B121,B121)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B121,$B$6:$B$305)=1)*($R$6:$R$305&gt;R121)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B121="",COUNTIF($B$6:$B121,B121)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R121)+(($R$6:$R$305=R121)*(ROW($B$6:$B$305)&lt;ROW(B121)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20872,7 +20862,7 @@
         <v/>
       </c>
       <c r="S122">
-        <f>IF(OR(B122="",COUNTIF($B$6:$B122,B122)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B122,$B$6:$B$305)=1)*($R$6:$R$305&gt;R122)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B122="",COUNTIF($B$6:$B122,B122)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R122)+(($R$6:$R$305=R122)*(ROW($B$6:$B$305)&lt;ROW(B122)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20894,7 +20884,7 @@
         <v/>
       </c>
       <c r="S123">
-        <f>IF(OR(B123="",COUNTIF($B$6:$B123,B123)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B123,$B$6:$B$305)=1)*($R$6:$R$305&gt;R123)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B123="",COUNTIF($B$6:$B123,B123)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R123)+(($R$6:$R$305=R123)*(ROW($B$6:$B$305)&lt;ROW(B123)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20916,7 +20906,7 @@
         <v/>
       </c>
       <c r="S124">
-        <f>IF(OR(B124="",COUNTIF($B$6:$B124,B124)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B124,$B$6:$B$305)=1)*($R$6:$R$305&gt;R124)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B124="",COUNTIF($B$6:$B124,B124)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R124)+(($R$6:$R$305=R124)*(ROW($B$6:$B$305)&lt;ROW(B124)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20938,7 +20928,7 @@
         <v/>
       </c>
       <c r="S125">
-        <f>IF(OR(B125="",COUNTIF($B$6:$B125,B125)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B125,$B$6:$B$305)=1)*($R$6:$R$305&gt;R125)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B125="",COUNTIF($B$6:$B125,B125)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R125)+(($R$6:$R$305=R125)*(ROW($B$6:$B$305)&lt;ROW(B125)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20960,7 +20950,7 @@
         <v/>
       </c>
       <c r="S126">
-        <f>IF(OR(B126="",COUNTIF($B$6:$B126,B126)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B126,$B$6:$B$305)=1)*($R$6:$R$305&gt;R126)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B126="",COUNTIF($B$6:$B126,B126)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R126)+(($R$6:$R$305=R126)*(ROW($B$6:$B$305)&lt;ROW(B126)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -20982,7 +20972,7 @@
         <v/>
       </c>
       <c r="S127">
-        <f>IF(OR(B127="",COUNTIF($B$6:$B127,B127)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B127,$B$6:$B$305)=1)*($R$6:$R$305&gt;R127)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B127="",COUNTIF($B$6:$B127,B127)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R127)+(($R$6:$R$305=R127)*(ROW($B$6:$B$305)&lt;ROW(B127)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21004,7 +20994,7 @@
         <v/>
       </c>
       <c r="S128">
-        <f>IF(OR(B128="",COUNTIF($B$6:$B128,B128)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B128,$B$6:$B$305)=1)*($R$6:$R$305&gt;R128)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B128="",COUNTIF($B$6:$B128,B128)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R128)+(($R$6:$R$305=R128)*(ROW($B$6:$B$305)&lt;ROW(B128)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21026,7 +21016,7 @@
         <v/>
       </c>
       <c r="S129">
-        <f>IF(OR(B129="",COUNTIF($B$6:$B129,B129)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B129,$B$6:$B$305)=1)*($R$6:$R$305&gt;R129)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B129="",COUNTIF($B$6:$B129,B129)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R129)+(($R$6:$R$305=R129)*(ROW($B$6:$B$305)&lt;ROW(B129)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21048,7 +21038,7 @@
         <v/>
       </c>
       <c r="S130">
-        <f>IF(OR(B130="",COUNTIF($B$6:$B130,B130)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B130,$B$6:$B$305)=1)*($R$6:$R$305&gt;R130)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B130="",COUNTIF($B$6:$B130,B130)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R130)+(($R$6:$R$305=R130)*(ROW($B$6:$B$305)&lt;ROW(B130)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21070,7 +21060,7 @@
         <v/>
       </c>
       <c r="S131">
-        <f>IF(OR(B131="",COUNTIF($B$6:$B131,B131)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B131,$B$6:$B$305)=1)*($R$6:$R$305&gt;R131)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B131="",COUNTIF($B$6:$B131,B131)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R131)+(($R$6:$R$305=R131)*(ROW($B$6:$B$305)&lt;ROW(B131)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21092,7 +21082,7 @@
         <v/>
       </c>
       <c r="S132">
-        <f>IF(OR(B132="",COUNTIF($B$6:$B132,B132)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B132,$B$6:$B$305)=1)*($R$6:$R$305&gt;R132)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B132="",COUNTIF($B$6:$B132,B132)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R132)+(($R$6:$R$305=R132)*(ROW($B$6:$B$305)&lt;ROW(B132)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21114,7 +21104,7 @@
         <v/>
       </c>
       <c r="S133">
-        <f>IF(OR(B133="",COUNTIF($B$6:$B133,B133)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B133,$B$6:$B$305)=1)*($R$6:$R$305&gt;R133)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B133="",COUNTIF($B$6:$B133,B133)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R133)+(($R$6:$R$305=R133)*(ROW($B$6:$B$305)&lt;ROW(B133)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21136,7 +21126,7 @@
         <v/>
       </c>
       <c r="S134">
-        <f>IF(OR(B134="",COUNTIF($B$6:$B134,B134)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B134,$B$6:$B$305)=1)*($R$6:$R$305&gt;R134)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B134="",COUNTIF($B$6:$B134,B134)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R134)+(($R$6:$R$305=R134)*(ROW($B$6:$B$305)&lt;ROW(B134)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21158,7 +21148,7 @@
         <v/>
       </c>
       <c r="S135">
-        <f>IF(OR(B135="",COUNTIF($B$6:$B135,B135)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B135,$B$6:$B$305)=1)*($R$6:$R$305&gt;R135)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B135="",COUNTIF($B$6:$B135,B135)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R135)+(($R$6:$R$305=R135)*(ROW($B$6:$B$305)&lt;ROW(B135)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21180,7 +21170,7 @@
         <v/>
       </c>
       <c r="S136">
-        <f>IF(OR(B136="",COUNTIF($B$6:$B136,B136)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B136,$B$6:$B$305)=1)*($R$6:$R$305&gt;R136)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B136="",COUNTIF($B$6:$B136,B136)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R136)+(($R$6:$R$305=R136)*(ROW($B$6:$B$305)&lt;ROW(B136)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21202,7 +21192,7 @@
         <v/>
       </c>
       <c r="S137">
-        <f>IF(OR(B137="",COUNTIF($B$6:$B137,B137)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B137,$B$6:$B$305)=1)*($R$6:$R$305&gt;R137)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B137="",COUNTIF($B$6:$B137,B137)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R137)+(($R$6:$R$305=R137)*(ROW($B$6:$B$305)&lt;ROW(B137)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21224,7 +21214,7 @@
         <v/>
       </c>
       <c r="S138">
-        <f>IF(OR(B138="",COUNTIF($B$6:$B138,B138)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B138,$B$6:$B$305)=1)*($R$6:$R$305&gt;R138)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B138="",COUNTIF($B$6:$B138,B138)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R138)+(($R$6:$R$305=R138)*(ROW($B$6:$B$305)&lt;ROW(B138)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21246,7 +21236,7 @@
         <v/>
       </c>
       <c r="S139">
-        <f>IF(OR(B139="",COUNTIF($B$6:$B139,B139)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B139,$B$6:$B$305)=1)*($R$6:$R$305&gt;R139)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B139="",COUNTIF($B$6:$B139,B139)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R139)+(($R$6:$R$305=R139)*(ROW($B$6:$B$305)&lt;ROW(B139)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21268,7 +21258,7 @@
         <v/>
       </c>
       <c r="S140">
-        <f>IF(OR(B140="",COUNTIF($B$6:$B140,B140)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B140,$B$6:$B$305)=1)*($R$6:$R$305&gt;R140)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B140="",COUNTIF($B$6:$B140,B140)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R140)+(($R$6:$R$305=R140)*(ROW($B$6:$B$305)&lt;ROW(B140)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21290,7 +21280,7 @@
         <v/>
       </c>
       <c r="S141">
-        <f>IF(OR(B141="",COUNTIF($B$6:$B141,B141)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B141,$B$6:$B$305)=1)*($R$6:$R$305&gt;R141)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B141="",COUNTIF($B$6:$B141,B141)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R141)+(($R$6:$R$305=R141)*(ROW($B$6:$B$305)&lt;ROW(B141)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21312,7 +21302,7 @@
         <v/>
       </c>
       <c r="S142">
-        <f>IF(OR(B142="",COUNTIF($B$6:$B142,B142)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B142,$B$6:$B$305)=1)*($R$6:$R$305&gt;R142)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B142="",COUNTIF($B$6:$B142,B142)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R142)+(($R$6:$R$305=R142)*(ROW($B$6:$B$305)&lt;ROW(B142)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21334,7 +21324,7 @@
         <v/>
       </c>
       <c r="S143">
-        <f>IF(OR(B143="",COUNTIF($B$6:$B143,B143)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B143,$B$6:$B$305)=1)*($R$6:$R$305&gt;R143)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B143="",COUNTIF($B$6:$B143,B143)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R143)+(($R$6:$R$305=R143)*(ROW($B$6:$B$305)&lt;ROW(B143)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21356,7 +21346,7 @@
         <v/>
       </c>
       <c r="S144">
-        <f>IF(OR(B144="",COUNTIF($B$6:$B144,B144)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B144,$B$6:$B$305)=1)*($R$6:$R$305&gt;R144)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B144="",COUNTIF($B$6:$B144,B144)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R144)+(($R$6:$R$305=R144)*(ROW($B$6:$B$305)&lt;ROW(B144)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21378,7 +21368,7 @@
         <v/>
       </c>
       <c r="S145">
-        <f>IF(OR(B145="",COUNTIF($B$6:$B145,B145)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B145,$B$6:$B$305)=1)*($R$6:$R$305&gt;R145)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B145="",COUNTIF($B$6:$B145,B145)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R145)+(($R$6:$R$305=R145)*(ROW($B$6:$B$305)&lt;ROW(B145)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21400,7 +21390,7 @@
         <v/>
       </c>
       <c r="S146">
-        <f>IF(OR(B146="",COUNTIF($B$6:$B146,B146)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B146,$B$6:$B$305)=1)*($R$6:$R$305&gt;R146)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B146="",COUNTIF($B$6:$B146,B146)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R146)+(($R$6:$R$305=R146)*(ROW($B$6:$B$305)&lt;ROW(B146)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21422,7 +21412,7 @@
         <v/>
       </c>
       <c r="S147">
-        <f>IF(OR(B147="",COUNTIF($B$6:$B147,B147)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B147,$B$6:$B$305)=1)*($R$6:$R$305&gt;R147)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B147="",COUNTIF($B$6:$B147,B147)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R147)+(($R$6:$R$305=R147)*(ROW($B$6:$B$305)&lt;ROW(B147)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21444,7 +21434,7 @@
         <v/>
       </c>
       <c r="S148">
-        <f>IF(OR(B148="",COUNTIF($B$6:$B148,B148)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B148,$B$6:$B$305)=1)*($R$6:$R$305&gt;R148)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B148="",COUNTIF($B$6:$B148,B148)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R148)+(($R$6:$R$305=R148)*(ROW($B$6:$B$305)&lt;ROW(B148)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21466,7 +21456,7 @@
         <v/>
       </c>
       <c r="S149">
-        <f>IF(OR(B149="",COUNTIF($B$6:$B149,B149)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B149,$B$6:$B$305)=1)*($R$6:$R$305&gt;R149)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B149="",COUNTIF($B$6:$B149,B149)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R149)+(($R$6:$R$305=R149)*(ROW($B$6:$B$305)&lt;ROW(B149)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21488,7 +21478,7 @@
         <v/>
       </c>
       <c r="S150">
-        <f>IF(OR(B150="",COUNTIF($B$6:$B150,B150)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B150,$B$6:$B$305)=1)*($R$6:$R$305&gt;R150)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B150="",COUNTIF($B$6:$B150,B150)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R150)+(($R$6:$R$305=R150)*(ROW($B$6:$B$305)&lt;ROW(B150)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21510,7 +21500,7 @@
         <v/>
       </c>
       <c r="S151">
-        <f>IF(OR(B151="",COUNTIF($B$6:$B151,B151)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B151,$B$6:$B$305)=1)*($R$6:$R$305&gt;R151)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B151="",COUNTIF($B$6:$B151,B151)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R151)+(($R$6:$R$305=R151)*(ROW($B$6:$B$305)&lt;ROW(B151)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21532,7 +21522,7 @@
         <v/>
       </c>
       <c r="S152">
-        <f>IF(OR(B152="",COUNTIF($B$6:$B152,B152)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B152,$B$6:$B$305)=1)*($R$6:$R$305&gt;R152)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B152="",COUNTIF($B$6:$B152,B152)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R152)+(($R$6:$R$305=R152)*(ROW($B$6:$B$305)&lt;ROW(B152)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21554,7 +21544,7 @@
         <v/>
       </c>
       <c r="S153">
-        <f>IF(OR(B153="",COUNTIF($B$6:$B153,B153)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B153,$B$6:$B$305)=1)*($R$6:$R$305&gt;R153)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B153="",COUNTIF($B$6:$B153,B153)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R153)+(($R$6:$R$305=R153)*(ROW($B$6:$B$305)&lt;ROW(B153)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21576,7 +21566,7 @@
         <v/>
       </c>
       <c r="S154">
-        <f>IF(OR(B154="",COUNTIF($B$6:$B154,B154)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B154,$B$6:$B$305)=1)*($R$6:$R$305&gt;R154)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B154="",COUNTIF($B$6:$B154,B154)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R154)+(($R$6:$R$305=R154)*(ROW($B$6:$B$305)&lt;ROW(B154)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21598,7 +21588,7 @@
         <v/>
       </c>
       <c r="S155">
-        <f>IF(OR(B155="",COUNTIF($B$6:$B155,B155)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B155,$B$6:$B$305)=1)*($R$6:$R$305&gt;R155)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B155="",COUNTIF($B$6:$B155,B155)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R155)+(($R$6:$R$305=R155)*(ROW($B$6:$B$305)&lt;ROW(B155)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21620,7 +21610,7 @@
         <v/>
       </c>
       <c r="S156">
-        <f>IF(OR(B156="",COUNTIF($B$6:$B156,B156)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B156,$B$6:$B$305)=1)*($R$6:$R$305&gt;R156)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B156="",COUNTIF($B$6:$B156,B156)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R156)+(($R$6:$R$305=R156)*(ROW($B$6:$B$305)&lt;ROW(B156)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21642,7 +21632,7 @@
         <v/>
       </c>
       <c r="S157">
-        <f>IF(OR(B157="",COUNTIF($B$6:$B157,B157)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B157,$B$6:$B$305)=1)*($R$6:$R$305&gt;R157)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B157="",COUNTIF($B$6:$B157,B157)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R157)+(($R$6:$R$305=R157)*(ROW($B$6:$B$305)&lt;ROW(B157)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21664,7 +21654,7 @@
         <v/>
       </c>
       <c r="S158">
-        <f>IF(OR(B158="",COUNTIF($B$6:$B158,B158)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B158,$B$6:$B$305)=1)*($R$6:$R$305&gt;R158)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B158="",COUNTIF($B$6:$B158,B158)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R158)+(($R$6:$R$305=R158)*(ROW($B$6:$B$305)&lt;ROW(B158)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21686,7 +21676,7 @@
         <v/>
       </c>
       <c r="S159">
-        <f>IF(OR(B159="",COUNTIF($B$6:$B159,B159)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B159,$B$6:$B$305)=1)*($R$6:$R$305&gt;R159)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B159="",COUNTIF($B$6:$B159,B159)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R159)+(($R$6:$R$305=R159)*(ROW($B$6:$B$305)&lt;ROW(B159)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21708,7 +21698,7 @@
         <v/>
       </c>
       <c r="S160">
-        <f>IF(OR(B160="",COUNTIF($B$6:$B160,B160)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B160,$B$6:$B$305)=1)*($R$6:$R$305&gt;R160)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B160="",COUNTIF($B$6:$B160,B160)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R160)+(($R$6:$R$305=R160)*(ROW($B$6:$B$305)&lt;ROW(B160)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21730,7 +21720,7 @@
         <v/>
       </c>
       <c r="S161">
-        <f>IF(OR(B161="",COUNTIF($B$6:$B161,B161)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B161,$B$6:$B$305)=1)*($R$6:$R$305&gt;R161)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B161="",COUNTIF($B$6:$B161,B161)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R161)+(($R$6:$R$305=R161)*(ROW($B$6:$B$305)&lt;ROW(B161)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21752,7 +21742,7 @@
         <v/>
       </c>
       <c r="S162">
-        <f>IF(OR(B162="",COUNTIF($B$6:$B162,B162)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B162,$B$6:$B$305)=1)*($R$6:$R$305&gt;R162)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B162="",COUNTIF($B$6:$B162,B162)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R162)+(($R$6:$R$305=R162)*(ROW($B$6:$B$305)&lt;ROW(B162)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21774,7 +21764,7 @@
         <v/>
       </c>
       <c r="S163">
-        <f>IF(OR(B163="",COUNTIF($B$6:$B163,B163)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B163,$B$6:$B$305)=1)*($R$6:$R$305&gt;R163)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B163="",COUNTIF($B$6:$B163,B163)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R163)+(($R$6:$R$305=R163)*(ROW($B$6:$B$305)&lt;ROW(B163)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21796,7 +21786,7 @@
         <v/>
       </c>
       <c r="S164">
-        <f>IF(OR(B164="",COUNTIF($B$6:$B164,B164)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B164,$B$6:$B$305)=1)*($R$6:$R$305&gt;R164)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B164="",COUNTIF($B$6:$B164,B164)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R164)+(($R$6:$R$305=R164)*(ROW($B$6:$B$305)&lt;ROW(B164)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21818,7 +21808,7 @@
         <v/>
       </c>
       <c r="S165">
-        <f>IF(OR(B165="",COUNTIF($B$6:$B165,B165)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B165,$B$6:$B$305)=1)*($R$6:$R$305&gt;R165)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B165="",COUNTIF($B$6:$B165,B165)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R165)+(($R$6:$R$305=R165)*(ROW($B$6:$B$305)&lt;ROW(B165)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21840,7 +21830,7 @@
         <v/>
       </c>
       <c r="S166">
-        <f>IF(OR(B166="",COUNTIF($B$6:$B166,B166)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B166,$B$6:$B$305)=1)*($R$6:$R$305&gt;R166)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B166="",COUNTIF($B$6:$B166,B166)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R166)+(($R$6:$R$305=R166)*(ROW($B$6:$B$305)&lt;ROW(B166)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21862,7 +21852,7 @@
         <v/>
       </c>
       <c r="S167">
-        <f>IF(OR(B167="",COUNTIF($B$6:$B167,B167)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B167,$B$6:$B$305)=1)*($R$6:$R$305&gt;R167)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B167="",COUNTIF($B$6:$B167,B167)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R167)+(($R$6:$R$305=R167)*(ROW($B$6:$B$305)&lt;ROW(B167)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21884,7 +21874,7 @@
         <v/>
       </c>
       <c r="S168">
-        <f>IF(OR(B168="",COUNTIF($B$6:$B168,B168)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B168,$B$6:$B$305)=1)*($R$6:$R$305&gt;R168)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B168="",COUNTIF($B$6:$B168,B168)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R168)+(($R$6:$R$305=R168)*(ROW($B$6:$B$305)&lt;ROW(B168)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21906,7 +21896,7 @@
         <v/>
       </c>
       <c r="S169">
-        <f>IF(OR(B169="",COUNTIF($B$6:$B169,B169)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B169,$B$6:$B$305)=1)*($R$6:$R$305&gt;R169)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B169="",COUNTIF($B$6:$B169,B169)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R169)+(($R$6:$R$305=R169)*(ROW($B$6:$B$305)&lt;ROW(B169)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21928,7 +21918,7 @@
         <v/>
       </c>
       <c r="S170">
-        <f>IF(OR(B170="",COUNTIF($B$6:$B170,B170)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B170,$B$6:$B$305)=1)*($R$6:$R$305&gt;R170)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B170="",COUNTIF($B$6:$B170,B170)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R170)+(($R$6:$R$305=R170)*(ROW($B$6:$B$305)&lt;ROW(B170)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21950,7 +21940,7 @@
         <v/>
       </c>
       <c r="S171">
-        <f>IF(OR(B171="",COUNTIF($B$6:$B171,B171)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B171,$B$6:$B$305)=1)*($R$6:$R$305&gt;R171)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B171="",COUNTIF($B$6:$B171,B171)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R171)+(($R$6:$R$305=R171)*(ROW($B$6:$B$305)&lt;ROW(B171)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21972,7 +21962,7 @@
         <v/>
       </c>
       <c r="S172">
-        <f>IF(OR(B172="",COUNTIF($B$6:$B172,B172)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B172,$B$6:$B$305)=1)*($R$6:$R$305&gt;R172)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B172="",COUNTIF($B$6:$B172,B172)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R172)+(($R$6:$R$305=R172)*(ROW($B$6:$B$305)&lt;ROW(B172)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -21994,7 +21984,7 @@
         <v/>
       </c>
       <c r="S173">
-        <f>IF(OR(B173="",COUNTIF($B$6:$B173,B173)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B173,$B$6:$B$305)=1)*($R$6:$R$305&gt;R173)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B173="",COUNTIF($B$6:$B173,B173)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R173)+(($R$6:$R$305=R173)*(ROW($B$6:$B$305)&lt;ROW(B173)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22016,7 +22006,7 @@
         <v/>
       </c>
       <c r="S174">
-        <f>IF(OR(B174="",COUNTIF($B$6:$B174,B174)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B174,$B$6:$B$305)=1)*($R$6:$R$305&gt;R174)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B174="",COUNTIF($B$6:$B174,B174)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R174)+(($R$6:$R$305=R174)*(ROW($B$6:$B$305)&lt;ROW(B174)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22038,7 +22028,7 @@
         <v/>
       </c>
       <c r="S175">
-        <f>IF(OR(B175="",COUNTIF($B$6:$B175,B175)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B175,$B$6:$B$305)=1)*($R$6:$R$305&gt;R175)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B175="",COUNTIF($B$6:$B175,B175)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R175)+(($R$6:$R$305=R175)*(ROW($B$6:$B$305)&lt;ROW(B175)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22060,7 +22050,7 @@
         <v/>
       </c>
       <c r="S176">
-        <f>IF(OR(B176="",COUNTIF($B$6:$B176,B176)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B176,$B$6:$B$305)=1)*($R$6:$R$305&gt;R176)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B176="",COUNTIF($B$6:$B176,B176)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R176)+(($R$6:$R$305=R176)*(ROW($B$6:$B$305)&lt;ROW(B176)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22082,7 +22072,7 @@
         <v/>
       </c>
       <c r="S177">
-        <f>IF(OR(B177="",COUNTIF($B$6:$B177,B177)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B177,$B$6:$B$305)=1)*($R$6:$R$305&gt;R177)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B177="",COUNTIF($B$6:$B177,B177)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R177)+(($R$6:$R$305=R177)*(ROW($B$6:$B$305)&lt;ROW(B177)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22104,7 +22094,7 @@
         <v/>
       </c>
       <c r="S178">
-        <f>IF(OR(B178="",COUNTIF($B$6:$B178,B178)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B178,$B$6:$B$305)=1)*($R$6:$R$305&gt;R178)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B178="",COUNTIF($B$6:$B178,B178)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R178)+(($R$6:$R$305=R178)*(ROW($B$6:$B$305)&lt;ROW(B178)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22126,7 +22116,7 @@
         <v/>
       </c>
       <c r="S179">
-        <f>IF(OR(B179="",COUNTIF($B$6:$B179,B179)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B179,$B$6:$B$305)=1)*($R$6:$R$305&gt;R179)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B179="",COUNTIF($B$6:$B179,B179)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R179)+(($R$6:$R$305=R179)*(ROW($B$6:$B$305)&lt;ROW(B179)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22148,7 +22138,7 @@
         <v/>
       </c>
       <c r="S180">
-        <f>IF(OR(B180="",COUNTIF($B$6:$B180,B180)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B180,$B$6:$B$305)=1)*($R$6:$R$305&gt;R180)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B180="",COUNTIF($B$6:$B180,B180)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R180)+(($R$6:$R$305=R180)*(ROW($B$6:$B$305)&lt;ROW(B180)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22170,7 +22160,7 @@
         <v/>
       </c>
       <c r="S181">
-        <f>IF(OR(B181="",COUNTIF($B$6:$B181,B181)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B181,$B$6:$B$305)=1)*($R$6:$R$305&gt;R181)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B181="",COUNTIF($B$6:$B181,B181)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R181)+(($R$6:$R$305=R181)*(ROW($B$6:$B$305)&lt;ROW(B181)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22192,7 +22182,7 @@
         <v/>
       </c>
       <c r="S182">
-        <f>IF(OR(B182="",COUNTIF($B$6:$B182,B182)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B182,$B$6:$B$305)=1)*($R$6:$R$305&gt;R182)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B182="",COUNTIF($B$6:$B182,B182)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R182)+(($R$6:$R$305=R182)*(ROW($B$6:$B$305)&lt;ROW(B182)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22214,7 +22204,7 @@
         <v/>
       </c>
       <c r="S183">
-        <f>IF(OR(B183="",COUNTIF($B$6:$B183,B183)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B183,$B$6:$B$305)=1)*($R$6:$R$305&gt;R183)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B183="",COUNTIF($B$6:$B183,B183)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R183)+(($R$6:$R$305=R183)*(ROW($B$6:$B$305)&lt;ROW(B183)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22236,7 +22226,7 @@
         <v/>
       </c>
       <c r="S184">
-        <f>IF(OR(B184="",COUNTIF($B$6:$B184,B184)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B184,$B$6:$B$305)=1)*($R$6:$R$305&gt;R184)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B184="",COUNTIF($B$6:$B184,B184)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R184)+(($R$6:$R$305=R184)*(ROW($B$6:$B$305)&lt;ROW(B184)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22258,7 +22248,7 @@
         <v/>
       </c>
       <c r="S185">
-        <f>IF(OR(B185="",COUNTIF($B$6:$B185,B185)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B185,$B$6:$B$305)=1)*($R$6:$R$305&gt;R185)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B185="",COUNTIF($B$6:$B185,B185)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R185)+(($R$6:$R$305=R185)*(ROW($B$6:$B$305)&lt;ROW(B185)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22280,7 +22270,7 @@
         <v/>
       </c>
       <c r="S186">
-        <f>IF(OR(B186="",COUNTIF($B$6:$B186,B186)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B186,$B$6:$B$305)=1)*($R$6:$R$305&gt;R186)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B186="",COUNTIF($B$6:$B186,B186)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R186)+(($R$6:$R$305=R186)*(ROW($B$6:$B$305)&lt;ROW(B186)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22302,7 +22292,7 @@
         <v/>
       </c>
       <c r="S187">
-        <f>IF(OR(B187="",COUNTIF($B$6:$B187,B187)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B187,$B$6:$B$305)=1)*($R$6:$R$305&gt;R187)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B187="",COUNTIF($B$6:$B187,B187)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R187)+(($R$6:$R$305=R187)*(ROW($B$6:$B$305)&lt;ROW(B187)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22324,7 +22314,7 @@
         <v/>
       </c>
       <c r="S188">
-        <f>IF(OR(B188="",COUNTIF($B$6:$B188,B188)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B188,$B$6:$B$305)=1)*($R$6:$R$305&gt;R188)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B188="",COUNTIF($B$6:$B188,B188)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R188)+(($R$6:$R$305=R188)*(ROW($B$6:$B$305)&lt;ROW(B188)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22346,7 +22336,7 @@
         <v/>
       </c>
       <c r="S189">
-        <f>IF(OR(B189="",COUNTIF($B$6:$B189,B189)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B189,$B$6:$B$305)=1)*($R$6:$R$305&gt;R189)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B189="",COUNTIF($B$6:$B189,B189)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R189)+(($R$6:$R$305=R189)*(ROW($B$6:$B$305)&lt;ROW(B189)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22368,7 +22358,7 @@
         <v/>
       </c>
       <c r="S190">
-        <f>IF(OR(B190="",COUNTIF($B$6:$B190,B190)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B190,$B$6:$B$305)=1)*($R$6:$R$305&gt;R190)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B190="",COUNTIF($B$6:$B190,B190)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R190)+(($R$6:$R$305=R190)*(ROW($B$6:$B$305)&lt;ROW(B190)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22390,7 +22380,7 @@
         <v/>
       </c>
       <c r="S191">
-        <f>IF(OR(B191="",COUNTIF($B$6:$B191,B191)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B191,$B$6:$B$305)=1)*($R$6:$R$305&gt;R191)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B191="",COUNTIF($B$6:$B191,B191)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R191)+(($R$6:$R$305=R191)*(ROW($B$6:$B$305)&lt;ROW(B191)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22412,7 +22402,7 @@
         <v/>
       </c>
       <c r="S192">
-        <f>IF(OR(B192="",COUNTIF($B$6:$B192,B192)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B192,$B$6:$B$305)=1)*($R$6:$R$305&gt;R192)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B192="",COUNTIF($B$6:$B192,B192)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R192)+(($R$6:$R$305=R192)*(ROW($B$6:$B$305)&lt;ROW(B192)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22434,7 +22424,7 @@
         <v/>
       </c>
       <c r="S193">
-        <f>IF(OR(B193="",COUNTIF($B$6:$B193,B193)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B193,$B$6:$B$305)=1)*($R$6:$R$305&gt;R193)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B193="",COUNTIF($B$6:$B193,B193)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R193)+(($R$6:$R$305=R193)*(ROW($B$6:$B$305)&lt;ROW(B193)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22456,7 +22446,7 @@
         <v/>
       </c>
       <c r="S194">
-        <f>IF(OR(B194="",COUNTIF($B$6:$B194,B194)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B194,$B$6:$B$305)=1)*($R$6:$R$305&gt;R194)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B194="",COUNTIF($B$6:$B194,B194)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R194)+(($R$6:$R$305=R194)*(ROW($B$6:$B$305)&lt;ROW(B194)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22478,7 +22468,7 @@
         <v/>
       </c>
       <c r="S195">
-        <f>IF(OR(B195="",COUNTIF($B$6:$B195,B195)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B195,$B$6:$B$305)=1)*($R$6:$R$305&gt;R195)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B195="",COUNTIF($B$6:$B195,B195)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R195)+(($R$6:$R$305=R195)*(ROW($B$6:$B$305)&lt;ROW(B195)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22500,7 +22490,7 @@
         <v/>
       </c>
       <c r="S196">
-        <f>IF(OR(B196="",COUNTIF($B$6:$B196,B196)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B196,$B$6:$B$305)=1)*($R$6:$R$305&gt;R196)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B196="",COUNTIF($B$6:$B196,B196)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R196)+(($R$6:$R$305=R196)*(ROW($B$6:$B$305)&lt;ROW(B196)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22522,7 +22512,7 @@
         <v/>
       </c>
       <c r="S197">
-        <f>IF(OR(B197="",COUNTIF($B$6:$B197,B197)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B197,$B$6:$B$305)=1)*($R$6:$R$305&gt;R197)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B197="",COUNTIF($B$6:$B197,B197)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R197)+(($R$6:$R$305=R197)*(ROW($B$6:$B$305)&lt;ROW(B197)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22544,7 +22534,7 @@
         <v/>
       </c>
       <c r="S198">
-        <f>IF(OR(B198="",COUNTIF($B$6:$B198,B198)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B198,$B$6:$B$305)=1)*($R$6:$R$305&gt;R198)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B198="",COUNTIF($B$6:$B198,B198)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R198)+(($R$6:$R$305=R198)*(ROW($B$6:$B$305)&lt;ROW(B198)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22566,7 +22556,7 @@
         <v/>
       </c>
       <c r="S199">
-        <f>IF(OR(B199="",COUNTIF($B$6:$B199,B199)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B199,$B$6:$B$305)=1)*($R$6:$R$305&gt;R199)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B199="",COUNTIF($B$6:$B199,B199)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R199)+(($R$6:$R$305=R199)*(ROW($B$6:$B$305)&lt;ROW(B199)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22588,7 +22578,7 @@
         <v/>
       </c>
       <c r="S200">
-        <f>IF(OR(B200="",COUNTIF($B$6:$B200,B200)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B200,$B$6:$B$305)=1)*($R$6:$R$305&gt;R200)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B200="",COUNTIF($B$6:$B200,B200)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R200)+(($R$6:$R$305=R200)*(ROW($B$6:$B$305)&lt;ROW(B200)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22610,7 +22600,7 @@
         <v/>
       </c>
       <c r="S201">
-        <f>IF(OR(B201="",COUNTIF($B$6:$B201,B201)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B201,$B$6:$B$305)=1)*($R$6:$R$305&gt;R201)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B201="",COUNTIF($B$6:$B201,B201)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R201)+(($R$6:$R$305=R201)*(ROW($B$6:$B$305)&lt;ROW(B201)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22632,7 +22622,7 @@
         <v/>
       </c>
       <c r="S202">
-        <f>IF(OR(B202="",COUNTIF($B$6:$B202,B202)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B202,$B$6:$B$305)=1)*($R$6:$R$305&gt;R202)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B202="",COUNTIF($B$6:$B202,B202)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R202)+(($R$6:$R$305=R202)*(ROW($B$6:$B$305)&lt;ROW(B202)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22654,7 +22644,7 @@
         <v/>
       </c>
       <c r="S203">
-        <f>IF(OR(B203="",COUNTIF($B$6:$B203,B203)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B203,$B$6:$B$305)=1)*($R$6:$R$305&gt;R203)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B203="",COUNTIF($B$6:$B203,B203)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R203)+(($R$6:$R$305=R203)*(ROW($B$6:$B$305)&lt;ROW(B203)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22676,7 +22666,7 @@
         <v/>
       </c>
       <c r="S204">
-        <f>IF(OR(B204="",COUNTIF($B$6:$B204,B204)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B204,$B$6:$B$305)=1)*($R$6:$R$305&gt;R204)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B204="",COUNTIF($B$6:$B204,B204)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R204)+(($R$6:$R$305=R204)*(ROW($B$6:$B$305)&lt;ROW(B204)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22698,7 +22688,7 @@
         <v/>
       </c>
       <c r="S205">
-        <f>IF(OR(B205="",COUNTIF($B$6:$B205,B205)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B205,$B$6:$B$305)=1)*($R$6:$R$305&gt;R205)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B205="",COUNTIF($B$6:$B205,B205)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R205)+(($R$6:$R$305=R205)*(ROW($B$6:$B$305)&lt;ROW(B205)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22720,7 +22710,7 @@
         <v/>
       </c>
       <c r="S206">
-        <f>IF(OR(B206="",COUNTIF($B$6:$B206,B206)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B206,$B$6:$B$305)=1)*($R$6:$R$305&gt;R206)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B206="",COUNTIF($B$6:$B206,B206)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R206)+(($R$6:$R$305=R206)*(ROW($B$6:$B$305)&lt;ROW(B206)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22742,7 +22732,7 @@
         <v/>
       </c>
       <c r="S207">
-        <f>IF(OR(B207="",COUNTIF($B$6:$B207,B207)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B207,$B$6:$B$305)=1)*($R$6:$R$305&gt;R207)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B207="",COUNTIF($B$6:$B207,B207)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R207)+(($R$6:$R$305=R207)*(ROW($B$6:$B$305)&lt;ROW(B207)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22764,7 +22754,7 @@
         <v/>
       </c>
       <c r="S208">
-        <f>IF(OR(B208="",COUNTIF($B$6:$B208,B208)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B208,$B$6:$B$305)=1)*($R$6:$R$305&gt;R208)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B208="",COUNTIF($B$6:$B208,B208)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R208)+(($R$6:$R$305=R208)*(ROW($B$6:$B$305)&lt;ROW(B208)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22786,7 +22776,7 @@
         <v/>
       </c>
       <c r="S209">
-        <f>IF(OR(B209="",COUNTIF($B$6:$B209,B209)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B209,$B$6:$B$305)=1)*($R$6:$R$305&gt;R209)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B209="",COUNTIF($B$6:$B209,B209)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R209)+(($R$6:$R$305=R209)*(ROW($B$6:$B$305)&lt;ROW(B209)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22808,7 +22798,7 @@
         <v/>
       </c>
       <c r="S210">
-        <f>IF(OR(B210="",COUNTIF($B$6:$B210,B210)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B210,$B$6:$B$305)=1)*($R$6:$R$305&gt;R210)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B210="",COUNTIF($B$6:$B210,B210)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R210)+(($R$6:$R$305=R210)*(ROW($B$6:$B$305)&lt;ROW(B210)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22830,7 +22820,7 @@
         <v/>
       </c>
       <c r="S211">
-        <f>IF(OR(B211="",COUNTIF($B$6:$B211,B211)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B211,$B$6:$B$305)=1)*($R$6:$R$305&gt;R211)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B211="",COUNTIF($B$6:$B211,B211)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R211)+(($R$6:$R$305=R211)*(ROW($B$6:$B$305)&lt;ROW(B211)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22852,7 +22842,7 @@
         <v/>
       </c>
       <c r="S212">
-        <f>IF(OR(B212="",COUNTIF($B$6:$B212,B212)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B212,$B$6:$B$305)=1)*($R$6:$R$305&gt;R212)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B212="",COUNTIF($B$6:$B212,B212)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R212)+(($R$6:$R$305=R212)*(ROW($B$6:$B$305)&lt;ROW(B212)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22874,7 +22864,7 @@
         <v/>
       </c>
       <c r="S213">
-        <f>IF(OR(B213="",COUNTIF($B$6:$B213,B213)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B213,$B$6:$B$305)=1)*($R$6:$R$305&gt;R213)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B213="",COUNTIF($B$6:$B213,B213)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R213)+(($R$6:$R$305=R213)*(ROW($B$6:$B$305)&lt;ROW(B213)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22896,7 +22886,7 @@
         <v/>
       </c>
       <c r="S214">
-        <f>IF(OR(B214="",COUNTIF($B$6:$B214,B214)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B214,$B$6:$B$305)=1)*($R$6:$R$305&gt;R214)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B214="",COUNTIF($B$6:$B214,B214)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R214)+(($R$6:$R$305=R214)*(ROW($B$6:$B$305)&lt;ROW(B214)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22918,7 +22908,7 @@
         <v/>
       </c>
       <c r="S215">
-        <f>IF(OR(B215="",COUNTIF($B$6:$B215,B215)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B215,$B$6:$B$305)=1)*($R$6:$R$305&gt;R215)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B215="",COUNTIF($B$6:$B215,B215)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R215)+(($R$6:$R$305=R215)*(ROW($B$6:$B$305)&lt;ROW(B215)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22940,7 +22930,7 @@
         <v/>
       </c>
       <c r="S216">
-        <f>IF(OR(B216="",COUNTIF($B$6:$B216,B216)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B216,$B$6:$B$305)=1)*($R$6:$R$305&gt;R216)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B216="",COUNTIF($B$6:$B216,B216)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R216)+(($R$6:$R$305=R216)*(ROW($B$6:$B$305)&lt;ROW(B216)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22962,7 +22952,7 @@
         <v/>
       </c>
       <c r="S217">
-        <f>IF(OR(B217="",COUNTIF($B$6:$B217,B217)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B217,$B$6:$B$305)=1)*($R$6:$R$305&gt;R217)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B217="",COUNTIF($B$6:$B217,B217)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R217)+(($R$6:$R$305=R217)*(ROW($B$6:$B$305)&lt;ROW(B217)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -22984,7 +22974,7 @@
         <v/>
       </c>
       <c r="S218">
-        <f>IF(OR(B218="",COUNTIF($B$6:$B218,B218)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B218,$B$6:$B$305)=1)*($R$6:$R$305&gt;R218)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B218="",COUNTIF($B$6:$B218,B218)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R218)+(($R$6:$R$305=R218)*(ROW($B$6:$B$305)&lt;ROW(B218)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23006,7 +22996,7 @@
         <v/>
       </c>
       <c r="S219">
-        <f>IF(OR(B219="",COUNTIF($B$6:$B219,B219)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B219,$B$6:$B$305)=1)*($R$6:$R$305&gt;R219)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B219="",COUNTIF($B$6:$B219,B219)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R219)+(($R$6:$R$305=R219)*(ROW($B$6:$B$305)&lt;ROW(B219)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23028,7 +23018,7 @@
         <v/>
       </c>
       <c r="S220">
-        <f>IF(OR(B220="",COUNTIF($B$6:$B220,B220)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B220,$B$6:$B$305)=1)*($R$6:$R$305&gt;R220)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B220="",COUNTIF($B$6:$B220,B220)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R220)+(($R$6:$R$305=R220)*(ROW($B$6:$B$305)&lt;ROW(B220)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23050,7 +23040,7 @@
         <v/>
       </c>
       <c r="S221">
-        <f>IF(OR(B221="",COUNTIF($B$6:$B221,B221)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B221,$B$6:$B$305)=1)*($R$6:$R$305&gt;R221)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B221="",COUNTIF($B$6:$B221,B221)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R221)+(($R$6:$R$305=R221)*(ROW($B$6:$B$305)&lt;ROW(B221)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23072,7 +23062,7 @@
         <v/>
       </c>
       <c r="S222">
-        <f>IF(OR(B222="",COUNTIF($B$6:$B222,B222)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B222,$B$6:$B$305)=1)*($R$6:$R$305&gt;R222)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B222="",COUNTIF($B$6:$B222,B222)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R222)+(($R$6:$R$305=R222)*(ROW($B$6:$B$305)&lt;ROW(B222)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23094,7 +23084,7 @@
         <v/>
       </c>
       <c r="S223">
-        <f>IF(OR(B223="",COUNTIF($B$6:$B223,B223)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B223,$B$6:$B$305)=1)*($R$6:$R$305&gt;R223)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B223="",COUNTIF($B$6:$B223,B223)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R223)+(($R$6:$R$305=R223)*(ROW($B$6:$B$305)&lt;ROW(B223)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23116,7 +23106,7 @@
         <v/>
       </c>
       <c r="S224">
-        <f>IF(OR(B224="",COUNTIF($B$6:$B224,B224)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B224,$B$6:$B$305)=1)*($R$6:$R$305&gt;R224)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B224="",COUNTIF($B$6:$B224,B224)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R224)+(($R$6:$R$305=R224)*(ROW($B$6:$B$305)&lt;ROW(B224)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23138,7 +23128,7 @@
         <v/>
       </c>
       <c r="S225">
-        <f>IF(OR(B225="",COUNTIF($B$6:$B225,B225)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B225,$B$6:$B$305)=1)*($R$6:$R$305&gt;R225)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B225="",COUNTIF($B$6:$B225,B225)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R225)+(($R$6:$R$305=R225)*(ROW($B$6:$B$305)&lt;ROW(B225)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23160,7 +23150,7 @@
         <v/>
       </c>
       <c r="S226">
-        <f>IF(OR(B226="",COUNTIF($B$6:$B226,B226)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B226,$B$6:$B$305)=1)*($R$6:$R$305&gt;R226)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B226="",COUNTIF($B$6:$B226,B226)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R226)+(($R$6:$R$305=R226)*(ROW($B$6:$B$305)&lt;ROW(B226)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23182,7 +23172,7 @@
         <v/>
       </c>
       <c r="S227">
-        <f>IF(OR(B227="",COUNTIF($B$6:$B227,B227)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B227,$B$6:$B$305)=1)*($R$6:$R$305&gt;R227)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B227="",COUNTIF($B$6:$B227,B227)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R227)+(($R$6:$R$305=R227)*(ROW($B$6:$B$305)&lt;ROW(B227)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23204,7 +23194,7 @@
         <v/>
       </c>
       <c r="S228">
-        <f>IF(OR(B228="",COUNTIF($B$6:$B228,B228)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B228,$B$6:$B$305)=1)*($R$6:$R$305&gt;R228)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B228="",COUNTIF($B$6:$B228,B228)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R228)+(($R$6:$R$305=R228)*(ROW($B$6:$B$305)&lt;ROW(B228)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23226,7 +23216,7 @@
         <v/>
       </c>
       <c r="S229">
-        <f>IF(OR(B229="",COUNTIF($B$6:$B229,B229)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B229,$B$6:$B$305)=1)*($R$6:$R$305&gt;R229)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B229="",COUNTIF($B$6:$B229,B229)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R229)+(($R$6:$R$305=R229)*(ROW($B$6:$B$305)&lt;ROW(B229)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23248,7 +23238,7 @@
         <v/>
       </c>
       <c r="S230">
-        <f>IF(OR(B230="",COUNTIF($B$6:$B230,B230)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B230,$B$6:$B$305)=1)*($R$6:$R$305&gt;R230)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B230="",COUNTIF($B$6:$B230,B230)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R230)+(($R$6:$R$305=R230)*(ROW($B$6:$B$305)&lt;ROW(B230)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23270,7 +23260,7 @@
         <v/>
       </c>
       <c r="S231">
-        <f>IF(OR(B231="",COUNTIF($B$6:$B231,B231)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B231,$B$6:$B$305)=1)*($R$6:$R$305&gt;R231)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B231="",COUNTIF($B$6:$B231,B231)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R231)+(($R$6:$R$305=R231)*(ROW($B$6:$B$305)&lt;ROW(B231)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23292,7 +23282,7 @@
         <v/>
       </c>
       <c r="S232">
-        <f>IF(OR(B232="",COUNTIF($B$6:$B232,B232)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B232,$B$6:$B$305)=1)*($R$6:$R$305&gt;R232)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B232="",COUNTIF($B$6:$B232,B232)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R232)+(($R$6:$R$305=R232)*(ROW($B$6:$B$305)&lt;ROW(B232)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23314,7 +23304,7 @@
         <v/>
       </c>
       <c r="S233">
-        <f>IF(OR(B233="",COUNTIF($B$6:$B233,B233)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B233,$B$6:$B$305)=1)*($R$6:$R$305&gt;R233)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B233="",COUNTIF($B$6:$B233,B233)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R233)+(($R$6:$R$305=R233)*(ROW($B$6:$B$305)&lt;ROW(B233)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23336,7 +23326,7 @@
         <v/>
       </c>
       <c r="S234">
-        <f>IF(OR(B234="",COUNTIF($B$6:$B234,B234)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B234,$B$6:$B$305)=1)*($R$6:$R$305&gt;R234)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B234="",COUNTIF($B$6:$B234,B234)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R234)+(($R$6:$R$305=R234)*(ROW($B$6:$B$305)&lt;ROW(B234)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23358,7 +23348,7 @@
         <v/>
       </c>
       <c r="S235">
-        <f>IF(OR(B235="",COUNTIF($B$6:$B235,B235)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B235,$B$6:$B$305)=1)*($R$6:$R$305&gt;R235)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B235="",COUNTIF($B$6:$B235,B235)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R235)+(($R$6:$R$305=R235)*(ROW($B$6:$B$305)&lt;ROW(B235)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23380,7 +23370,7 @@
         <v/>
       </c>
       <c r="S236">
-        <f>IF(OR(B236="",COUNTIF($B$6:$B236,B236)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B236,$B$6:$B$305)=1)*($R$6:$R$305&gt;R236)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B236="",COUNTIF($B$6:$B236,B236)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R236)+(($R$6:$R$305=R236)*(ROW($B$6:$B$305)&lt;ROW(B236)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23402,7 +23392,7 @@
         <v/>
       </c>
       <c r="S237">
-        <f>IF(OR(B237="",COUNTIF($B$6:$B237,B237)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B237,$B$6:$B$305)=1)*($R$6:$R$305&gt;R237)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B237="",COUNTIF($B$6:$B237,B237)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R237)+(($R$6:$R$305=R237)*(ROW($B$6:$B$305)&lt;ROW(B237)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23424,7 +23414,7 @@
         <v/>
       </c>
       <c r="S238">
-        <f>IF(OR(B238="",COUNTIF($B$6:$B238,B238)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B238,$B$6:$B$305)=1)*($R$6:$R$305&gt;R238)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B238="",COUNTIF($B$6:$B238,B238)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R238)+(($R$6:$R$305=R238)*(ROW($B$6:$B$305)&lt;ROW(B238)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23446,7 +23436,7 @@
         <v/>
       </c>
       <c r="S239">
-        <f>IF(OR(B239="",COUNTIF($B$6:$B239,B239)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B239,$B$6:$B$305)=1)*($R$6:$R$305&gt;R239)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B239="",COUNTIF($B$6:$B239,B239)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R239)+(($R$6:$R$305=R239)*(ROW($B$6:$B$305)&lt;ROW(B239)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23468,7 +23458,7 @@
         <v/>
       </c>
       <c r="S240">
-        <f>IF(OR(B240="",COUNTIF($B$6:$B240,B240)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B240,$B$6:$B$305)=1)*($R$6:$R$305&gt;R240)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B240="",COUNTIF($B$6:$B240,B240)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R240)+(($R$6:$R$305=R240)*(ROW($B$6:$B$305)&lt;ROW(B240)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23490,7 +23480,7 @@
         <v/>
       </c>
       <c r="S241">
-        <f>IF(OR(B241="",COUNTIF($B$6:$B241,B241)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B241,$B$6:$B$305)=1)*($R$6:$R$305&gt;R241)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B241="",COUNTIF($B$6:$B241,B241)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R241)+(($R$6:$R$305=R241)*(ROW($B$6:$B$305)&lt;ROW(B241)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23512,7 +23502,7 @@
         <v/>
       </c>
       <c r="S242">
-        <f>IF(OR(B242="",COUNTIF($B$6:$B242,B242)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B242,$B$6:$B$305)=1)*($R$6:$R$305&gt;R242)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B242="",COUNTIF($B$6:$B242,B242)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R242)+(($R$6:$R$305=R242)*(ROW($B$6:$B$305)&lt;ROW(B242)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23534,7 +23524,7 @@
         <v/>
       </c>
       <c r="S243">
-        <f>IF(OR(B243="",COUNTIF($B$6:$B243,B243)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B243,$B$6:$B$305)=1)*($R$6:$R$305&gt;R243)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B243="",COUNTIF($B$6:$B243,B243)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R243)+(($R$6:$R$305=R243)*(ROW($B$6:$B$305)&lt;ROW(B243)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23556,7 +23546,7 @@
         <v/>
       </c>
       <c r="S244">
-        <f>IF(OR(B244="",COUNTIF($B$6:$B244,B244)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B244,$B$6:$B$305)=1)*($R$6:$R$305&gt;R244)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B244="",COUNTIF($B$6:$B244,B244)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R244)+(($R$6:$R$305=R244)*(ROW($B$6:$B$305)&lt;ROW(B244)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23578,7 +23568,7 @@
         <v/>
       </c>
       <c r="S245">
-        <f>IF(OR(B245="",COUNTIF($B$6:$B245,B245)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B245,$B$6:$B$305)=1)*($R$6:$R$305&gt;R245)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B245="",COUNTIF($B$6:$B245,B245)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R245)+(($R$6:$R$305=R245)*(ROW($B$6:$B$305)&lt;ROW(B245)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23600,7 +23590,7 @@
         <v/>
       </c>
       <c r="S246">
-        <f>IF(OR(B246="",COUNTIF($B$6:$B246,B246)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B246,$B$6:$B$305)=1)*($R$6:$R$305&gt;R246)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B246="",COUNTIF($B$6:$B246,B246)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R246)+(($R$6:$R$305=R246)*(ROW($B$6:$B$305)&lt;ROW(B246)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23622,7 +23612,7 @@
         <v/>
       </c>
       <c r="S247">
-        <f>IF(OR(B247="",COUNTIF($B$6:$B247,B247)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B247,$B$6:$B$305)=1)*($R$6:$R$305&gt;R247)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B247="",COUNTIF($B$6:$B247,B247)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R247)+(($R$6:$R$305=R247)*(ROW($B$6:$B$305)&lt;ROW(B247)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23644,7 +23634,7 @@
         <v/>
       </c>
       <c r="S248">
-        <f>IF(OR(B248="",COUNTIF($B$6:$B248,B248)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B248,$B$6:$B$305)=1)*($R$6:$R$305&gt;R248)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B248="",COUNTIF($B$6:$B248,B248)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R248)+(($R$6:$R$305=R248)*(ROW($B$6:$B$305)&lt;ROW(B248)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23666,7 +23656,7 @@
         <v/>
       </c>
       <c r="S249">
-        <f>IF(OR(B249="",COUNTIF($B$6:$B249,B249)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B249,$B$6:$B$305)=1)*($R$6:$R$305&gt;R249)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B249="",COUNTIF($B$6:$B249,B249)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R249)+(($R$6:$R$305=R249)*(ROW($B$6:$B$305)&lt;ROW(B249)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23688,7 +23678,7 @@
         <v/>
       </c>
       <c r="S250">
-        <f>IF(OR(B250="",COUNTIF($B$6:$B250,B250)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B250,$B$6:$B$305)=1)*($R$6:$R$305&gt;R250)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B250="",COUNTIF($B$6:$B250,B250)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R250)+(($R$6:$R$305=R250)*(ROW($B$6:$B$305)&lt;ROW(B250)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23710,7 +23700,7 @@
         <v/>
       </c>
       <c r="S251">
-        <f>IF(OR(B251="",COUNTIF($B$6:$B251,B251)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B251,$B$6:$B$305)=1)*($R$6:$R$305&gt;R251)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B251="",COUNTIF($B$6:$B251,B251)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R251)+(($R$6:$R$305=R251)*(ROW($B$6:$B$305)&lt;ROW(B251)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23732,7 +23722,7 @@
         <v/>
       </c>
       <c r="S252">
-        <f>IF(OR(B252="",COUNTIF($B$6:$B252,B252)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B252,$B$6:$B$305)=1)*($R$6:$R$305&gt;R252)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B252="",COUNTIF($B$6:$B252,B252)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R252)+(($R$6:$R$305=R252)*(ROW($B$6:$B$305)&lt;ROW(B252)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23754,7 +23744,7 @@
         <v/>
       </c>
       <c r="S253">
-        <f>IF(OR(B253="",COUNTIF($B$6:$B253,B253)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B253,$B$6:$B$305)=1)*($R$6:$R$305&gt;R253)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B253="",COUNTIF($B$6:$B253,B253)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R253)+(($R$6:$R$305=R253)*(ROW($B$6:$B$305)&lt;ROW(B253)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23776,7 +23766,7 @@
         <v/>
       </c>
       <c r="S254">
-        <f>IF(OR(B254="",COUNTIF($B$6:$B254,B254)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B254,$B$6:$B$305)=1)*($R$6:$R$305&gt;R254)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B254="",COUNTIF($B$6:$B254,B254)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R254)+(($R$6:$R$305=R254)*(ROW($B$6:$B$305)&lt;ROW(B254)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23798,7 +23788,7 @@
         <v/>
       </c>
       <c r="S255">
-        <f>IF(OR(B255="",COUNTIF($B$6:$B255,B255)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B255,$B$6:$B$305)=1)*($R$6:$R$305&gt;R255)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B255="",COUNTIF($B$6:$B255,B255)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R255)+(($R$6:$R$305=R255)*(ROW($B$6:$B$305)&lt;ROW(B255)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23820,7 +23810,7 @@
         <v/>
       </c>
       <c r="S256">
-        <f>IF(OR(B256="",COUNTIF($B$6:$B256,B256)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B256,$B$6:$B$305)=1)*($R$6:$R$305&gt;R256)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B256="",COUNTIF($B$6:$B256,B256)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R256)+(($R$6:$R$305=R256)*(ROW($B$6:$B$305)&lt;ROW(B256)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23842,7 +23832,7 @@
         <v/>
       </c>
       <c r="S257">
-        <f>IF(OR(B257="",COUNTIF($B$6:$B257,B257)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B257,$B$6:$B$305)=1)*($R$6:$R$305&gt;R257)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B257="",COUNTIF($B$6:$B257,B257)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R257)+(($R$6:$R$305=R257)*(ROW($B$6:$B$305)&lt;ROW(B257)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23864,7 +23854,7 @@
         <v/>
       </c>
       <c r="S258">
-        <f>IF(OR(B258="",COUNTIF($B$6:$B258,B258)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B258,$B$6:$B$305)=1)*($R$6:$R$305&gt;R258)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B258="",COUNTIF($B$6:$B258,B258)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R258)+(($R$6:$R$305=R258)*(ROW($B$6:$B$305)&lt;ROW(B258)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23886,7 +23876,7 @@
         <v/>
       </c>
       <c r="S259">
-        <f>IF(OR(B259="",COUNTIF($B$6:$B259,B259)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B259,$B$6:$B$305)=1)*($R$6:$R$305&gt;R259)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B259="",COUNTIF($B$6:$B259,B259)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R259)+(($R$6:$R$305=R259)*(ROW($B$6:$B$305)&lt;ROW(B259)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23908,7 +23898,7 @@
         <v/>
       </c>
       <c r="S260">
-        <f>IF(OR(B260="",COUNTIF($B$6:$B260,B260)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B260,$B$6:$B$305)=1)*($R$6:$R$305&gt;R260)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B260="",COUNTIF($B$6:$B260,B260)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R260)+(($R$6:$R$305=R260)*(ROW($B$6:$B$305)&lt;ROW(B260)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23930,7 +23920,7 @@
         <v/>
       </c>
       <c r="S261">
-        <f>IF(OR(B261="",COUNTIF($B$6:$B261,B261)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B261,$B$6:$B$305)=1)*($R$6:$R$305&gt;R261)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B261="",COUNTIF($B$6:$B261,B261)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R261)+(($R$6:$R$305=R261)*(ROW($B$6:$B$305)&lt;ROW(B261)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23952,7 +23942,7 @@
         <v/>
       </c>
       <c r="S262">
-        <f>IF(OR(B262="",COUNTIF($B$6:$B262,B262)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B262,$B$6:$B$305)=1)*($R$6:$R$305&gt;R262)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B262="",COUNTIF($B$6:$B262,B262)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R262)+(($R$6:$R$305=R262)*(ROW($B$6:$B$305)&lt;ROW(B262)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23974,7 +23964,7 @@
         <v/>
       </c>
       <c r="S263">
-        <f>IF(OR(B263="",COUNTIF($B$6:$B263,B263)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B263,$B$6:$B$305)=1)*($R$6:$R$305&gt;R263)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B263="",COUNTIF($B$6:$B263,B263)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R263)+(($R$6:$R$305=R263)*(ROW($B$6:$B$305)&lt;ROW(B263)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -23996,7 +23986,7 @@
         <v/>
       </c>
       <c r="S264">
-        <f>IF(OR(B264="",COUNTIF($B$6:$B264,B264)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B264,$B$6:$B$305)=1)*($R$6:$R$305&gt;R264)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B264="",COUNTIF($B$6:$B264,B264)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R264)+(($R$6:$R$305=R264)*(ROW($B$6:$B$305)&lt;ROW(B264)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24018,7 +24008,7 @@
         <v/>
       </c>
       <c r="S265">
-        <f>IF(OR(B265="",COUNTIF($B$6:$B265,B265)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B265,$B$6:$B$305)=1)*($R$6:$R$305&gt;R265)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B265="",COUNTIF($B$6:$B265,B265)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R265)+(($R$6:$R$305=R265)*(ROW($B$6:$B$305)&lt;ROW(B265)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24040,7 +24030,7 @@
         <v/>
       </c>
       <c r="S266">
-        <f>IF(OR(B266="",COUNTIF($B$6:$B266,B266)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B266,$B$6:$B$305)=1)*($R$6:$R$305&gt;R266)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B266="",COUNTIF($B$6:$B266,B266)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R266)+(($R$6:$R$305=R266)*(ROW($B$6:$B$305)&lt;ROW(B266)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24062,7 +24052,7 @@
         <v/>
       </c>
       <c r="S267">
-        <f>IF(OR(B267="",COUNTIF($B$6:$B267,B267)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B267,$B$6:$B$305)=1)*($R$6:$R$305&gt;R267)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B267="",COUNTIF($B$6:$B267,B267)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R267)+(($R$6:$R$305=R267)*(ROW($B$6:$B$305)&lt;ROW(B267)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24084,7 +24074,7 @@
         <v/>
       </c>
       <c r="S268">
-        <f>IF(OR(B268="",COUNTIF($B$6:$B268,B268)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B268,$B$6:$B$305)=1)*($R$6:$R$305&gt;R268)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B268="",COUNTIF($B$6:$B268,B268)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R268)+(($R$6:$R$305=R268)*(ROW($B$6:$B$305)&lt;ROW(B268)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24106,7 +24096,7 @@
         <v/>
       </c>
       <c r="S269">
-        <f>IF(OR(B269="",COUNTIF($B$6:$B269,B269)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B269,$B$6:$B$305)=1)*($R$6:$R$305&gt;R269)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B269="",COUNTIF($B$6:$B269,B269)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R269)+(($R$6:$R$305=R269)*(ROW($B$6:$B$305)&lt;ROW(B269)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24128,7 +24118,7 @@
         <v/>
       </c>
       <c r="S270">
-        <f>IF(OR(B270="",COUNTIF($B$6:$B270,B270)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B270,$B$6:$B$305)=1)*($R$6:$R$305&gt;R270)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B270="",COUNTIF($B$6:$B270,B270)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R270)+(($R$6:$R$305=R270)*(ROW($B$6:$B$305)&lt;ROW(B270)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24150,7 +24140,7 @@
         <v/>
       </c>
       <c r="S271">
-        <f>IF(OR(B271="",COUNTIF($B$6:$B271,B271)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B271,$B$6:$B$305)=1)*($R$6:$R$305&gt;R271)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B271="",COUNTIF($B$6:$B271,B271)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R271)+(($R$6:$R$305=R271)*(ROW($B$6:$B$305)&lt;ROW(B271)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24172,7 +24162,7 @@
         <v/>
       </c>
       <c r="S272">
-        <f>IF(OR(B272="",COUNTIF($B$6:$B272,B272)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B272,$B$6:$B$305)=1)*($R$6:$R$305&gt;R272)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B272="",COUNTIF($B$6:$B272,B272)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R272)+(($R$6:$R$305=R272)*(ROW($B$6:$B$305)&lt;ROW(B272)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24194,7 +24184,7 @@
         <v/>
       </c>
       <c r="S273">
-        <f>IF(OR(B273="",COUNTIF($B$6:$B273,B273)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B273,$B$6:$B$305)=1)*($R$6:$R$305&gt;R273)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B273="",COUNTIF($B$6:$B273,B273)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R273)+(($R$6:$R$305=R273)*(ROW($B$6:$B$305)&lt;ROW(B273)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24216,7 +24206,7 @@
         <v/>
       </c>
       <c r="S274">
-        <f>IF(OR(B274="",COUNTIF($B$6:$B274,B274)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B274,$B$6:$B$305)=1)*($R$6:$R$305&gt;R274)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B274="",COUNTIF($B$6:$B274,B274)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R274)+(($R$6:$R$305=R274)*(ROW($B$6:$B$305)&lt;ROW(B274)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24238,7 +24228,7 @@
         <v/>
       </c>
       <c r="S275">
-        <f>IF(OR(B275="",COUNTIF($B$6:$B275,B275)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B275,$B$6:$B$305)=1)*($R$6:$R$305&gt;R275)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B275="",COUNTIF($B$6:$B275,B275)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R275)+(($R$6:$R$305=R275)*(ROW($B$6:$B$305)&lt;ROW(B275)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24260,7 +24250,7 @@
         <v/>
       </c>
       <c r="S276">
-        <f>IF(OR(B276="",COUNTIF($B$6:$B276,B276)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B276,$B$6:$B$305)=1)*($R$6:$R$305&gt;R276)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B276="",COUNTIF($B$6:$B276,B276)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R276)+(($R$6:$R$305=R276)*(ROW($B$6:$B$305)&lt;ROW(B276)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24282,7 +24272,7 @@
         <v/>
       </c>
       <c r="S277">
-        <f>IF(OR(B277="",COUNTIF($B$6:$B277,B277)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B277,$B$6:$B$305)=1)*($R$6:$R$305&gt;R277)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B277="",COUNTIF($B$6:$B277,B277)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R277)+(($R$6:$R$305=R277)*(ROW($B$6:$B$305)&lt;ROW(B277)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24304,7 +24294,7 @@
         <v/>
       </c>
       <c r="S278">
-        <f>IF(OR(B278="",COUNTIF($B$6:$B278,B278)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B278,$B$6:$B$305)=1)*($R$6:$R$305&gt;R278)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B278="",COUNTIF($B$6:$B278,B278)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R278)+(($R$6:$R$305=R278)*(ROW($B$6:$B$305)&lt;ROW(B278)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24326,7 +24316,7 @@
         <v/>
       </c>
       <c r="S279">
-        <f>IF(OR(B279="",COUNTIF($B$6:$B279,B279)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B279,$B$6:$B$305)=1)*($R$6:$R$305&gt;R279)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B279="",COUNTIF($B$6:$B279,B279)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R279)+(($R$6:$R$305=R279)*(ROW($B$6:$B$305)&lt;ROW(B279)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24348,7 +24338,7 @@
         <v/>
       </c>
       <c r="S280">
-        <f>IF(OR(B280="",COUNTIF($B$6:$B280,B280)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B280,$B$6:$B$305)=1)*($R$6:$R$305&gt;R280)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B280="",COUNTIF($B$6:$B280,B280)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R280)+(($R$6:$R$305=R280)*(ROW($B$6:$B$305)&lt;ROW(B280)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24370,7 +24360,7 @@
         <v/>
       </c>
       <c r="S281">
-        <f>IF(OR(B281="",COUNTIF($B$6:$B281,B281)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B281,$B$6:$B$305)=1)*($R$6:$R$305&gt;R281)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B281="",COUNTIF($B$6:$B281,B281)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R281)+(($R$6:$R$305=R281)*(ROW($B$6:$B$305)&lt;ROW(B281)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24392,7 +24382,7 @@
         <v/>
       </c>
       <c r="S282">
-        <f>IF(OR(B282="",COUNTIF($B$6:$B282,B282)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B282,$B$6:$B$305)=1)*($R$6:$R$305&gt;R282)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B282="",COUNTIF($B$6:$B282,B282)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R282)+(($R$6:$R$305=R282)*(ROW($B$6:$B$305)&lt;ROW(B282)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24414,7 +24404,7 @@
         <v/>
       </c>
       <c r="S283">
-        <f>IF(OR(B283="",COUNTIF($B$6:$B283,B283)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B283,$B$6:$B$305)=1)*($R$6:$R$305&gt;R283)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B283="",COUNTIF($B$6:$B283,B283)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R283)+(($R$6:$R$305=R283)*(ROW($B$6:$B$305)&lt;ROW(B283)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24436,7 +24426,7 @@
         <v/>
       </c>
       <c r="S284">
-        <f>IF(OR(B284="",COUNTIF($B$6:$B284,B284)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B284,$B$6:$B$305)=1)*($R$6:$R$305&gt;R284)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B284="",COUNTIF($B$6:$B284,B284)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R284)+(($R$6:$R$305=R284)*(ROW($B$6:$B$305)&lt;ROW(B284)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24458,7 +24448,7 @@
         <v/>
       </c>
       <c r="S285">
-        <f>IF(OR(B285="",COUNTIF($B$6:$B285,B285)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B285,$B$6:$B$305)=1)*($R$6:$R$305&gt;R285)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B285="",COUNTIF($B$6:$B285,B285)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R285)+(($R$6:$R$305=R285)*(ROW($B$6:$B$305)&lt;ROW(B285)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24480,7 +24470,7 @@
         <v/>
       </c>
       <c r="S286">
-        <f>IF(OR(B286="",COUNTIF($B$6:$B286,B286)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B286,$B$6:$B$305)=1)*($R$6:$R$305&gt;R286)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B286="",COUNTIF($B$6:$B286,B286)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R286)+(($R$6:$R$305=R286)*(ROW($B$6:$B$305)&lt;ROW(B286)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24502,7 +24492,7 @@
         <v/>
       </c>
       <c r="S287">
-        <f>IF(OR(B287="",COUNTIF($B$6:$B287,B287)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B287,$B$6:$B$305)=1)*($R$6:$R$305&gt;R287)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B287="",COUNTIF($B$6:$B287,B287)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R287)+(($R$6:$R$305=R287)*(ROW($B$6:$B$305)&lt;ROW(B287)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24524,7 +24514,7 @@
         <v/>
       </c>
       <c r="S288">
-        <f>IF(OR(B288="",COUNTIF($B$6:$B288,B288)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B288,$B$6:$B$305)=1)*($R$6:$R$305&gt;R288)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B288="",COUNTIF($B$6:$B288,B288)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R288)+(($R$6:$R$305=R288)*(ROW($B$6:$B$305)&lt;ROW(B288)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24546,7 +24536,7 @@
         <v/>
       </c>
       <c r="S289">
-        <f>IF(OR(B289="",COUNTIF($B$6:$B289,B289)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B289,$B$6:$B$305)=1)*($R$6:$R$305&gt;R289)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B289="",COUNTIF($B$6:$B289,B289)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R289)+(($R$6:$R$305=R289)*(ROW($B$6:$B$305)&lt;ROW(B289)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24568,7 +24558,7 @@
         <v/>
       </c>
       <c r="S290">
-        <f>IF(OR(B290="",COUNTIF($B$6:$B290,B290)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B290,$B$6:$B$305)=1)*($R$6:$R$305&gt;R290)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B290="",COUNTIF($B$6:$B290,B290)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R290)+(($R$6:$R$305=R290)*(ROW($B$6:$B$305)&lt;ROW(B290)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24590,7 +24580,7 @@
         <v/>
       </c>
       <c r="S291">
-        <f>IF(OR(B291="",COUNTIF($B$6:$B291,B291)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B291,$B$6:$B$305)=1)*($R$6:$R$305&gt;R291)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B291="",COUNTIF($B$6:$B291,B291)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R291)+(($R$6:$R$305=R291)*(ROW($B$6:$B$305)&lt;ROW(B291)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24612,7 +24602,7 @@
         <v/>
       </c>
       <c r="S292">
-        <f>IF(OR(B292="",COUNTIF($B$6:$B292,B292)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B292,$B$6:$B$305)=1)*($R$6:$R$305&gt;R292)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B292="",COUNTIF($B$6:$B292,B292)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R292)+(($R$6:$R$305=R292)*(ROW($B$6:$B$305)&lt;ROW(B292)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24634,7 +24624,7 @@
         <v/>
       </c>
       <c r="S293">
-        <f>IF(OR(B293="",COUNTIF($B$6:$B293,B293)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B293,$B$6:$B$305)=1)*($R$6:$R$305&gt;R293)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B293="",COUNTIF($B$6:$B293,B293)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R293)+(($R$6:$R$305=R293)*(ROW($B$6:$B$305)&lt;ROW(B293)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24656,7 +24646,7 @@
         <v/>
       </c>
       <c r="S294">
-        <f>IF(OR(B294="",COUNTIF($B$6:$B294,B294)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B294,$B$6:$B$305)=1)*($R$6:$R$305&gt;R294)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B294="",COUNTIF($B$6:$B294,B294)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R294)+(($R$6:$R$305=R294)*(ROW($B$6:$B$305)&lt;ROW(B294)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24678,7 +24668,7 @@
         <v/>
       </c>
       <c r="S295">
-        <f>IF(OR(B295="",COUNTIF($B$6:$B295,B295)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B295,$B$6:$B$305)=1)*($R$6:$R$305&gt;R295)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B295="",COUNTIF($B$6:$B295,B295)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R295)+(($R$6:$R$305=R295)*(ROW($B$6:$B$305)&lt;ROW(B295)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24700,7 +24690,7 @@
         <v/>
       </c>
       <c r="S296">
-        <f>IF(OR(B296="",COUNTIF($B$6:$B296,B296)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B296,$B$6:$B$305)=1)*($R$6:$R$305&gt;R296)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B296="",COUNTIF($B$6:$B296,B296)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R296)+(($R$6:$R$305=R296)*(ROW($B$6:$B$305)&lt;ROW(B296)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24722,7 +24712,7 @@
         <v/>
       </c>
       <c r="S297">
-        <f>IF(OR(B297="",COUNTIF($B$6:$B297,B297)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B297,$B$6:$B$305)=1)*($R$6:$R$305&gt;R297)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B297="",COUNTIF($B$6:$B297,B297)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R297)+(($R$6:$R$305=R297)*(ROW($B$6:$B$305)&lt;ROW(B297)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24744,7 +24734,7 @@
         <v/>
       </c>
       <c r="S298">
-        <f>IF(OR(B298="",COUNTIF($B$6:$B298,B298)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B298,$B$6:$B$305)=1)*($R$6:$R$305&gt;R298)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B298="",COUNTIF($B$6:$B298,B298)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R298)+(($R$6:$R$305=R298)*(ROW($B$6:$B$305)&lt;ROW(B298)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24766,7 +24756,7 @@
         <v/>
       </c>
       <c r="S299">
-        <f>IF(OR(B299="",COUNTIF($B$6:$B299,B299)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B299,$B$6:$B$305)=1)*($R$6:$R$305&gt;R299)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B299="",COUNTIF($B$6:$B299,B299)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R299)+(($R$6:$R$305=R299)*(ROW($B$6:$B$305)&lt;ROW(B299)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24788,7 +24778,7 @@
         <v/>
       </c>
       <c r="S300">
-        <f>IF(OR(B300="",COUNTIF($B$6:$B300,B300)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B300,$B$6:$B$305)=1)*($R$6:$R$305&gt;R300)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B300="",COUNTIF($B$6:$B300,B300)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R300)+(($R$6:$R$305=R300)*(ROW($B$6:$B$305)&lt;ROW(B300)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24810,7 +24800,7 @@
         <v/>
       </c>
       <c r="S301">
-        <f>IF(OR(B301="",COUNTIF($B$6:$B301,B301)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B301,$B$6:$B$305)=1)*($R$6:$R$305&gt;R301)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B301="",COUNTIF($B$6:$B301,B301)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R301)+(($R$6:$R$305=R301)*(ROW($B$6:$B$305)&lt;ROW(B301)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24832,7 +24822,7 @@
         <v/>
       </c>
       <c r="S302">
-        <f>IF(OR(B302="",COUNTIF($B$6:$B302,B302)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B302,$B$6:$B$305)=1)*($R$6:$R$305&gt;R302)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B302="",COUNTIF($B$6:$B302,B302)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R302)+(($R$6:$R$305=R302)*(ROW($B$6:$B$305)&lt;ROW(B302)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24854,7 +24844,7 @@
         <v/>
       </c>
       <c r="S303">
-        <f>IF(OR(B303="",COUNTIF($B$6:$B303,B303)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B303,$B$6:$B$305)=1)*($R$6:$R$305&gt;R303)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B303="",COUNTIF($B$6:$B303,B303)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R303)+(($R$6:$R$305=R303)*(ROW($B$6:$B$305)&lt;ROW(B303)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24876,7 +24866,7 @@
         <v/>
       </c>
       <c r="S304">
-        <f>IF(OR(B304="",COUNTIF($B$6:$B304,B304)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B304,$B$6:$B$305)=1)*($R$6:$R$305&gt;R304)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B304="",COUNTIF($B$6:$B304,B304)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R304)+(($R$6:$R$305=R304)*(ROW($B$6:$B$305)&lt;ROW(B304)))))+1)</f>
         <v/>
       </c>
     </row>
@@ -24898,7 +24888,7 @@
         <v/>
       </c>
       <c r="S305">
-        <f>IF(OR(B305="",COUNTIF($B$6:$B305,B305)&gt;1),"",SUMPRODUCT((COUNTIF($B$5:B305,$B$6:$B$305)=1)*($R$6:$R$305&gt;R305)*($B$6:$B$305&lt;&gt;""))+1)</f>
+        <f>IF(OR(B305="",COUNTIF($B$6:$B305,B305)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R305)+(($R$6:$R$305=R305)*(ROW($B$6:$B$305)&lt;ROW(B305)))))+1)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Golden Boot: use 1/COUNTIF for Excel-compatible unique ranking
</commit_message>
<xml_diff>
--- a/WorldCup2026_Sweepstake.xlsx
+++ b/WorldCup2026_Sweepstake.xlsx
@@ -15540,7 +15540,7 @@
         <v/>
       </c>
       <c r="S6">
-        <f>IF(OR(B6="",COUNTIF($B$6:$B6,B6)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R6)+(($R$6:$R$305=R6)*(ROW($B$6:$B$305)&lt;ROW(B6)))))+1)</f>
+        <f>IF(OR(B6="",COUNTIF($B$6:$B6,B6)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R6)+(($R$6:$R$305=R6)*($B$6:$B$305&lt;B6)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T6">
@@ -15608,7 +15608,7 @@
         <v/>
       </c>
       <c r="S7">
-        <f>IF(OR(B7="",COUNTIF($B$6:$B7,B7)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R7)+(($R$6:$R$305=R7)*(ROW($B$6:$B$305)&lt;ROW(B7)))))+1)</f>
+        <f>IF(OR(B7="",COUNTIF($B$6:$B7,B7)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R7)+(($R$6:$R$305=R7)*($B$6:$B$305&lt;B7)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T7">
@@ -15676,7 +15676,7 @@
         <v/>
       </c>
       <c r="S8">
-        <f>IF(OR(B8="",COUNTIF($B$6:$B8,B8)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R8)+(($R$6:$R$305=R8)*(ROW($B$6:$B$305)&lt;ROW(B8)))))+1)</f>
+        <f>IF(OR(B8="",COUNTIF($B$6:$B8,B8)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R8)+(($R$6:$R$305=R8)*($B$6:$B$305&lt;B8)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T8">
@@ -15744,7 +15744,7 @@
         <v/>
       </c>
       <c r="S9">
-        <f>IF(OR(B9="",COUNTIF($B$6:$B9,B9)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R9)+(($R$6:$R$305=R9)*(ROW($B$6:$B$305)&lt;ROW(B9)))))+1)</f>
+        <f>IF(OR(B9="",COUNTIF($B$6:$B9,B9)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R9)+(($R$6:$R$305=R9)*($B$6:$B$305&lt;B9)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T9">
@@ -15812,7 +15812,7 @@
         <v/>
       </c>
       <c r="S10">
-        <f>IF(OR(B10="",COUNTIF($B$6:$B10,B10)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R10)+(($R$6:$R$305=R10)*(ROW($B$6:$B$305)&lt;ROW(B10)))))+1)</f>
+        <f>IF(OR(B10="",COUNTIF($B$6:$B10,B10)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R10)+(($R$6:$R$305=R10)*($B$6:$B$305&lt;B10)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T10">
@@ -15880,7 +15880,7 @@
         <v/>
       </c>
       <c r="S11">
-        <f>IF(OR(B11="",COUNTIF($B$6:$B11,B11)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R11)+(($R$6:$R$305=R11)*(ROW($B$6:$B$305)&lt;ROW(B11)))))+1)</f>
+        <f>IF(OR(B11="",COUNTIF($B$6:$B11,B11)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R11)+(($R$6:$R$305=R11)*($B$6:$B$305&lt;B11)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T11">
@@ -15948,7 +15948,7 @@
         <v/>
       </c>
       <c r="S12">
-        <f>IF(OR(B12="",COUNTIF($B$6:$B12,B12)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R12)+(($R$6:$R$305=R12)*(ROW($B$6:$B$305)&lt;ROW(B12)))))+1)</f>
+        <f>IF(OR(B12="",COUNTIF($B$6:$B12,B12)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R12)+(($R$6:$R$305=R12)*($B$6:$B$305&lt;B12)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T12">
@@ -16016,7 +16016,7 @@
         <v/>
       </c>
       <c r="S13">
-        <f>IF(OR(B13="",COUNTIF($B$6:$B13,B13)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R13)+(($R$6:$R$305=R13)*(ROW($B$6:$B$305)&lt;ROW(B13)))))+1)</f>
+        <f>IF(OR(B13="",COUNTIF($B$6:$B13,B13)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R13)+(($R$6:$R$305=R13)*($B$6:$B$305&lt;B13)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T13">
@@ -16084,7 +16084,7 @@
         <v/>
       </c>
       <c r="S14">
-        <f>IF(OR(B14="",COUNTIF($B$6:$B14,B14)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R14)+(($R$6:$R$305=R14)*(ROW($B$6:$B$305)&lt;ROW(B14)))))+1)</f>
+        <f>IF(OR(B14="",COUNTIF($B$6:$B14,B14)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R14)+(($R$6:$R$305=R14)*($B$6:$B$305&lt;B14)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T14">
@@ -16152,7 +16152,7 @@
         <v/>
       </c>
       <c r="S15">
-        <f>IF(OR(B15="",COUNTIF($B$6:$B15,B15)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R15)+(($R$6:$R$305=R15)*(ROW($B$6:$B$305)&lt;ROW(B15)))))+1)</f>
+        <f>IF(OR(B15="",COUNTIF($B$6:$B15,B15)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R15)+(($R$6:$R$305=R15)*($B$6:$B$305&lt;B15)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T15">
@@ -16220,7 +16220,7 @@
         <v/>
       </c>
       <c r="S16">
-        <f>IF(OR(B16="",COUNTIF($B$6:$B16,B16)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R16)+(($R$6:$R$305=R16)*(ROW($B$6:$B$305)&lt;ROW(B16)))))+1)</f>
+        <f>IF(OR(B16="",COUNTIF($B$6:$B16,B16)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R16)+(($R$6:$R$305=R16)*($B$6:$B$305&lt;B16)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T16">
@@ -16288,7 +16288,7 @@
         <v/>
       </c>
       <c r="S17">
-        <f>IF(OR(B17="",COUNTIF($B$6:$B17,B17)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R17)+(($R$6:$R$305=R17)*(ROW($B$6:$B$305)&lt;ROW(B17)))))+1)</f>
+        <f>IF(OR(B17="",COUNTIF($B$6:$B17,B17)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R17)+(($R$6:$R$305=R17)*($B$6:$B$305&lt;B17)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T17">
@@ -16356,7 +16356,7 @@
         <v/>
       </c>
       <c r="S18">
-        <f>IF(OR(B18="",COUNTIF($B$6:$B18,B18)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R18)+(($R$6:$R$305=R18)*(ROW($B$6:$B$305)&lt;ROW(B18)))))+1)</f>
+        <f>IF(OR(B18="",COUNTIF($B$6:$B18,B18)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R18)+(($R$6:$R$305=R18)*($B$6:$B$305&lt;B18)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T18">
@@ -16424,7 +16424,7 @@
         <v/>
       </c>
       <c r="S19">
-        <f>IF(OR(B19="",COUNTIF($B$6:$B19,B19)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R19)+(($R$6:$R$305=R19)*(ROW($B$6:$B$305)&lt;ROW(B19)))))+1)</f>
+        <f>IF(OR(B19="",COUNTIF($B$6:$B19,B19)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R19)+(($R$6:$R$305=R19)*($B$6:$B$305&lt;B19)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T19">
@@ -16492,7 +16492,7 @@
         <v/>
       </c>
       <c r="S20">
-        <f>IF(OR(B20="",COUNTIF($B$6:$B20,B20)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R20)+(($R$6:$R$305=R20)*(ROW($B$6:$B$305)&lt;ROW(B20)))))+1)</f>
+        <f>IF(OR(B20="",COUNTIF($B$6:$B20,B20)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R20)+(($R$6:$R$305=R20)*($B$6:$B$305&lt;B20)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T20">
@@ -16560,7 +16560,7 @@
         <v/>
       </c>
       <c r="S21">
-        <f>IF(OR(B21="",COUNTIF($B$6:$B21,B21)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R21)+(($R$6:$R$305=R21)*(ROW($B$6:$B$305)&lt;ROW(B21)))))+1)</f>
+        <f>IF(OR(B21="",COUNTIF($B$6:$B21,B21)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R21)+(($R$6:$R$305=R21)*($B$6:$B$305&lt;B21)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T21">
@@ -16628,7 +16628,7 @@
         <v/>
       </c>
       <c r="S22">
-        <f>IF(OR(B22="",COUNTIF($B$6:$B22,B22)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R22)+(($R$6:$R$305=R22)*(ROW($B$6:$B$305)&lt;ROW(B22)))))+1)</f>
+        <f>IF(OR(B22="",COUNTIF($B$6:$B22,B22)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R22)+(($R$6:$R$305=R22)*($B$6:$B$305&lt;B22)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T22">
@@ -16696,7 +16696,7 @@
         <v/>
       </c>
       <c r="S23">
-        <f>IF(OR(B23="",COUNTIF($B$6:$B23,B23)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R23)+(($R$6:$R$305=R23)*(ROW($B$6:$B$305)&lt;ROW(B23)))))+1)</f>
+        <f>IF(OR(B23="",COUNTIF($B$6:$B23,B23)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R23)+(($R$6:$R$305=R23)*($B$6:$B$305&lt;B23)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T23">
@@ -16764,7 +16764,7 @@
         <v/>
       </c>
       <c r="S24">
-        <f>IF(OR(B24="",COUNTIF($B$6:$B24,B24)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R24)+(($R$6:$R$305=R24)*(ROW($B$6:$B$305)&lt;ROW(B24)))))+1)</f>
+        <f>IF(OR(B24="",COUNTIF($B$6:$B24,B24)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R24)+(($R$6:$R$305=R24)*($B$6:$B$305&lt;B24)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T24">
@@ -16832,7 +16832,7 @@
         <v/>
       </c>
       <c r="S25">
-        <f>IF(OR(B25="",COUNTIF($B$6:$B25,B25)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R25)+(($R$6:$R$305=R25)*(ROW($B$6:$B$305)&lt;ROW(B25)))))+1)</f>
+        <f>IF(OR(B25="",COUNTIF($B$6:$B25,B25)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R25)+(($R$6:$R$305=R25)*($B$6:$B$305&lt;B25)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T25">
@@ -16900,7 +16900,7 @@
         <v/>
       </c>
       <c r="S26">
-        <f>IF(OR(B26="",COUNTIF($B$6:$B26,B26)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R26)+(($R$6:$R$305=R26)*(ROW($B$6:$B$305)&lt;ROW(B26)))))+1)</f>
+        <f>IF(OR(B26="",COUNTIF($B$6:$B26,B26)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R26)+(($R$6:$R$305=R26)*($B$6:$B$305&lt;B26)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T26">
@@ -16968,7 +16968,7 @@
         <v/>
       </c>
       <c r="S27">
-        <f>IF(OR(B27="",COUNTIF($B$6:$B27,B27)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R27)+(($R$6:$R$305=R27)*(ROW($B$6:$B$305)&lt;ROW(B27)))))+1)</f>
+        <f>IF(OR(B27="",COUNTIF($B$6:$B27,B27)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R27)+(($R$6:$R$305=R27)*($B$6:$B$305&lt;B27)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T27">
@@ -17036,7 +17036,7 @@
         <v/>
       </c>
       <c r="S28">
-        <f>IF(OR(B28="",COUNTIF($B$6:$B28,B28)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R28)+(($R$6:$R$305=R28)*(ROW($B$6:$B$305)&lt;ROW(B28)))))+1)</f>
+        <f>IF(OR(B28="",COUNTIF($B$6:$B28,B28)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R28)+(($R$6:$R$305=R28)*($B$6:$B$305&lt;B28)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T28">
@@ -17104,7 +17104,7 @@
         <v/>
       </c>
       <c r="S29">
-        <f>IF(OR(B29="",COUNTIF($B$6:$B29,B29)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R29)+(($R$6:$R$305=R29)*(ROW($B$6:$B$305)&lt;ROW(B29)))))+1)</f>
+        <f>IF(OR(B29="",COUNTIF($B$6:$B29,B29)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R29)+(($R$6:$R$305=R29)*($B$6:$B$305&lt;B29)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T29">
@@ -17172,7 +17172,7 @@
         <v/>
       </c>
       <c r="S30">
-        <f>IF(OR(B30="",COUNTIF($B$6:$B30,B30)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R30)+(($R$6:$R$305=R30)*(ROW($B$6:$B$305)&lt;ROW(B30)))))+1)</f>
+        <f>IF(OR(B30="",COUNTIF($B$6:$B30,B30)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R30)+(($R$6:$R$305=R30)*($B$6:$B$305&lt;B30)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T30">
@@ -17240,7 +17240,7 @@
         <v/>
       </c>
       <c r="S31">
-        <f>IF(OR(B31="",COUNTIF($B$6:$B31,B31)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R31)+(($R$6:$R$305=R31)*(ROW($B$6:$B$305)&lt;ROW(B31)))))+1)</f>
+        <f>IF(OR(B31="",COUNTIF($B$6:$B31,B31)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R31)+(($R$6:$R$305=R31)*($B$6:$B$305&lt;B31)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T31">
@@ -17308,7 +17308,7 @@
         <v/>
       </c>
       <c r="S32">
-        <f>IF(OR(B32="",COUNTIF($B$6:$B32,B32)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R32)+(($R$6:$R$305=R32)*(ROW($B$6:$B$305)&lt;ROW(B32)))))+1)</f>
+        <f>IF(OR(B32="",COUNTIF($B$6:$B32,B32)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R32)+(($R$6:$R$305=R32)*($B$6:$B$305&lt;B32)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T32">
@@ -17376,7 +17376,7 @@
         <v/>
       </c>
       <c r="S33">
-        <f>IF(OR(B33="",COUNTIF($B$6:$B33,B33)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R33)+(($R$6:$R$305=R33)*(ROW($B$6:$B$305)&lt;ROW(B33)))))+1)</f>
+        <f>IF(OR(B33="",COUNTIF($B$6:$B33,B33)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R33)+(($R$6:$R$305=R33)*($B$6:$B$305&lt;B33)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T33">
@@ -17444,7 +17444,7 @@
         <v/>
       </c>
       <c r="S34">
-        <f>IF(OR(B34="",COUNTIF($B$6:$B34,B34)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R34)+(($R$6:$R$305=R34)*(ROW($B$6:$B$305)&lt;ROW(B34)))))+1)</f>
+        <f>IF(OR(B34="",COUNTIF($B$6:$B34,B34)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R34)+(($R$6:$R$305=R34)*($B$6:$B$305&lt;B34)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T34">
@@ -17512,7 +17512,7 @@
         <v/>
       </c>
       <c r="S35">
-        <f>IF(OR(B35="",COUNTIF($B$6:$B35,B35)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R35)+(($R$6:$R$305=R35)*(ROW($B$6:$B$305)&lt;ROW(B35)))))+1)</f>
+        <f>IF(OR(B35="",COUNTIF($B$6:$B35,B35)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R35)+(($R$6:$R$305=R35)*($B$6:$B$305&lt;B35)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T35">
@@ -17565,7 +17565,7 @@
         <v/>
       </c>
       <c r="S36">
-        <f>IF(OR(B36="",COUNTIF($B$6:$B36,B36)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R36)+(($R$6:$R$305=R36)*(ROW($B$6:$B$305)&lt;ROW(B36)))))+1)</f>
+        <f>IF(OR(B36="",COUNTIF($B$6:$B36,B36)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R36)+(($R$6:$R$305=R36)*($B$6:$B$305&lt;B36)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T36">
@@ -17618,7 +17618,7 @@
         <v/>
       </c>
       <c r="S37">
-        <f>IF(OR(B37="",COUNTIF($B$6:$B37,B37)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R37)+(($R$6:$R$305=R37)*(ROW($B$6:$B$305)&lt;ROW(B37)))))+1)</f>
+        <f>IF(OR(B37="",COUNTIF($B$6:$B37,B37)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R37)+(($R$6:$R$305=R37)*($B$6:$B$305&lt;B37)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T37">
@@ -17671,7 +17671,7 @@
         <v/>
       </c>
       <c r="S38">
-        <f>IF(OR(B38="",COUNTIF($B$6:$B38,B38)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R38)+(($R$6:$R$305=R38)*(ROW($B$6:$B$305)&lt;ROW(B38)))))+1)</f>
+        <f>IF(OR(B38="",COUNTIF($B$6:$B38,B38)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R38)+(($R$6:$R$305=R38)*($B$6:$B$305&lt;B38)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T38">
@@ -17724,7 +17724,7 @@
         <v/>
       </c>
       <c r="S39">
-        <f>IF(OR(B39="",COUNTIF($B$6:$B39,B39)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R39)+(($R$6:$R$305=R39)*(ROW($B$6:$B$305)&lt;ROW(B39)))))+1)</f>
+        <f>IF(OR(B39="",COUNTIF($B$6:$B39,B39)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R39)+(($R$6:$R$305=R39)*($B$6:$B$305&lt;B39)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T39">
@@ -17777,7 +17777,7 @@
         <v/>
       </c>
       <c r="S40">
-        <f>IF(OR(B40="",COUNTIF($B$6:$B40,B40)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R40)+(($R$6:$R$305=R40)*(ROW($B$6:$B$305)&lt;ROW(B40)))))+1)</f>
+        <f>IF(OR(B40="",COUNTIF($B$6:$B40,B40)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R40)+(($R$6:$R$305=R40)*($B$6:$B$305&lt;B40)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T40">
@@ -17830,7 +17830,7 @@
         <v/>
       </c>
       <c r="S41">
-        <f>IF(OR(B41="",COUNTIF($B$6:$B41,B41)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R41)+(($R$6:$R$305=R41)*(ROW($B$6:$B$305)&lt;ROW(B41)))))+1)</f>
+        <f>IF(OR(B41="",COUNTIF($B$6:$B41,B41)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R41)+(($R$6:$R$305=R41)*($B$6:$B$305&lt;B41)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T41">
@@ -17883,7 +17883,7 @@
         <v/>
       </c>
       <c r="S42">
-        <f>IF(OR(B42="",COUNTIF($B$6:$B42,B42)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R42)+(($R$6:$R$305=R42)*(ROW($B$6:$B$305)&lt;ROW(B42)))))+1)</f>
+        <f>IF(OR(B42="",COUNTIF($B$6:$B42,B42)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R42)+(($R$6:$R$305=R42)*($B$6:$B$305&lt;B42)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T42">
@@ -17936,7 +17936,7 @@
         <v/>
       </c>
       <c r="S43">
-        <f>IF(OR(B43="",COUNTIF($B$6:$B43,B43)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R43)+(($R$6:$R$305=R43)*(ROW($B$6:$B$305)&lt;ROW(B43)))))+1)</f>
+        <f>IF(OR(B43="",COUNTIF($B$6:$B43,B43)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R43)+(($R$6:$R$305=R43)*($B$6:$B$305&lt;B43)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T43">
@@ -17989,7 +17989,7 @@
         <v/>
       </c>
       <c r="S44">
-        <f>IF(OR(B44="",COUNTIF($B$6:$B44,B44)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R44)+(($R$6:$R$305=R44)*(ROW($B$6:$B$305)&lt;ROW(B44)))))+1)</f>
+        <f>IF(OR(B44="",COUNTIF($B$6:$B44,B44)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R44)+(($R$6:$R$305=R44)*($B$6:$B$305&lt;B44)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T44">
@@ -18042,7 +18042,7 @@
         <v/>
       </c>
       <c r="S45">
-        <f>IF(OR(B45="",COUNTIF($B$6:$B45,B45)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R45)+(($R$6:$R$305=R45)*(ROW($B$6:$B$305)&lt;ROW(B45)))))+1)</f>
+        <f>IF(OR(B45="",COUNTIF($B$6:$B45,B45)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R45)+(($R$6:$R$305=R45)*($B$6:$B$305&lt;B45)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T45">
@@ -18095,7 +18095,7 @@
         <v/>
       </c>
       <c r="S46">
-        <f>IF(OR(B46="",COUNTIF($B$6:$B46,B46)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R46)+(($R$6:$R$305=R46)*(ROW($B$6:$B$305)&lt;ROW(B46)))))+1)</f>
+        <f>IF(OR(B46="",COUNTIF($B$6:$B46,B46)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R46)+(($R$6:$R$305=R46)*($B$6:$B$305&lt;B46)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T46">
@@ -18148,7 +18148,7 @@
         <v/>
       </c>
       <c r="S47">
-        <f>IF(OR(B47="",COUNTIF($B$6:$B47,B47)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R47)+(($R$6:$R$305=R47)*(ROW($B$6:$B$305)&lt;ROW(B47)))))+1)</f>
+        <f>IF(OR(B47="",COUNTIF($B$6:$B47,B47)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R47)+(($R$6:$R$305=R47)*($B$6:$B$305&lt;B47)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T47">
@@ -18201,7 +18201,7 @@
         <v/>
       </c>
       <c r="S48">
-        <f>IF(OR(B48="",COUNTIF($B$6:$B48,B48)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R48)+(($R$6:$R$305=R48)*(ROW($B$6:$B$305)&lt;ROW(B48)))))+1)</f>
+        <f>IF(OR(B48="",COUNTIF($B$6:$B48,B48)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R48)+(($R$6:$R$305=R48)*($B$6:$B$305&lt;B48)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T48">
@@ -18254,7 +18254,7 @@
         <v/>
       </c>
       <c r="S49">
-        <f>IF(OR(B49="",COUNTIF($B$6:$B49,B49)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R49)+(($R$6:$R$305=R49)*(ROW($B$6:$B$305)&lt;ROW(B49)))))+1)</f>
+        <f>IF(OR(B49="",COUNTIF($B$6:$B49,B49)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R49)+(($R$6:$R$305=R49)*($B$6:$B$305&lt;B49)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T49">
@@ -18307,7 +18307,7 @@
         <v/>
       </c>
       <c r="S50">
-        <f>IF(OR(B50="",COUNTIF($B$6:$B50,B50)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R50)+(($R$6:$R$305=R50)*(ROW($B$6:$B$305)&lt;ROW(B50)))))+1)</f>
+        <f>IF(OR(B50="",COUNTIF($B$6:$B50,B50)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R50)+(($R$6:$R$305=R50)*($B$6:$B$305&lt;B50)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T50">
@@ -18360,7 +18360,7 @@
         <v/>
       </c>
       <c r="S51">
-        <f>IF(OR(B51="",COUNTIF($B$6:$B51,B51)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R51)+(($R$6:$R$305=R51)*(ROW($B$6:$B$305)&lt;ROW(B51)))))+1)</f>
+        <f>IF(OR(B51="",COUNTIF($B$6:$B51,B51)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R51)+(($R$6:$R$305=R51)*($B$6:$B$305&lt;B51)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T51">
@@ -18413,7 +18413,7 @@
         <v/>
       </c>
       <c r="S52">
-        <f>IF(OR(B52="",COUNTIF($B$6:$B52,B52)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R52)+(($R$6:$R$305=R52)*(ROW($B$6:$B$305)&lt;ROW(B52)))))+1)</f>
+        <f>IF(OR(B52="",COUNTIF($B$6:$B52,B52)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R52)+(($R$6:$R$305=R52)*($B$6:$B$305&lt;B52)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T52">
@@ -18466,7 +18466,7 @@
         <v/>
       </c>
       <c r="S53">
-        <f>IF(OR(B53="",COUNTIF($B$6:$B53,B53)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R53)+(($R$6:$R$305=R53)*(ROW($B$6:$B$305)&lt;ROW(B53)))))+1)</f>
+        <f>IF(OR(B53="",COUNTIF($B$6:$B53,B53)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R53)+(($R$6:$R$305=R53)*($B$6:$B$305&lt;B53)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T53">
@@ -18519,7 +18519,7 @@
         <v/>
       </c>
       <c r="S54">
-        <f>IF(OR(B54="",COUNTIF($B$6:$B54,B54)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R54)+(($R$6:$R$305=R54)*(ROW($B$6:$B$305)&lt;ROW(B54)))))+1)</f>
+        <f>IF(OR(B54="",COUNTIF($B$6:$B54,B54)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R54)+(($R$6:$R$305=R54)*($B$6:$B$305&lt;B54)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T54">
@@ -18572,7 +18572,7 @@
         <v/>
       </c>
       <c r="S55">
-        <f>IF(OR(B55="",COUNTIF($B$6:$B55,B55)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R55)+(($R$6:$R$305=R55)*(ROW($B$6:$B$305)&lt;ROW(B55)))))+1)</f>
+        <f>IF(OR(B55="",COUNTIF($B$6:$B55,B55)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R55)+(($R$6:$R$305=R55)*($B$6:$B$305&lt;B55)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T55">
@@ -18610,7 +18610,7 @@
         <v/>
       </c>
       <c r="S56">
-        <f>IF(OR(B56="",COUNTIF($B$6:$B56,B56)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R56)+(($R$6:$R$305=R56)*(ROW($B$6:$B$305)&lt;ROW(B56)))))+1)</f>
+        <f>IF(OR(B56="",COUNTIF($B$6:$B56,B56)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R56)+(($R$6:$R$305=R56)*($B$6:$B$305&lt;B56)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T56">
@@ -18648,7 +18648,7 @@
         <v/>
       </c>
       <c r="S57">
-        <f>IF(OR(B57="",COUNTIF($B$6:$B57,B57)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R57)+(($R$6:$R$305=R57)*(ROW($B$6:$B$305)&lt;ROW(B57)))))+1)</f>
+        <f>IF(OR(B57="",COUNTIF($B$6:$B57,B57)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R57)+(($R$6:$R$305=R57)*($B$6:$B$305&lt;B57)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T57">
@@ -18686,7 +18686,7 @@
         <v/>
       </c>
       <c r="S58">
-        <f>IF(OR(B58="",COUNTIF($B$6:$B58,B58)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R58)+(($R$6:$R$305=R58)*(ROW($B$6:$B$305)&lt;ROW(B58)))))+1)</f>
+        <f>IF(OR(B58="",COUNTIF($B$6:$B58,B58)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R58)+(($R$6:$R$305=R58)*($B$6:$B$305&lt;B58)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T58">
@@ -18724,7 +18724,7 @@
         <v/>
       </c>
       <c r="S59">
-        <f>IF(OR(B59="",COUNTIF($B$6:$B59,B59)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R59)+(($R$6:$R$305=R59)*(ROW($B$6:$B$305)&lt;ROW(B59)))))+1)</f>
+        <f>IF(OR(B59="",COUNTIF($B$6:$B59,B59)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R59)+(($R$6:$R$305=R59)*($B$6:$B$305&lt;B59)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T59">
@@ -18762,7 +18762,7 @@
         <v/>
       </c>
       <c r="S60">
-        <f>IF(OR(B60="",COUNTIF($B$6:$B60,B60)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R60)+(($R$6:$R$305=R60)*(ROW($B$6:$B$305)&lt;ROW(B60)))))+1)</f>
+        <f>IF(OR(B60="",COUNTIF($B$6:$B60,B60)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R60)+(($R$6:$R$305=R60)*($B$6:$B$305&lt;B60)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T60">
@@ -18800,7 +18800,7 @@
         <v/>
       </c>
       <c r="S61">
-        <f>IF(OR(B61="",COUNTIF($B$6:$B61,B61)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R61)+(($R$6:$R$305=R61)*(ROW($B$6:$B$305)&lt;ROW(B61)))))+1)</f>
+        <f>IF(OR(B61="",COUNTIF($B$6:$B61,B61)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R61)+(($R$6:$R$305=R61)*($B$6:$B$305&lt;B61)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T61">
@@ -18838,7 +18838,7 @@
         <v/>
       </c>
       <c r="S62">
-        <f>IF(OR(B62="",COUNTIF($B$6:$B62,B62)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R62)+(($R$6:$R$305=R62)*(ROW($B$6:$B$305)&lt;ROW(B62)))))+1)</f>
+        <f>IF(OR(B62="",COUNTIF($B$6:$B62,B62)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R62)+(($R$6:$R$305=R62)*($B$6:$B$305&lt;B62)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T62">
@@ -18876,7 +18876,7 @@
         <v/>
       </c>
       <c r="S63">
-        <f>IF(OR(B63="",COUNTIF($B$6:$B63,B63)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R63)+(($R$6:$R$305=R63)*(ROW($B$6:$B$305)&lt;ROW(B63)))))+1)</f>
+        <f>IF(OR(B63="",COUNTIF($B$6:$B63,B63)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R63)+(($R$6:$R$305=R63)*($B$6:$B$305&lt;B63)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T63">
@@ -18914,7 +18914,7 @@
         <v/>
       </c>
       <c r="S64">
-        <f>IF(OR(B64="",COUNTIF($B$6:$B64,B64)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R64)+(($R$6:$R$305=R64)*(ROW($B$6:$B$305)&lt;ROW(B64)))))+1)</f>
+        <f>IF(OR(B64="",COUNTIF($B$6:$B64,B64)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R64)+(($R$6:$R$305=R64)*($B$6:$B$305&lt;B64)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T64">
@@ -18952,7 +18952,7 @@
         <v/>
       </c>
       <c r="S65">
-        <f>IF(OR(B65="",COUNTIF($B$6:$B65,B65)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R65)+(($R$6:$R$305=R65)*(ROW($B$6:$B$305)&lt;ROW(B65)))))+1)</f>
+        <f>IF(OR(B65="",COUNTIF($B$6:$B65,B65)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R65)+(($R$6:$R$305=R65)*($B$6:$B$305&lt;B65)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T65">
@@ -18990,7 +18990,7 @@
         <v/>
       </c>
       <c r="S66">
-        <f>IF(OR(B66="",COUNTIF($B$6:$B66,B66)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R66)+(($R$6:$R$305=R66)*(ROW($B$6:$B$305)&lt;ROW(B66)))))+1)</f>
+        <f>IF(OR(B66="",COUNTIF($B$6:$B66,B66)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R66)+(($R$6:$R$305=R66)*($B$6:$B$305&lt;B66)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T66">
@@ -19028,7 +19028,7 @@
         <v/>
       </c>
       <c r="S67">
-        <f>IF(OR(B67="",COUNTIF($B$6:$B67,B67)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R67)+(($R$6:$R$305=R67)*(ROW($B$6:$B$305)&lt;ROW(B67)))))+1)</f>
+        <f>IF(OR(B67="",COUNTIF($B$6:$B67,B67)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R67)+(($R$6:$R$305=R67)*($B$6:$B$305&lt;B67)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T67">
@@ -19066,7 +19066,7 @@
         <v/>
       </c>
       <c r="S68">
-        <f>IF(OR(B68="",COUNTIF($B$6:$B68,B68)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R68)+(($R$6:$R$305=R68)*(ROW($B$6:$B$305)&lt;ROW(B68)))))+1)</f>
+        <f>IF(OR(B68="",COUNTIF($B$6:$B68,B68)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R68)+(($R$6:$R$305=R68)*($B$6:$B$305&lt;B68)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T68">
@@ -19104,7 +19104,7 @@
         <v/>
       </c>
       <c r="S69">
-        <f>IF(OR(B69="",COUNTIF($B$6:$B69,B69)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R69)+(($R$6:$R$305=R69)*(ROW($B$6:$B$305)&lt;ROW(B69)))))+1)</f>
+        <f>IF(OR(B69="",COUNTIF($B$6:$B69,B69)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R69)+(($R$6:$R$305=R69)*($B$6:$B$305&lt;B69)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T69">
@@ -19142,7 +19142,7 @@
         <v/>
       </c>
       <c r="S70">
-        <f>IF(OR(B70="",COUNTIF($B$6:$B70,B70)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R70)+(($R$6:$R$305=R70)*(ROW($B$6:$B$305)&lt;ROW(B70)))))+1)</f>
+        <f>IF(OR(B70="",COUNTIF($B$6:$B70,B70)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R70)+(($R$6:$R$305=R70)*($B$6:$B$305&lt;B70)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T70">
@@ -19180,7 +19180,7 @@
         <v/>
       </c>
       <c r="S71">
-        <f>IF(OR(B71="",COUNTIF($B$6:$B71,B71)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R71)+(($R$6:$R$305=R71)*(ROW($B$6:$B$305)&lt;ROW(B71)))))+1)</f>
+        <f>IF(OR(B71="",COUNTIF($B$6:$B71,B71)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R71)+(($R$6:$R$305=R71)*($B$6:$B$305&lt;B71)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T71">
@@ -19218,7 +19218,7 @@
         <v/>
       </c>
       <c r="S72">
-        <f>IF(OR(B72="",COUNTIF($B$6:$B72,B72)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R72)+(($R$6:$R$305=R72)*(ROW($B$6:$B$305)&lt;ROW(B72)))))+1)</f>
+        <f>IF(OR(B72="",COUNTIF($B$6:$B72,B72)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R72)+(($R$6:$R$305=R72)*($B$6:$B$305&lt;B72)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T72">
@@ -19256,7 +19256,7 @@
         <v/>
       </c>
       <c r="S73">
-        <f>IF(OR(B73="",COUNTIF($B$6:$B73,B73)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R73)+(($R$6:$R$305=R73)*(ROW($B$6:$B$305)&lt;ROW(B73)))))+1)</f>
+        <f>IF(OR(B73="",COUNTIF($B$6:$B73,B73)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R73)+(($R$6:$R$305=R73)*($B$6:$B$305&lt;B73)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T73">
@@ -19294,7 +19294,7 @@
         <v/>
       </c>
       <c r="S74">
-        <f>IF(OR(B74="",COUNTIF($B$6:$B74,B74)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R74)+(($R$6:$R$305=R74)*(ROW($B$6:$B$305)&lt;ROW(B74)))))+1)</f>
+        <f>IF(OR(B74="",COUNTIF($B$6:$B74,B74)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R74)+(($R$6:$R$305=R74)*($B$6:$B$305&lt;B74)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T74">
@@ -19332,7 +19332,7 @@
         <v/>
       </c>
       <c r="S75">
-        <f>IF(OR(B75="",COUNTIF($B$6:$B75,B75)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R75)+(($R$6:$R$305=R75)*(ROW($B$6:$B$305)&lt;ROW(B75)))))+1)</f>
+        <f>IF(OR(B75="",COUNTIF($B$6:$B75,B75)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R75)+(($R$6:$R$305=R75)*($B$6:$B$305&lt;B75)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T75">
@@ -19370,7 +19370,7 @@
         <v/>
       </c>
       <c r="S76">
-        <f>IF(OR(B76="",COUNTIF($B$6:$B76,B76)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R76)+(($R$6:$R$305=R76)*(ROW($B$6:$B$305)&lt;ROW(B76)))))+1)</f>
+        <f>IF(OR(B76="",COUNTIF($B$6:$B76,B76)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R76)+(($R$6:$R$305=R76)*($B$6:$B$305&lt;B76)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T76">
@@ -19408,7 +19408,7 @@
         <v/>
       </c>
       <c r="S77">
-        <f>IF(OR(B77="",COUNTIF($B$6:$B77,B77)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R77)+(($R$6:$R$305=R77)*(ROW($B$6:$B$305)&lt;ROW(B77)))))+1)</f>
+        <f>IF(OR(B77="",COUNTIF($B$6:$B77,B77)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R77)+(($R$6:$R$305=R77)*($B$6:$B$305&lt;B77)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T77">
@@ -19446,7 +19446,7 @@
         <v/>
       </c>
       <c r="S78">
-        <f>IF(OR(B78="",COUNTIF($B$6:$B78,B78)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R78)+(($R$6:$R$305=R78)*(ROW($B$6:$B$305)&lt;ROW(B78)))))+1)</f>
+        <f>IF(OR(B78="",COUNTIF($B$6:$B78,B78)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R78)+(($R$6:$R$305=R78)*($B$6:$B$305&lt;B78)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T78">
@@ -19484,7 +19484,7 @@
         <v/>
       </c>
       <c r="S79">
-        <f>IF(OR(B79="",COUNTIF($B$6:$B79,B79)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R79)+(($R$6:$R$305=R79)*(ROW($B$6:$B$305)&lt;ROW(B79)))))+1)</f>
+        <f>IF(OR(B79="",COUNTIF($B$6:$B79,B79)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R79)+(($R$6:$R$305=R79)*($B$6:$B$305&lt;B79)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T79">
@@ -19522,7 +19522,7 @@
         <v/>
       </c>
       <c r="S80">
-        <f>IF(OR(B80="",COUNTIF($B$6:$B80,B80)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R80)+(($R$6:$R$305=R80)*(ROW($B$6:$B$305)&lt;ROW(B80)))))+1)</f>
+        <f>IF(OR(B80="",COUNTIF($B$6:$B80,B80)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R80)+(($R$6:$R$305=R80)*($B$6:$B$305&lt;B80)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T80">
@@ -19560,7 +19560,7 @@
         <v/>
       </c>
       <c r="S81">
-        <f>IF(OR(B81="",COUNTIF($B$6:$B81,B81)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R81)+(($R$6:$R$305=R81)*(ROW($B$6:$B$305)&lt;ROW(B81)))))+1)</f>
+        <f>IF(OR(B81="",COUNTIF($B$6:$B81,B81)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R81)+(($R$6:$R$305=R81)*($B$6:$B$305&lt;B81)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T81">
@@ -19598,7 +19598,7 @@
         <v/>
       </c>
       <c r="S82">
-        <f>IF(OR(B82="",COUNTIF($B$6:$B82,B82)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R82)+(($R$6:$R$305=R82)*(ROW($B$6:$B$305)&lt;ROW(B82)))))+1)</f>
+        <f>IF(OR(B82="",COUNTIF($B$6:$B82,B82)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R82)+(($R$6:$R$305=R82)*($B$6:$B$305&lt;B82)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T82">
@@ -19636,7 +19636,7 @@
         <v/>
       </c>
       <c r="S83">
-        <f>IF(OR(B83="",COUNTIF($B$6:$B83,B83)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R83)+(($R$6:$R$305=R83)*(ROW($B$6:$B$305)&lt;ROW(B83)))))+1)</f>
+        <f>IF(OR(B83="",COUNTIF($B$6:$B83,B83)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R83)+(($R$6:$R$305=R83)*($B$6:$B$305&lt;B83)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T83">
@@ -19674,7 +19674,7 @@
         <v/>
       </c>
       <c r="S84">
-        <f>IF(OR(B84="",COUNTIF($B$6:$B84,B84)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R84)+(($R$6:$R$305=R84)*(ROW($B$6:$B$305)&lt;ROW(B84)))))+1)</f>
+        <f>IF(OR(B84="",COUNTIF($B$6:$B84,B84)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R84)+(($R$6:$R$305=R84)*($B$6:$B$305&lt;B84)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T84">
@@ -19712,7 +19712,7 @@
         <v/>
       </c>
       <c r="S85">
-        <f>IF(OR(B85="",COUNTIF($B$6:$B85,B85)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R85)+(($R$6:$R$305=R85)*(ROW($B$6:$B$305)&lt;ROW(B85)))))+1)</f>
+        <f>IF(OR(B85="",COUNTIF($B$6:$B85,B85)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R85)+(($R$6:$R$305=R85)*($B$6:$B$305&lt;B85)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T85">
@@ -19750,7 +19750,7 @@
         <v/>
       </c>
       <c r="S86">
-        <f>IF(OR(B86="",COUNTIF($B$6:$B86,B86)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R86)+(($R$6:$R$305=R86)*(ROW($B$6:$B$305)&lt;ROW(B86)))))+1)</f>
+        <f>IF(OR(B86="",COUNTIF($B$6:$B86,B86)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R86)+(($R$6:$R$305=R86)*($B$6:$B$305&lt;B86)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T86">
@@ -19788,7 +19788,7 @@
         <v/>
       </c>
       <c r="S87">
-        <f>IF(OR(B87="",COUNTIF($B$6:$B87,B87)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R87)+(($R$6:$R$305=R87)*(ROW($B$6:$B$305)&lt;ROW(B87)))))+1)</f>
+        <f>IF(OR(B87="",COUNTIF($B$6:$B87,B87)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R87)+(($R$6:$R$305=R87)*($B$6:$B$305&lt;B87)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T87">
@@ -19826,7 +19826,7 @@
         <v/>
       </c>
       <c r="S88">
-        <f>IF(OR(B88="",COUNTIF($B$6:$B88,B88)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R88)+(($R$6:$R$305=R88)*(ROW($B$6:$B$305)&lt;ROW(B88)))))+1)</f>
+        <f>IF(OR(B88="",COUNTIF($B$6:$B88,B88)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R88)+(($R$6:$R$305=R88)*($B$6:$B$305&lt;B88)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T88">
@@ -19864,7 +19864,7 @@
         <v/>
       </c>
       <c r="S89">
-        <f>IF(OR(B89="",COUNTIF($B$6:$B89,B89)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R89)+(($R$6:$R$305=R89)*(ROW($B$6:$B$305)&lt;ROW(B89)))))+1)</f>
+        <f>IF(OR(B89="",COUNTIF($B$6:$B89,B89)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R89)+(($R$6:$R$305=R89)*($B$6:$B$305&lt;B89)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T89">
@@ -19902,7 +19902,7 @@
         <v/>
       </c>
       <c r="S90">
-        <f>IF(OR(B90="",COUNTIF($B$6:$B90,B90)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R90)+(($R$6:$R$305=R90)*(ROW($B$6:$B$305)&lt;ROW(B90)))))+1)</f>
+        <f>IF(OR(B90="",COUNTIF($B$6:$B90,B90)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R90)+(($R$6:$R$305=R90)*($B$6:$B$305&lt;B90)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T90">
@@ -19940,7 +19940,7 @@
         <v/>
       </c>
       <c r="S91">
-        <f>IF(OR(B91="",COUNTIF($B$6:$B91,B91)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R91)+(($R$6:$R$305=R91)*(ROW($B$6:$B$305)&lt;ROW(B91)))))+1)</f>
+        <f>IF(OR(B91="",COUNTIF($B$6:$B91,B91)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R91)+(($R$6:$R$305=R91)*($B$6:$B$305&lt;B91)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T91">
@@ -19978,7 +19978,7 @@
         <v/>
       </c>
       <c r="S92">
-        <f>IF(OR(B92="",COUNTIF($B$6:$B92,B92)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R92)+(($R$6:$R$305=R92)*(ROW($B$6:$B$305)&lt;ROW(B92)))))+1)</f>
+        <f>IF(OR(B92="",COUNTIF($B$6:$B92,B92)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R92)+(($R$6:$R$305=R92)*($B$6:$B$305&lt;B92)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T92">
@@ -20016,7 +20016,7 @@
         <v/>
       </c>
       <c r="S93">
-        <f>IF(OR(B93="",COUNTIF($B$6:$B93,B93)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R93)+(($R$6:$R$305=R93)*(ROW($B$6:$B$305)&lt;ROW(B93)))))+1)</f>
+        <f>IF(OR(B93="",COUNTIF($B$6:$B93,B93)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R93)+(($R$6:$R$305=R93)*($B$6:$B$305&lt;B93)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T93">
@@ -20054,7 +20054,7 @@
         <v/>
       </c>
       <c r="S94">
-        <f>IF(OR(B94="",COUNTIF($B$6:$B94,B94)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R94)+(($R$6:$R$305=R94)*(ROW($B$6:$B$305)&lt;ROW(B94)))))+1)</f>
+        <f>IF(OR(B94="",COUNTIF($B$6:$B94,B94)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R94)+(($R$6:$R$305=R94)*($B$6:$B$305&lt;B94)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T94">
@@ -20092,7 +20092,7 @@
         <v/>
       </c>
       <c r="S95">
-        <f>IF(OR(B95="",COUNTIF($B$6:$B95,B95)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R95)+(($R$6:$R$305=R95)*(ROW($B$6:$B$305)&lt;ROW(B95)))))+1)</f>
+        <f>IF(OR(B95="",COUNTIF($B$6:$B95,B95)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R95)+(($R$6:$R$305=R95)*($B$6:$B$305&lt;B95)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T95">
@@ -20130,7 +20130,7 @@
         <v/>
       </c>
       <c r="S96">
-        <f>IF(OR(B96="",COUNTIF($B$6:$B96,B96)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R96)+(($R$6:$R$305=R96)*(ROW($B$6:$B$305)&lt;ROW(B96)))))+1)</f>
+        <f>IF(OR(B96="",COUNTIF($B$6:$B96,B96)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R96)+(($R$6:$R$305=R96)*($B$6:$B$305&lt;B96)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T96">
@@ -20168,7 +20168,7 @@
         <v/>
       </c>
       <c r="S97">
-        <f>IF(OR(B97="",COUNTIF($B$6:$B97,B97)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R97)+(($R$6:$R$305=R97)*(ROW($B$6:$B$305)&lt;ROW(B97)))))+1)</f>
+        <f>IF(OR(B97="",COUNTIF($B$6:$B97,B97)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R97)+(($R$6:$R$305=R97)*($B$6:$B$305&lt;B97)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T97">
@@ -20206,7 +20206,7 @@
         <v/>
       </c>
       <c r="S98">
-        <f>IF(OR(B98="",COUNTIF($B$6:$B98,B98)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R98)+(($R$6:$R$305=R98)*(ROW($B$6:$B$305)&lt;ROW(B98)))))+1)</f>
+        <f>IF(OR(B98="",COUNTIF($B$6:$B98,B98)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R98)+(($R$6:$R$305=R98)*($B$6:$B$305&lt;B98)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T98">
@@ -20244,7 +20244,7 @@
         <v/>
       </c>
       <c r="S99">
-        <f>IF(OR(B99="",COUNTIF($B$6:$B99,B99)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R99)+(($R$6:$R$305=R99)*(ROW($B$6:$B$305)&lt;ROW(B99)))))+1)</f>
+        <f>IF(OR(B99="",COUNTIF($B$6:$B99,B99)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R99)+(($R$6:$R$305=R99)*($B$6:$B$305&lt;B99)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T99">
@@ -20282,7 +20282,7 @@
         <v/>
       </c>
       <c r="S100">
-        <f>IF(OR(B100="",COUNTIF($B$6:$B100,B100)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R100)+(($R$6:$R$305=R100)*(ROW($B$6:$B$305)&lt;ROW(B100)))))+1)</f>
+        <f>IF(OR(B100="",COUNTIF($B$6:$B100,B100)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R100)+(($R$6:$R$305=R100)*($B$6:$B$305&lt;B100)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T100">
@@ -20320,7 +20320,7 @@
         <v/>
       </c>
       <c r="S101">
-        <f>IF(OR(B101="",COUNTIF($B$6:$B101,B101)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R101)+(($R$6:$R$305=R101)*(ROW($B$6:$B$305)&lt;ROW(B101)))))+1)</f>
+        <f>IF(OR(B101="",COUNTIF($B$6:$B101,B101)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R101)+(($R$6:$R$305=R101)*($B$6:$B$305&lt;B101)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T101">
@@ -20358,7 +20358,7 @@
         <v/>
       </c>
       <c r="S102">
-        <f>IF(OR(B102="",COUNTIF($B$6:$B102,B102)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R102)+(($R$6:$R$305=R102)*(ROW($B$6:$B$305)&lt;ROW(B102)))))+1)</f>
+        <f>IF(OR(B102="",COUNTIF($B$6:$B102,B102)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R102)+(($R$6:$R$305=R102)*($B$6:$B$305&lt;B102)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T102">
@@ -20396,7 +20396,7 @@
         <v/>
       </c>
       <c r="S103">
-        <f>IF(OR(B103="",COUNTIF($B$6:$B103,B103)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R103)+(($R$6:$R$305=R103)*(ROW($B$6:$B$305)&lt;ROW(B103)))))+1)</f>
+        <f>IF(OR(B103="",COUNTIF($B$6:$B103,B103)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R103)+(($R$6:$R$305=R103)*($B$6:$B$305&lt;B103)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T103">
@@ -20434,7 +20434,7 @@
         <v/>
       </c>
       <c r="S104">
-        <f>IF(OR(B104="",COUNTIF($B$6:$B104,B104)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R104)+(($R$6:$R$305=R104)*(ROW($B$6:$B$305)&lt;ROW(B104)))))+1)</f>
+        <f>IF(OR(B104="",COUNTIF($B$6:$B104,B104)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R104)+(($R$6:$R$305=R104)*($B$6:$B$305&lt;B104)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T104">
@@ -20472,7 +20472,7 @@
         <v/>
       </c>
       <c r="S105">
-        <f>IF(OR(B105="",COUNTIF($B$6:$B105,B105)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R105)+(($R$6:$R$305=R105)*(ROW($B$6:$B$305)&lt;ROW(B105)))))+1)</f>
+        <f>IF(OR(B105="",COUNTIF($B$6:$B105,B105)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R105)+(($R$6:$R$305=R105)*($B$6:$B$305&lt;B105)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
       <c r="T105">
@@ -20510,7 +20510,7 @@
         <v/>
       </c>
       <c r="S106">
-        <f>IF(OR(B106="",COUNTIF($B$6:$B106,B106)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R106)+(($R$6:$R$305=R106)*(ROW($B$6:$B$305)&lt;ROW(B106)))))+1)</f>
+        <f>IF(OR(B106="",COUNTIF($B$6:$B106,B106)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R106)+(($R$6:$R$305=R106)*($B$6:$B$305&lt;B106)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20532,7 +20532,7 @@
         <v/>
       </c>
       <c r="S107">
-        <f>IF(OR(B107="",COUNTIF($B$6:$B107,B107)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R107)+(($R$6:$R$305=R107)*(ROW($B$6:$B$305)&lt;ROW(B107)))))+1)</f>
+        <f>IF(OR(B107="",COUNTIF($B$6:$B107,B107)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R107)+(($R$6:$R$305=R107)*($B$6:$B$305&lt;B107)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20554,7 +20554,7 @@
         <v/>
       </c>
       <c r="S108">
-        <f>IF(OR(B108="",COUNTIF($B$6:$B108,B108)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R108)+(($R$6:$R$305=R108)*(ROW($B$6:$B$305)&lt;ROW(B108)))))+1)</f>
+        <f>IF(OR(B108="",COUNTIF($B$6:$B108,B108)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R108)+(($R$6:$R$305=R108)*($B$6:$B$305&lt;B108)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20576,7 +20576,7 @@
         <v/>
       </c>
       <c r="S109">
-        <f>IF(OR(B109="",COUNTIF($B$6:$B109,B109)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R109)+(($R$6:$R$305=R109)*(ROW($B$6:$B$305)&lt;ROW(B109)))))+1)</f>
+        <f>IF(OR(B109="",COUNTIF($B$6:$B109,B109)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R109)+(($R$6:$R$305=R109)*($B$6:$B$305&lt;B109)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20598,7 +20598,7 @@
         <v/>
       </c>
       <c r="S110">
-        <f>IF(OR(B110="",COUNTIF($B$6:$B110,B110)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R110)+(($R$6:$R$305=R110)*(ROW($B$6:$B$305)&lt;ROW(B110)))))+1)</f>
+        <f>IF(OR(B110="",COUNTIF($B$6:$B110,B110)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R110)+(($R$6:$R$305=R110)*($B$6:$B$305&lt;B110)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20620,7 +20620,7 @@
         <v/>
       </c>
       <c r="S111">
-        <f>IF(OR(B111="",COUNTIF($B$6:$B111,B111)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R111)+(($R$6:$R$305=R111)*(ROW($B$6:$B$305)&lt;ROW(B111)))))+1)</f>
+        <f>IF(OR(B111="",COUNTIF($B$6:$B111,B111)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R111)+(($R$6:$R$305=R111)*($B$6:$B$305&lt;B111)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20642,7 +20642,7 @@
         <v/>
       </c>
       <c r="S112">
-        <f>IF(OR(B112="",COUNTIF($B$6:$B112,B112)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R112)+(($R$6:$R$305=R112)*(ROW($B$6:$B$305)&lt;ROW(B112)))))+1)</f>
+        <f>IF(OR(B112="",COUNTIF($B$6:$B112,B112)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R112)+(($R$6:$R$305=R112)*($B$6:$B$305&lt;B112)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20664,7 +20664,7 @@
         <v/>
       </c>
       <c r="S113">
-        <f>IF(OR(B113="",COUNTIF($B$6:$B113,B113)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R113)+(($R$6:$R$305=R113)*(ROW($B$6:$B$305)&lt;ROW(B113)))))+1)</f>
+        <f>IF(OR(B113="",COUNTIF($B$6:$B113,B113)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R113)+(($R$6:$R$305=R113)*($B$6:$B$305&lt;B113)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20686,7 +20686,7 @@
         <v/>
       </c>
       <c r="S114">
-        <f>IF(OR(B114="",COUNTIF($B$6:$B114,B114)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R114)+(($R$6:$R$305=R114)*(ROW($B$6:$B$305)&lt;ROW(B114)))))+1)</f>
+        <f>IF(OR(B114="",COUNTIF($B$6:$B114,B114)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R114)+(($R$6:$R$305=R114)*($B$6:$B$305&lt;B114)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20708,7 +20708,7 @@
         <v/>
       </c>
       <c r="S115">
-        <f>IF(OR(B115="",COUNTIF($B$6:$B115,B115)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R115)+(($R$6:$R$305=R115)*(ROW($B$6:$B$305)&lt;ROW(B115)))))+1)</f>
+        <f>IF(OR(B115="",COUNTIF($B$6:$B115,B115)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R115)+(($R$6:$R$305=R115)*($B$6:$B$305&lt;B115)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20730,7 +20730,7 @@
         <v/>
       </c>
       <c r="S116">
-        <f>IF(OR(B116="",COUNTIF($B$6:$B116,B116)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R116)+(($R$6:$R$305=R116)*(ROW($B$6:$B$305)&lt;ROW(B116)))))+1)</f>
+        <f>IF(OR(B116="",COUNTIF($B$6:$B116,B116)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R116)+(($R$6:$R$305=R116)*($B$6:$B$305&lt;B116)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20752,7 +20752,7 @@
         <v/>
       </c>
       <c r="S117">
-        <f>IF(OR(B117="",COUNTIF($B$6:$B117,B117)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R117)+(($R$6:$R$305=R117)*(ROW($B$6:$B$305)&lt;ROW(B117)))))+1)</f>
+        <f>IF(OR(B117="",COUNTIF($B$6:$B117,B117)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R117)+(($R$6:$R$305=R117)*($B$6:$B$305&lt;B117)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20774,7 +20774,7 @@
         <v/>
       </c>
       <c r="S118">
-        <f>IF(OR(B118="",COUNTIF($B$6:$B118,B118)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R118)+(($R$6:$R$305=R118)*(ROW($B$6:$B$305)&lt;ROW(B118)))))+1)</f>
+        <f>IF(OR(B118="",COUNTIF($B$6:$B118,B118)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R118)+(($R$6:$R$305=R118)*($B$6:$B$305&lt;B118)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20796,7 +20796,7 @@
         <v/>
       </c>
       <c r="S119">
-        <f>IF(OR(B119="",COUNTIF($B$6:$B119,B119)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R119)+(($R$6:$R$305=R119)*(ROW($B$6:$B$305)&lt;ROW(B119)))))+1)</f>
+        <f>IF(OR(B119="",COUNTIF($B$6:$B119,B119)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R119)+(($R$6:$R$305=R119)*($B$6:$B$305&lt;B119)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20818,7 +20818,7 @@
         <v/>
       </c>
       <c r="S120">
-        <f>IF(OR(B120="",COUNTIF($B$6:$B120,B120)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R120)+(($R$6:$R$305=R120)*(ROW($B$6:$B$305)&lt;ROW(B120)))))+1)</f>
+        <f>IF(OR(B120="",COUNTIF($B$6:$B120,B120)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R120)+(($R$6:$R$305=R120)*($B$6:$B$305&lt;B120)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20840,7 +20840,7 @@
         <v/>
       </c>
       <c r="S121">
-        <f>IF(OR(B121="",COUNTIF($B$6:$B121,B121)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R121)+(($R$6:$R$305=R121)*(ROW($B$6:$B$305)&lt;ROW(B121)))))+1)</f>
+        <f>IF(OR(B121="",COUNTIF($B$6:$B121,B121)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R121)+(($R$6:$R$305=R121)*($B$6:$B$305&lt;B121)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20862,7 +20862,7 @@
         <v/>
       </c>
       <c r="S122">
-        <f>IF(OR(B122="",COUNTIF($B$6:$B122,B122)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R122)+(($R$6:$R$305=R122)*(ROW($B$6:$B$305)&lt;ROW(B122)))))+1)</f>
+        <f>IF(OR(B122="",COUNTIF($B$6:$B122,B122)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R122)+(($R$6:$R$305=R122)*($B$6:$B$305&lt;B122)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20884,7 +20884,7 @@
         <v/>
       </c>
       <c r="S123">
-        <f>IF(OR(B123="",COUNTIF($B$6:$B123,B123)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R123)+(($R$6:$R$305=R123)*(ROW($B$6:$B$305)&lt;ROW(B123)))))+1)</f>
+        <f>IF(OR(B123="",COUNTIF($B$6:$B123,B123)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R123)+(($R$6:$R$305=R123)*($B$6:$B$305&lt;B123)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20906,7 +20906,7 @@
         <v/>
       </c>
       <c r="S124">
-        <f>IF(OR(B124="",COUNTIF($B$6:$B124,B124)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R124)+(($R$6:$R$305=R124)*(ROW($B$6:$B$305)&lt;ROW(B124)))))+1)</f>
+        <f>IF(OR(B124="",COUNTIF($B$6:$B124,B124)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R124)+(($R$6:$R$305=R124)*($B$6:$B$305&lt;B124)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20928,7 +20928,7 @@
         <v/>
       </c>
       <c r="S125">
-        <f>IF(OR(B125="",COUNTIF($B$6:$B125,B125)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R125)+(($R$6:$R$305=R125)*(ROW($B$6:$B$305)&lt;ROW(B125)))))+1)</f>
+        <f>IF(OR(B125="",COUNTIF($B$6:$B125,B125)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R125)+(($R$6:$R$305=R125)*($B$6:$B$305&lt;B125)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20950,7 +20950,7 @@
         <v/>
       </c>
       <c r="S126">
-        <f>IF(OR(B126="",COUNTIF($B$6:$B126,B126)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R126)+(($R$6:$R$305=R126)*(ROW($B$6:$B$305)&lt;ROW(B126)))))+1)</f>
+        <f>IF(OR(B126="",COUNTIF($B$6:$B126,B126)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R126)+(($R$6:$R$305=R126)*($B$6:$B$305&lt;B126)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20972,7 +20972,7 @@
         <v/>
       </c>
       <c r="S127">
-        <f>IF(OR(B127="",COUNTIF($B$6:$B127,B127)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R127)+(($R$6:$R$305=R127)*(ROW($B$6:$B$305)&lt;ROW(B127)))))+1)</f>
+        <f>IF(OR(B127="",COUNTIF($B$6:$B127,B127)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R127)+(($R$6:$R$305=R127)*($B$6:$B$305&lt;B127)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -20994,7 +20994,7 @@
         <v/>
       </c>
       <c r="S128">
-        <f>IF(OR(B128="",COUNTIF($B$6:$B128,B128)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R128)+(($R$6:$R$305=R128)*(ROW($B$6:$B$305)&lt;ROW(B128)))))+1)</f>
+        <f>IF(OR(B128="",COUNTIF($B$6:$B128,B128)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R128)+(($R$6:$R$305=R128)*($B$6:$B$305&lt;B128)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21016,7 +21016,7 @@
         <v/>
       </c>
       <c r="S129">
-        <f>IF(OR(B129="",COUNTIF($B$6:$B129,B129)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R129)+(($R$6:$R$305=R129)*(ROW($B$6:$B$305)&lt;ROW(B129)))))+1)</f>
+        <f>IF(OR(B129="",COUNTIF($B$6:$B129,B129)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R129)+(($R$6:$R$305=R129)*($B$6:$B$305&lt;B129)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21038,7 +21038,7 @@
         <v/>
       </c>
       <c r="S130">
-        <f>IF(OR(B130="",COUNTIF($B$6:$B130,B130)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R130)+(($R$6:$R$305=R130)*(ROW($B$6:$B$305)&lt;ROW(B130)))))+1)</f>
+        <f>IF(OR(B130="",COUNTIF($B$6:$B130,B130)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R130)+(($R$6:$R$305=R130)*($B$6:$B$305&lt;B130)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21060,7 +21060,7 @@
         <v/>
       </c>
       <c r="S131">
-        <f>IF(OR(B131="",COUNTIF($B$6:$B131,B131)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R131)+(($R$6:$R$305=R131)*(ROW($B$6:$B$305)&lt;ROW(B131)))))+1)</f>
+        <f>IF(OR(B131="",COUNTIF($B$6:$B131,B131)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R131)+(($R$6:$R$305=R131)*($B$6:$B$305&lt;B131)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21082,7 +21082,7 @@
         <v/>
       </c>
       <c r="S132">
-        <f>IF(OR(B132="",COUNTIF($B$6:$B132,B132)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R132)+(($R$6:$R$305=R132)*(ROW($B$6:$B$305)&lt;ROW(B132)))))+1)</f>
+        <f>IF(OR(B132="",COUNTIF($B$6:$B132,B132)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R132)+(($R$6:$R$305=R132)*($B$6:$B$305&lt;B132)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21104,7 +21104,7 @@
         <v/>
       </c>
       <c r="S133">
-        <f>IF(OR(B133="",COUNTIF($B$6:$B133,B133)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R133)+(($R$6:$R$305=R133)*(ROW($B$6:$B$305)&lt;ROW(B133)))))+1)</f>
+        <f>IF(OR(B133="",COUNTIF($B$6:$B133,B133)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R133)+(($R$6:$R$305=R133)*($B$6:$B$305&lt;B133)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21126,7 +21126,7 @@
         <v/>
       </c>
       <c r="S134">
-        <f>IF(OR(B134="",COUNTIF($B$6:$B134,B134)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R134)+(($R$6:$R$305=R134)*(ROW($B$6:$B$305)&lt;ROW(B134)))))+1)</f>
+        <f>IF(OR(B134="",COUNTIF($B$6:$B134,B134)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R134)+(($R$6:$R$305=R134)*($B$6:$B$305&lt;B134)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21148,7 +21148,7 @@
         <v/>
       </c>
       <c r="S135">
-        <f>IF(OR(B135="",COUNTIF($B$6:$B135,B135)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R135)+(($R$6:$R$305=R135)*(ROW($B$6:$B$305)&lt;ROW(B135)))))+1)</f>
+        <f>IF(OR(B135="",COUNTIF($B$6:$B135,B135)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R135)+(($R$6:$R$305=R135)*($B$6:$B$305&lt;B135)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21170,7 +21170,7 @@
         <v/>
       </c>
       <c r="S136">
-        <f>IF(OR(B136="",COUNTIF($B$6:$B136,B136)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R136)+(($R$6:$R$305=R136)*(ROW($B$6:$B$305)&lt;ROW(B136)))))+1)</f>
+        <f>IF(OR(B136="",COUNTIF($B$6:$B136,B136)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R136)+(($R$6:$R$305=R136)*($B$6:$B$305&lt;B136)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21192,7 +21192,7 @@
         <v/>
       </c>
       <c r="S137">
-        <f>IF(OR(B137="",COUNTIF($B$6:$B137,B137)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R137)+(($R$6:$R$305=R137)*(ROW($B$6:$B$305)&lt;ROW(B137)))))+1)</f>
+        <f>IF(OR(B137="",COUNTIF($B$6:$B137,B137)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R137)+(($R$6:$R$305=R137)*($B$6:$B$305&lt;B137)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21214,7 +21214,7 @@
         <v/>
       </c>
       <c r="S138">
-        <f>IF(OR(B138="",COUNTIF($B$6:$B138,B138)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R138)+(($R$6:$R$305=R138)*(ROW($B$6:$B$305)&lt;ROW(B138)))))+1)</f>
+        <f>IF(OR(B138="",COUNTIF($B$6:$B138,B138)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R138)+(($R$6:$R$305=R138)*($B$6:$B$305&lt;B138)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21236,7 +21236,7 @@
         <v/>
       </c>
       <c r="S139">
-        <f>IF(OR(B139="",COUNTIF($B$6:$B139,B139)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R139)+(($R$6:$R$305=R139)*(ROW($B$6:$B$305)&lt;ROW(B139)))))+1)</f>
+        <f>IF(OR(B139="",COUNTIF($B$6:$B139,B139)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R139)+(($R$6:$R$305=R139)*($B$6:$B$305&lt;B139)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21258,7 +21258,7 @@
         <v/>
       </c>
       <c r="S140">
-        <f>IF(OR(B140="",COUNTIF($B$6:$B140,B140)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R140)+(($R$6:$R$305=R140)*(ROW($B$6:$B$305)&lt;ROW(B140)))))+1)</f>
+        <f>IF(OR(B140="",COUNTIF($B$6:$B140,B140)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R140)+(($R$6:$R$305=R140)*($B$6:$B$305&lt;B140)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21280,7 +21280,7 @@
         <v/>
       </c>
       <c r="S141">
-        <f>IF(OR(B141="",COUNTIF($B$6:$B141,B141)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R141)+(($R$6:$R$305=R141)*(ROW($B$6:$B$305)&lt;ROW(B141)))))+1)</f>
+        <f>IF(OR(B141="",COUNTIF($B$6:$B141,B141)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R141)+(($R$6:$R$305=R141)*($B$6:$B$305&lt;B141)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21302,7 +21302,7 @@
         <v/>
       </c>
       <c r="S142">
-        <f>IF(OR(B142="",COUNTIF($B$6:$B142,B142)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R142)+(($R$6:$R$305=R142)*(ROW($B$6:$B$305)&lt;ROW(B142)))))+1)</f>
+        <f>IF(OR(B142="",COUNTIF($B$6:$B142,B142)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R142)+(($R$6:$R$305=R142)*($B$6:$B$305&lt;B142)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21324,7 +21324,7 @@
         <v/>
       </c>
       <c r="S143">
-        <f>IF(OR(B143="",COUNTIF($B$6:$B143,B143)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R143)+(($R$6:$R$305=R143)*(ROW($B$6:$B$305)&lt;ROW(B143)))))+1)</f>
+        <f>IF(OR(B143="",COUNTIF($B$6:$B143,B143)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R143)+(($R$6:$R$305=R143)*($B$6:$B$305&lt;B143)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21346,7 +21346,7 @@
         <v/>
       </c>
       <c r="S144">
-        <f>IF(OR(B144="",COUNTIF($B$6:$B144,B144)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R144)+(($R$6:$R$305=R144)*(ROW($B$6:$B$305)&lt;ROW(B144)))))+1)</f>
+        <f>IF(OR(B144="",COUNTIF($B$6:$B144,B144)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R144)+(($R$6:$R$305=R144)*($B$6:$B$305&lt;B144)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21368,7 +21368,7 @@
         <v/>
       </c>
       <c r="S145">
-        <f>IF(OR(B145="",COUNTIF($B$6:$B145,B145)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R145)+(($R$6:$R$305=R145)*(ROW($B$6:$B$305)&lt;ROW(B145)))))+1)</f>
+        <f>IF(OR(B145="",COUNTIF($B$6:$B145,B145)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R145)+(($R$6:$R$305=R145)*($B$6:$B$305&lt;B145)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21390,7 +21390,7 @@
         <v/>
       </c>
       <c r="S146">
-        <f>IF(OR(B146="",COUNTIF($B$6:$B146,B146)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R146)+(($R$6:$R$305=R146)*(ROW($B$6:$B$305)&lt;ROW(B146)))))+1)</f>
+        <f>IF(OR(B146="",COUNTIF($B$6:$B146,B146)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R146)+(($R$6:$R$305=R146)*($B$6:$B$305&lt;B146)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21412,7 +21412,7 @@
         <v/>
       </c>
       <c r="S147">
-        <f>IF(OR(B147="",COUNTIF($B$6:$B147,B147)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R147)+(($R$6:$R$305=R147)*(ROW($B$6:$B$305)&lt;ROW(B147)))))+1)</f>
+        <f>IF(OR(B147="",COUNTIF($B$6:$B147,B147)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R147)+(($R$6:$R$305=R147)*($B$6:$B$305&lt;B147)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21434,7 +21434,7 @@
         <v/>
       </c>
       <c r="S148">
-        <f>IF(OR(B148="",COUNTIF($B$6:$B148,B148)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R148)+(($R$6:$R$305=R148)*(ROW($B$6:$B$305)&lt;ROW(B148)))))+1)</f>
+        <f>IF(OR(B148="",COUNTIF($B$6:$B148,B148)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R148)+(($R$6:$R$305=R148)*($B$6:$B$305&lt;B148)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21456,7 +21456,7 @@
         <v/>
       </c>
       <c r="S149">
-        <f>IF(OR(B149="",COUNTIF($B$6:$B149,B149)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R149)+(($R$6:$R$305=R149)*(ROW($B$6:$B$305)&lt;ROW(B149)))))+1)</f>
+        <f>IF(OR(B149="",COUNTIF($B$6:$B149,B149)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R149)+(($R$6:$R$305=R149)*($B$6:$B$305&lt;B149)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21478,7 +21478,7 @@
         <v/>
       </c>
       <c r="S150">
-        <f>IF(OR(B150="",COUNTIF($B$6:$B150,B150)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R150)+(($R$6:$R$305=R150)*(ROW($B$6:$B$305)&lt;ROW(B150)))))+1)</f>
+        <f>IF(OR(B150="",COUNTIF($B$6:$B150,B150)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R150)+(($R$6:$R$305=R150)*($B$6:$B$305&lt;B150)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21500,7 +21500,7 @@
         <v/>
       </c>
       <c r="S151">
-        <f>IF(OR(B151="",COUNTIF($B$6:$B151,B151)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R151)+(($R$6:$R$305=R151)*(ROW($B$6:$B$305)&lt;ROW(B151)))))+1)</f>
+        <f>IF(OR(B151="",COUNTIF($B$6:$B151,B151)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R151)+(($R$6:$R$305=R151)*($B$6:$B$305&lt;B151)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21522,7 +21522,7 @@
         <v/>
       </c>
       <c r="S152">
-        <f>IF(OR(B152="",COUNTIF($B$6:$B152,B152)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R152)+(($R$6:$R$305=R152)*(ROW($B$6:$B$305)&lt;ROW(B152)))))+1)</f>
+        <f>IF(OR(B152="",COUNTIF($B$6:$B152,B152)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R152)+(($R$6:$R$305=R152)*($B$6:$B$305&lt;B152)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21544,7 +21544,7 @@
         <v/>
       </c>
       <c r="S153">
-        <f>IF(OR(B153="",COUNTIF($B$6:$B153,B153)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R153)+(($R$6:$R$305=R153)*(ROW($B$6:$B$305)&lt;ROW(B153)))))+1)</f>
+        <f>IF(OR(B153="",COUNTIF($B$6:$B153,B153)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R153)+(($R$6:$R$305=R153)*($B$6:$B$305&lt;B153)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21566,7 +21566,7 @@
         <v/>
       </c>
       <c r="S154">
-        <f>IF(OR(B154="",COUNTIF($B$6:$B154,B154)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R154)+(($R$6:$R$305=R154)*(ROW($B$6:$B$305)&lt;ROW(B154)))))+1)</f>
+        <f>IF(OR(B154="",COUNTIF($B$6:$B154,B154)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R154)+(($R$6:$R$305=R154)*($B$6:$B$305&lt;B154)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21588,7 +21588,7 @@
         <v/>
       </c>
       <c r="S155">
-        <f>IF(OR(B155="",COUNTIF($B$6:$B155,B155)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R155)+(($R$6:$R$305=R155)*(ROW($B$6:$B$305)&lt;ROW(B155)))))+1)</f>
+        <f>IF(OR(B155="",COUNTIF($B$6:$B155,B155)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R155)+(($R$6:$R$305=R155)*($B$6:$B$305&lt;B155)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21610,7 +21610,7 @@
         <v/>
       </c>
       <c r="S156">
-        <f>IF(OR(B156="",COUNTIF($B$6:$B156,B156)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R156)+(($R$6:$R$305=R156)*(ROW($B$6:$B$305)&lt;ROW(B156)))))+1)</f>
+        <f>IF(OR(B156="",COUNTIF($B$6:$B156,B156)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R156)+(($R$6:$R$305=R156)*($B$6:$B$305&lt;B156)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21632,7 +21632,7 @@
         <v/>
       </c>
       <c r="S157">
-        <f>IF(OR(B157="",COUNTIF($B$6:$B157,B157)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R157)+(($R$6:$R$305=R157)*(ROW($B$6:$B$305)&lt;ROW(B157)))))+1)</f>
+        <f>IF(OR(B157="",COUNTIF($B$6:$B157,B157)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R157)+(($R$6:$R$305=R157)*($B$6:$B$305&lt;B157)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21654,7 +21654,7 @@
         <v/>
       </c>
       <c r="S158">
-        <f>IF(OR(B158="",COUNTIF($B$6:$B158,B158)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R158)+(($R$6:$R$305=R158)*(ROW($B$6:$B$305)&lt;ROW(B158)))))+1)</f>
+        <f>IF(OR(B158="",COUNTIF($B$6:$B158,B158)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R158)+(($R$6:$R$305=R158)*($B$6:$B$305&lt;B158)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21676,7 +21676,7 @@
         <v/>
       </c>
       <c r="S159">
-        <f>IF(OR(B159="",COUNTIF($B$6:$B159,B159)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R159)+(($R$6:$R$305=R159)*(ROW($B$6:$B$305)&lt;ROW(B159)))))+1)</f>
+        <f>IF(OR(B159="",COUNTIF($B$6:$B159,B159)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R159)+(($R$6:$R$305=R159)*($B$6:$B$305&lt;B159)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21698,7 +21698,7 @@
         <v/>
       </c>
       <c r="S160">
-        <f>IF(OR(B160="",COUNTIF($B$6:$B160,B160)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R160)+(($R$6:$R$305=R160)*(ROW($B$6:$B$305)&lt;ROW(B160)))))+1)</f>
+        <f>IF(OR(B160="",COUNTIF($B$6:$B160,B160)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R160)+(($R$6:$R$305=R160)*($B$6:$B$305&lt;B160)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21720,7 +21720,7 @@
         <v/>
       </c>
       <c r="S161">
-        <f>IF(OR(B161="",COUNTIF($B$6:$B161,B161)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R161)+(($R$6:$R$305=R161)*(ROW($B$6:$B$305)&lt;ROW(B161)))))+1)</f>
+        <f>IF(OR(B161="",COUNTIF($B$6:$B161,B161)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R161)+(($R$6:$R$305=R161)*($B$6:$B$305&lt;B161)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21742,7 +21742,7 @@
         <v/>
       </c>
       <c r="S162">
-        <f>IF(OR(B162="",COUNTIF($B$6:$B162,B162)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R162)+(($R$6:$R$305=R162)*(ROW($B$6:$B$305)&lt;ROW(B162)))))+1)</f>
+        <f>IF(OR(B162="",COUNTIF($B$6:$B162,B162)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R162)+(($R$6:$R$305=R162)*($B$6:$B$305&lt;B162)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21764,7 +21764,7 @@
         <v/>
       </c>
       <c r="S163">
-        <f>IF(OR(B163="",COUNTIF($B$6:$B163,B163)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R163)+(($R$6:$R$305=R163)*(ROW($B$6:$B$305)&lt;ROW(B163)))))+1)</f>
+        <f>IF(OR(B163="",COUNTIF($B$6:$B163,B163)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R163)+(($R$6:$R$305=R163)*($B$6:$B$305&lt;B163)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21786,7 +21786,7 @@
         <v/>
       </c>
       <c r="S164">
-        <f>IF(OR(B164="",COUNTIF($B$6:$B164,B164)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R164)+(($R$6:$R$305=R164)*(ROW($B$6:$B$305)&lt;ROW(B164)))))+1)</f>
+        <f>IF(OR(B164="",COUNTIF($B$6:$B164,B164)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R164)+(($R$6:$R$305=R164)*($B$6:$B$305&lt;B164)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21808,7 +21808,7 @@
         <v/>
       </c>
       <c r="S165">
-        <f>IF(OR(B165="",COUNTIF($B$6:$B165,B165)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R165)+(($R$6:$R$305=R165)*(ROW($B$6:$B$305)&lt;ROW(B165)))))+1)</f>
+        <f>IF(OR(B165="",COUNTIF($B$6:$B165,B165)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R165)+(($R$6:$R$305=R165)*($B$6:$B$305&lt;B165)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21830,7 +21830,7 @@
         <v/>
       </c>
       <c r="S166">
-        <f>IF(OR(B166="",COUNTIF($B$6:$B166,B166)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R166)+(($R$6:$R$305=R166)*(ROW($B$6:$B$305)&lt;ROW(B166)))))+1)</f>
+        <f>IF(OR(B166="",COUNTIF($B$6:$B166,B166)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R166)+(($R$6:$R$305=R166)*($B$6:$B$305&lt;B166)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21852,7 +21852,7 @@
         <v/>
       </c>
       <c r="S167">
-        <f>IF(OR(B167="",COUNTIF($B$6:$B167,B167)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R167)+(($R$6:$R$305=R167)*(ROW($B$6:$B$305)&lt;ROW(B167)))))+1)</f>
+        <f>IF(OR(B167="",COUNTIF($B$6:$B167,B167)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R167)+(($R$6:$R$305=R167)*($B$6:$B$305&lt;B167)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21874,7 +21874,7 @@
         <v/>
       </c>
       <c r="S168">
-        <f>IF(OR(B168="",COUNTIF($B$6:$B168,B168)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R168)+(($R$6:$R$305=R168)*(ROW($B$6:$B$305)&lt;ROW(B168)))))+1)</f>
+        <f>IF(OR(B168="",COUNTIF($B$6:$B168,B168)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R168)+(($R$6:$R$305=R168)*($B$6:$B$305&lt;B168)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21896,7 +21896,7 @@
         <v/>
       </c>
       <c r="S169">
-        <f>IF(OR(B169="",COUNTIF($B$6:$B169,B169)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R169)+(($R$6:$R$305=R169)*(ROW($B$6:$B$305)&lt;ROW(B169)))))+1)</f>
+        <f>IF(OR(B169="",COUNTIF($B$6:$B169,B169)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R169)+(($R$6:$R$305=R169)*($B$6:$B$305&lt;B169)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21918,7 +21918,7 @@
         <v/>
       </c>
       <c r="S170">
-        <f>IF(OR(B170="",COUNTIF($B$6:$B170,B170)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R170)+(($R$6:$R$305=R170)*(ROW($B$6:$B$305)&lt;ROW(B170)))))+1)</f>
+        <f>IF(OR(B170="",COUNTIF($B$6:$B170,B170)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R170)+(($R$6:$R$305=R170)*($B$6:$B$305&lt;B170)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21940,7 +21940,7 @@
         <v/>
       </c>
       <c r="S171">
-        <f>IF(OR(B171="",COUNTIF($B$6:$B171,B171)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R171)+(($R$6:$R$305=R171)*(ROW($B$6:$B$305)&lt;ROW(B171)))))+1)</f>
+        <f>IF(OR(B171="",COUNTIF($B$6:$B171,B171)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R171)+(($R$6:$R$305=R171)*($B$6:$B$305&lt;B171)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21962,7 +21962,7 @@
         <v/>
       </c>
       <c r="S172">
-        <f>IF(OR(B172="",COUNTIF($B$6:$B172,B172)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R172)+(($R$6:$R$305=R172)*(ROW($B$6:$B$305)&lt;ROW(B172)))))+1)</f>
+        <f>IF(OR(B172="",COUNTIF($B$6:$B172,B172)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R172)+(($R$6:$R$305=R172)*($B$6:$B$305&lt;B172)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -21984,7 +21984,7 @@
         <v/>
       </c>
       <c r="S173">
-        <f>IF(OR(B173="",COUNTIF($B$6:$B173,B173)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R173)+(($R$6:$R$305=R173)*(ROW($B$6:$B$305)&lt;ROW(B173)))))+1)</f>
+        <f>IF(OR(B173="",COUNTIF($B$6:$B173,B173)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R173)+(($R$6:$R$305=R173)*($B$6:$B$305&lt;B173)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22006,7 +22006,7 @@
         <v/>
       </c>
       <c r="S174">
-        <f>IF(OR(B174="",COUNTIF($B$6:$B174,B174)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R174)+(($R$6:$R$305=R174)*(ROW($B$6:$B$305)&lt;ROW(B174)))))+1)</f>
+        <f>IF(OR(B174="",COUNTIF($B$6:$B174,B174)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R174)+(($R$6:$R$305=R174)*($B$6:$B$305&lt;B174)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22028,7 +22028,7 @@
         <v/>
       </c>
       <c r="S175">
-        <f>IF(OR(B175="",COUNTIF($B$6:$B175,B175)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R175)+(($R$6:$R$305=R175)*(ROW($B$6:$B$305)&lt;ROW(B175)))))+1)</f>
+        <f>IF(OR(B175="",COUNTIF($B$6:$B175,B175)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R175)+(($R$6:$R$305=R175)*($B$6:$B$305&lt;B175)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22050,7 +22050,7 @@
         <v/>
       </c>
       <c r="S176">
-        <f>IF(OR(B176="",COUNTIF($B$6:$B176,B176)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R176)+(($R$6:$R$305=R176)*(ROW($B$6:$B$305)&lt;ROW(B176)))))+1)</f>
+        <f>IF(OR(B176="",COUNTIF($B$6:$B176,B176)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R176)+(($R$6:$R$305=R176)*($B$6:$B$305&lt;B176)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22072,7 +22072,7 @@
         <v/>
       </c>
       <c r="S177">
-        <f>IF(OR(B177="",COUNTIF($B$6:$B177,B177)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R177)+(($R$6:$R$305=R177)*(ROW($B$6:$B$305)&lt;ROW(B177)))))+1)</f>
+        <f>IF(OR(B177="",COUNTIF($B$6:$B177,B177)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R177)+(($R$6:$R$305=R177)*($B$6:$B$305&lt;B177)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22094,7 +22094,7 @@
         <v/>
       </c>
       <c r="S178">
-        <f>IF(OR(B178="",COUNTIF($B$6:$B178,B178)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R178)+(($R$6:$R$305=R178)*(ROW($B$6:$B$305)&lt;ROW(B178)))))+1)</f>
+        <f>IF(OR(B178="",COUNTIF($B$6:$B178,B178)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R178)+(($R$6:$R$305=R178)*($B$6:$B$305&lt;B178)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22116,7 +22116,7 @@
         <v/>
       </c>
       <c r="S179">
-        <f>IF(OR(B179="",COUNTIF($B$6:$B179,B179)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R179)+(($R$6:$R$305=R179)*(ROW($B$6:$B$305)&lt;ROW(B179)))))+1)</f>
+        <f>IF(OR(B179="",COUNTIF($B$6:$B179,B179)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R179)+(($R$6:$R$305=R179)*($B$6:$B$305&lt;B179)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22138,7 +22138,7 @@
         <v/>
       </c>
       <c r="S180">
-        <f>IF(OR(B180="",COUNTIF($B$6:$B180,B180)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R180)+(($R$6:$R$305=R180)*(ROW($B$6:$B$305)&lt;ROW(B180)))))+1)</f>
+        <f>IF(OR(B180="",COUNTIF($B$6:$B180,B180)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R180)+(($R$6:$R$305=R180)*($B$6:$B$305&lt;B180)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22160,7 +22160,7 @@
         <v/>
       </c>
       <c r="S181">
-        <f>IF(OR(B181="",COUNTIF($B$6:$B181,B181)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R181)+(($R$6:$R$305=R181)*(ROW($B$6:$B$305)&lt;ROW(B181)))))+1)</f>
+        <f>IF(OR(B181="",COUNTIF($B$6:$B181,B181)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R181)+(($R$6:$R$305=R181)*($B$6:$B$305&lt;B181)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22182,7 +22182,7 @@
         <v/>
       </c>
       <c r="S182">
-        <f>IF(OR(B182="",COUNTIF($B$6:$B182,B182)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R182)+(($R$6:$R$305=R182)*(ROW($B$6:$B$305)&lt;ROW(B182)))))+1)</f>
+        <f>IF(OR(B182="",COUNTIF($B$6:$B182,B182)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R182)+(($R$6:$R$305=R182)*($B$6:$B$305&lt;B182)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22204,7 +22204,7 @@
         <v/>
       </c>
       <c r="S183">
-        <f>IF(OR(B183="",COUNTIF($B$6:$B183,B183)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R183)+(($R$6:$R$305=R183)*(ROW($B$6:$B$305)&lt;ROW(B183)))))+1)</f>
+        <f>IF(OR(B183="",COUNTIF($B$6:$B183,B183)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R183)+(($R$6:$R$305=R183)*($B$6:$B$305&lt;B183)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22226,7 +22226,7 @@
         <v/>
       </c>
       <c r="S184">
-        <f>IF(OR(B184="",COUNTIF($B$6:$B184,B184)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R184)+(($R$6:$R$305=R184)*(ROW($B$6:$B$305)&lt;ROW(B184)))))+1)</f>
+        <f>IF(OR(B184="",COUNTIF($B$6:$B184,B184)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R184)+(($R$6:$R$305=R184)*($B$6:$B$305&lt;B184)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22248,7 +22248,7 @@
         <v/>
       </c>
       <c r="S185">
-        <f>IF(OR(B185="",COUNTIF($B$6:$B185,B185)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R185)+(($R$6:$R$305=R185)*(ROW($B$6:$B$305)&lt;ROW(B185)))))+1)</f>
+        <f>IF(OR(B185="",COUNTIF($B$6:$B185,B185)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R185)+(($R$6:$R$305=R185)*($B$6:$B$305&lt;B185)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22270,7 +22270,7 @@
         <v/>
       </c>
       <c r="S186">
-        <f>IF(OR(B186="",COUNTIF($B$6:$B186,B186)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R186)+(($R$6:$R$305=R186)*(ROW($B$6:$B$305)&lt;ROW(B186)))))+1)</f>
+        <f>IF(OR(B186="",COUNTIF($B$6:$B186,B186)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R186)+(($R$6:$R$305=R186)*($B$6:$B$305&lt;B186)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22292,7 +22292,7 @@
         <v/>
       </c>
       <c r="S187">
-        <f>IF(OR(B187="",COUNTIF($B$6:$B187,B187)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R187)+(($R$6:$R$305=R187)*(ROW($B$6:$B$305)&lt;ROW(B187)))))+1)</f>
+        <f>IF(OR(B187="",COUNTIF($B$6:$B187,B187)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R187)+(($R$6:$R$305=R187)*($B$6:$B$305&lt;B187)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22314,7 +22314,7 @@
         <v/>
       </c>
       <c r="S188">
-        <f>IF(OR(B188="",COUNTIF($B$6:$B188,B188)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R188)+(($R$6:$R$305=R188)*(ROW($B$6:$B$305)&lt;ROW(B188)))))+1)</f>
+        <f>IF(OR(B188="",COUNTIF($B$6:$B188,B188)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R188)+(($R$6:$R$305=R188)*($B$6:$B$305&lt;B188)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22336,7 +22336,7 @@
         <v/>
       </c>
       <c r="S189">
-        <f>IF(OR(B189="",COUNTIF($B$6:$B189,B189)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R189)+(($R$6:$R$305=R189)*(ROW($B$6:$B$305)&lt;ROW(B189)))))+1)</f>
+        <f>IF(OR(B189="",COUNTIF($B$6:$B189,B189)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R189)+(($R$6:$R$305=R189)*($B$6:$B$305&lt;B189)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22358,7 +22358,7 @@
         <v/>
       </c>
       <c r="S190">
-        <f>IF(OR(B190="",COUNTIF($B$6:$B190,B190)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R190)+(($R$6:$R$305=R190)*(ROW($B$6:$B$305)&lt;ROW(B190)))))+1)</f>
+        <f>IF(OR(B190="",COUNTIF($B$6:$B190,B190)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R190)+(($R$6:$R$305=R190)*($B$6:$B$305&lt;B190)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22380,7 +22380,7 @@
         <v/>
       </c>
       <c r="S191">
-        <f>IF(OR(B191="",COUNTIF($B$6:$B191,B191)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R191)+(($R$6:$R$305=R191)*(ROW($B$6:$B$305)&lt;ROW(B191)))))+1)</f>
+        <f>IF(OR(B191="",COUNTIF($B$6:$B191,B191)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R191)+(($R$6:$R$305=R191)*($B$6:$B$305&lt;B191)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22402,7 +22402,7 @@
         <v/>
       </c>
       <c r="S192">
-        <f>IF(OR(B192="",COUNTIF($B$6:$B192,B192)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R192)+(($R$6:$R$305=R192)*(ROW($B$6:$B$305)&lt;ROW(B192)))))+1)</f>
+        <f>IF(OR(B192="",COUNTIF($B$6:$B192,B192)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R192)+(($R$6:$R$305=R192)*($B$6:$B$305&lt;B192)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22424,7 +22424,7 @@
         <v/>
       </c>
       <c r="S193">
-        <f>IF(OR(B193="",COUNTIF($B$6:$B193,B193)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R193)+(($R$6:$R$305=R193)*(ROW($B$6:$B$305)&lt;ROW(B193)))))+1)</f>
+        <f>IF(OR(B193="",COUNTIF($B$6:$B193,B193)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R193)+(($R$6:$R$305=R193)*($B$6:$B$305&lt;B193)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22446,7 +22446,7 @@
         <v/>
       </c>
       <c r="S194">
-        <f>IF(OR(B194="",COUNTIF($B$6:$B194,B194)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R194)+(($R$6:$R$305=R194)*(ROW($B$6:$B$305)&lt;ROW(B194)))))+1)</f>
+        <f>IF(OR(B194="",COUNTIF($B$6:$B194,B194)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R194)+(($R$6:$R$305=R194)*($B$6:$B$305&lt;B194)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22468,7 +22468,7 @@
         <v/>
       </c>
       <c r="S195">
-        <f>IF(OR(B195="",COUNTIF($B$6:$B195,B195)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R195)+(($R$6:$R$305=R195)*(ROW($B$6:$B$305)&lt;ROW(B195)))))+1)</f>
+        <f>IF(OR(B195="",COUNTIF($B$6:$B195,B195)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R195)+(($R$6:$R$305=R195)*($B$6:$B$305&lt;B195)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22490,7 +22490,7 @@
         <v/>
       </c>
       <c r="S196">
-        <f>IF(OR(B196="",COUNTIF($B$6:$B196,B196)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R196)+(($R$6:$R$305=R196)*(ROW($B$6:$B$305)&lt;ROW(B196)))))+1)</f>
+        <f>IF(OR(B196="",COUNTIF($B$6:$B196,B196)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R196)+(($R$6:$R$305=R196)*($B$6:$B$305&lt;B196)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22512,7 +22512,7 @@
         <v/>
       </c>
       <c r="S197">
-        <f>IF(OR(B197="",COUNTIF($B$6:$B197,B197)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R197)+(($R$6:$R$305=R197)*(ROW($B$6:$B$305)&lt;ROW(B197)))))+1)</f>
+        <f>IF(OR(B197="",COUNTIF($B$6:$B197,B197)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R197)+(($R$6:$R$305=R197)*($B$6:$B$305&lt;B197)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22534,7 +22534,7 @@
         <v/>
       </c>
       <c r="S198">
-        <f>IF(OR(B198="",COUNTIF($B$6:$B198,B198)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R198)+(($R$6:$R$305=R198)*(ROW($B$6:$B$305)&lt;ROW(B198)))))+1)</f>
+        <f>IF(OR(B198="",COUNTIF($B$6:$B198,B198)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R198)+(($R$6:$R$305=R198)*($B$6:$B$305&lt;B198)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22556,7 +22556,7 @@
         <v/>
       </c>
       <c r="S199">
-        <f>IF(OR(B199="",COUNTIF($B$6:$B199,B199)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R199)+(($R$6:$R$305=R199)*(ROW($B$6:$B$305)&lt;ROW(B199)))))+1)</f>
+        <f>IF(OR(B199="",COUNTIF($B$6:$B199,B199)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R199)+(($R$6:$R$305=R199)*($B$6:$B$305&lt;B199)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22578,7 +22578,7 @@
         <v/>
       </c>
       <c r="S200">
-        <f>IF(OR(B200="",COUNTIF($B$6:$B200,B200)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R200)+(($R$6:$R$305=R200)*(ROW($B$6:$B$305)&lt;ROW(B200)))))+1)</f>
+        <f>IF(OR(B200="",COUNTIF($B$6:$B200,B200)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R200)+(($R$6:$R$305=R200)*($B$6:$B$305&lt;B200)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22600,7 +22600,7 @@
         <v/>
       </c>
       <c r="S201">
-        <f>IF(OR(B201="",COUNTIF($B$6:$B201,B201)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R201)+(($R$6:$R$305=R201)*(ROW($B$6:$B$305)&lt;ROW(B201)))))+1)</f>
+        <f>IF(OR(B201="",COUNTIF($B$6:$B201,B201)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R201)+(($R$6:$R$305=R201)*($B$6:$B$305&lt;B201)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22622,7 +22622,7 @@
         <v/>
       </c>
       <c r="S202">
-        <f>IF(OR(B202="",COUNTIF($B$6:$B202,B202)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R202)+(($R$6:$R$305=R202)*(ROW($B$6:$B$305)&lt;ROW(B202)))))+1)</f>
+        <f>IF(OR(B202="",COUNTIF($B$6:$B202,B202)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R202)+(($R$6:$R$305=R202)*($B$6:$B$305&lt;B202)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22644,7 +22644,7 @@
         <v/>
       </c>
       <c r="S203">
-        <f>IF(OR(B203="",COUNTIF($B$6:$B203,B203)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R203)+(($R$6:$R$305=R203)*(ROW($B$6:$B$305)&lt;ROW(B203)))))+1)</f>
+        <f>IF(OR(B203="",COUNTIF($B$6:$B203,B203)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R203)+(($R$6:$R$305=R203)*($B$6:$B$305&lt;B203)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22666,7 +22666,7 @@
         <v/>
       </c>
       <c r="S204">
-        <f>IF(OR(B204="",COUNTIF($B$6:$B204,B204)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R204)+(($R$6:$R$305=R204)*(ROW($B$6:$B$305)&lt;ROW(B204)))))+1)</f>
+        <f>IF(OR(B204="",COUNTIF($B$6:$B204,B204)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R204)+(($R$6:$R$305=R204)*($B$6:$B$305&lt;B204)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22688,7 +22688,7 @@
         <v/>
       </c>
       <c r="S205">
-        <f>IF(OR(B205="",COUNTIF($B$6:$B205,B205)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R205)+(($R$6:$R$305=R205)*(ROW($B$6:$B$305)&lt;ROW(B205)))))+1)</f>
+        <f>IF(OR(B205="",COUNTIF($B$6:$B205,B205)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R205)+(($R$6:$R$305=R205)*($B$6:$B$305&lt;B205)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22710,7 +22710,7 @@
         <v/>
       </c>
       <c r="S206">
-        <f>IF(OR(B206="",COUNTIF($B$6:$B206,B206)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R206)+(($R$6:$R$305=R206)*(ROW($B$6:$B$305)&lt;ROW(B206)))))+1)</f>
+        <f>IF(OR(B206="",COUNTIF($B$6:$B206,B206)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R206)+(($R$6:$R$305=R206)*($B$6:$B$305&lt;B206)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22732,7 +22732,7 @@
         <v/>
       </c>
       <c r="S207">
-        <f>IF(OR(B207="",COUNTIF($B$6:$B207,B207)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R207)+(($R$6:$R$305=R207)*(ROW($B$6:$B$305)&lt;ROW(B207)))))+1)</f>
+        <f>IF(OR(B207="",COUNTIF($B$6:$B207,B207)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R207)+(($R$6:$R$305=R207)*($B$6:$B$305&lt;B207)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22754,7 +22754,7 @@
         <v/>
       </c>
       <c r="S208">
-        <f>IF(OR(B208="",COUNTIF($B$6:$B208,B208)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R208)+(($R$6:$R$305=R208)*(ROW($B$6:$B$305)&lt;ROW(B208)))))+1)</f>
+        <f>IF(OR(B208="",COUNTIF($B$6:$B208,B208)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R208)+(($R$6:$R$305=R208)*($B$6:$B$305&lt;B208)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22776,7 +22776,7 @@
         <v/>
       </c>
       <c r="S209">
-        <f>IF(OR(B209="",COUNTIF($B$6:$B209,B209)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R209)+(($R$6:$R$305=R209)*(ROW($B$6:$B$305)&lt;ROW(B209)))))+1)</f>
+        <f>IF(OR(B209="",COUNTIF($B$6:$B209,B209)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R209)+(($R$6:$R$305=R209)*($B$6:$B$305&lt;B209)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22798,7 +22798,7 @@
         <v/>
       </c>
       <c r="S210">
-        <f>IF(OR(B210="",COUNTIF($B$6:$B210,B210)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R210)+(($R$6:$R$305=R210)*(ROW($B$6:$B$305)&lt;ROW(B210)))))+1)</f>
+        <f>IF(OR(B210="",COUNTIF($B$6:$B210,B210)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R210)+(($R$6:$R$305=R210)*($B$6:$B$305&lt;B210)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22820,7 +22820,7 @@
         <v/>
       </c>
       <c r="S211">
-        <f>IF(OR(B211="",COUNTIF($B$6:$B211,B211)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R211)+(($R$6:$R$305=R211)*(ROW($B$6:$B$305)&lt;ROW(B211)))))+1)</f>
+        <f>IF(OR(B211="",COUNTIF($B$6:$B211,B211)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R211)+(($R$6:$R$305=R211)*($B$6:$B$305&lt;B211)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22842,7 +22842,7 @@
         <v/>
       </c>
       <c r="S212">
-        <f>IF(OR(B212="",COUNTIF($B$6:$B212,B212)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R212)+(($R$6:$R$305=R212)*(ROW($B$6:$B$305)&lt;ROW(B212)))))+1)</f>
+        <f>IF(OR(B212="",COUNTIF($B$6:$B212,B212)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R212)+(($R$6:$R$305=R212)*($B$6:$B$305&lt;B212)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22864,7 +22864,7 @@
         <v/>
       </c>
       <c r="S213">
-        <f>IF(OR(B213="",COUNTIF($B$6:$B213,B213)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R213)+(($R$6:$R$305=R213)*(ROW($B$6:$B$305)&lt;ROW(B213)))))+1)</f>
+        <f>IF(OR(B213="",COUNTIF($B$6:$B213,B213)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R213)+(($R$6:$R$305=R213)*($B$6:$B$305&lt;B213)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22886,7 +22886,7 @@
         <v/>
       </c>
       <c r="S214">
-        <f>IF(OR(B214="",COUNTIF($B$6:$B214,B214)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R214)+(($R$6:$R$305=R214)*(ROW($B$6:$B$305)&lt;ROW(B214)))))+1)</f>
+        <f>IF(OR(B214="",COUNTIF($B$6:$B214,B214)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R214)+(($R$6:$R$305=R214)*($B$6:$B$305&lt;B214)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22908,7 +22908,7 @@
         <v/>
       </c>
       <c r="S215">
-        <f>IF(OR(B215="",COUNTIF($B$6:$B215,B215)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R215)+(($R$6:$R$305=R215)*(ROW($B$6:$B$305)&lt;ROW(B215)))))+1)</f>
+        <f>IF(OR(B215="",COUNTIF($B$6:$B215,B215)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R215)+(($R$6:$R$305=R215)*($B$6:$B$305&lt;B215)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22930,7 +22930,7 @@
         <v/>
       </c>
       <c r="S216">
-        <f>IF(OR(B216="",COUNTIF($B$6:$B216,B216)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R216)+(($R$6:$R$305=R216)*(ROW($B$6:$B$305)&lt;ROW(B216)))))+1)</f>
+        <f>IF(OR(B216="",COUNTIF($B$6:$B216,B216)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R216)+(($R$6:$R$305=R216)*($B$6:$B$305&lt;B216)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22952,7 +22952,7 @@
         <v/>
       </c>
       <c r="S217">
-        <f>IF(OR(B217="",COUNTIF($B$6:$B217,B217)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R217)+(($R$6:$R$305=R217)*(ROW($B$6:$B$305)&lt;ROW(B217)))))+1)</f>
+        <f>IF(OR(B217="",COUNTIF($B$6:$B217,B217)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R217)+(($R$6:$R$305=R217)*($B$6:$B$305&lt;B217)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22974,7 +22974,7 @@
         <v/>
       </c>
       <c r="S218">
-        <f>IF(OR(B218="",COUNTIF($B$6:$B218,B218)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R218)+(($R$6:$R$305=R218)*(ROW($B$6:$B$305)&lt;ROW(B218)))))+1)</f>
+        <f>IF(OR(B218="",COUNTIF($B$6:$B218,B218)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R218)+(($R$6:$R$305=R218)*($B$6:$B$305&lt;B218)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -22996,7 +22996,7 @@
         <v/>
       </c>
       <c r="S219">
-        <f>IF(OR(B219="",COUNTIF($B$6:$B219,B219)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R219)+(($R$6:$R$305=R219)*(ROW($B$6:$B$305)&lt;ROW(B219)))))+1)</f>
+        <f>IF(OR(B219="",COUNTIF($B$6:$B219,B219)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R219)+(($R$6:$R$305=R219)*($B$6:$B$305&lt;B219)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23018,7 +23018,7 @@
         <v/>
       </c>
       <c r="S220">
-        <f>IF(OR(B220="",COUNTIF($B$6:$B220,B220)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R220)+(($R$6:$R$305=R220)*(ROW($B$6:$B$305)&lt;ROW(B220)))))+1)</f>
+        <f>IF(OR(B220="",COUNTIF($B$6:$B220,B220)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R220)+(($R$6:$R$305=R220)*($B$6:$B$305&lt;B220)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23040,7 +23040,7 @@
         <v/>
       </c>
       <c r="S221">
-        <f>IF(OR(B221="",COUNTIF($B$6:$B221,B221)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R221)+(($R$6:$R$305=R221)*(ROW($B$6:$B$305)&lt;ROW(B221)))))+1)</f>
+        <f>IF(OR(B221="",COUNTIF($B$6:$B221,B221)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R221)+(($R$6:$R$305=R221)*($B$6:$B$305&lt;B221)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23062,7 +23062,7 @@
         <v/>
       </c>
       <c r="S222">
-        <f>IF(OR(B222="",COUNTIF($B$6:$B222,B222)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R222)+(($R$6:$R$305=R222)*(ROW($B$6:$B$305)&lt;ROW(B222)))))+1)</f>
+        <f>IF(OR(B222="",COUNTIF($B$6:$B222,B222)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R222)+(($R$6:$R$305=R222)*($B$6:$B$305&lt;B222)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23084,7 +23084,7 @@
         <v/>
       </c>
       <c r="S223">
-        <f>IF(OR(B223="",COUNTIF($B$6:$B223,B223)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R223)+(($R$6:$R$305=R223)*(ROW($B$6:$B$305)&lt;ROW(B223)))))+1)</f>
+        <f>IF(OR(B223="",COUNTIF($B$6:$B223,B223)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R223)+(($R$6:$R$305=R223)*($B$6:$B$305&lt;B223)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23106,7 +23106,7 @@
         <v/>
       </c>
       <c r="S224">
-        <f>IF(OR(B224="",COUNTIF($B$6:$B224,B224)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R224)+(($R$6:$R$305=R224)*(ROW($B$6:$B$305)&lt;ROW(B224)))))+1)</f>
+        <f>IF(OR(B224="",COUNTIF($B$6:$B224,B224)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R224)+(($R$6:$R$305=R224)*($B$6:$B$305&lt;B224)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23128,7 +23128,7 @@
         <v/>
       </c>
       <c r="S225">
-        <f>IF(OR(B225="",COUNTIF($B$6:$B225,B225)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R225)+(($R$6:$R$305=R225)*(ROW($B$6:$B$305)&lt;ROW(B225)))))+1)</f>
+        <f>IF(OR(B225="",COUNTIF($B$6:$B225,B225)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R225)+(($R$6:$R$305=R225)*($B$6:$B$305&lt;B225)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23150,7 +23150,7 @@
         <v/>
       </c>
       <c r="S226">
-        <f>IF(OR(B226="",COUNTIF($B$6:$B226,B226)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R226)+(($R$6:$R$305=R226)*(ROW($B$6:$B$305)&lt;ROW(B226)))))+1)</f>
+        <f>IF(OR(B226="",COUNTIF($B$6:$B226,B226)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R226)+(($R$6:$R$305=R226)*($B$6:$B$305&lt;B226)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23172,7 +23172,7 @@
         <v/>
       </c>
       <c r="S227">
-        <f>IF(OR(B227="",COUNTIF($B$6:$B227,B227)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R227)+(($R$6:$R$305=R227)*(ROW($B$6:$B$305)&lt;ROW(B227)))))+1)</f>
+        <f>IF(OR(B227="",COUNTIF($B$6:$B227,B227)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R227)+(($R$6:$R$305=R227)*($B$6:$B$305&lt;B227)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23194,7 +23194,7 @@
         <v/>
       </c>
       <c r="S228">
-        <f>IF(OR(B228="",COUNTIF($B$6:$B228,B228)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R228)+(($R$6:$R$305=R228)*(ROW($B$6:$B$305)&lt;ROW(B228)))))+1)</f>
+        <f>IF(OR(B228="",COUNTIF($B$6:$B228,B228)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R228)+(($R$6:$R$305=R228)*($B$6:$B$305&lt;B228)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23216,7 +23216,7 @@
         <v/>
       </c>
       <c r="S229">
-        <f>IF(OR(B229="",COUNTIF($B$6:$B229,B229)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R229)+(($R$6:$R$305=R229)*(ROW($B$6:$B$305)&lt;ROW(B229)))))+1)</f>
+        <f>IF(OR(B229="",COUNTIF($B$6:$B229,B229)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R229)+(($R$6:$R$305=R229)*($B$6:$B$305&lt;B229)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23238,7 +23238,7 @@
         <v/>
       </c>
       <c r="S230">
-        <f>IF(OR(B230="",COUNTIF($B$6:$B230,B230)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R230)+(($R$6:$R$305=R230)*(ROW($B$6:$B$305)&lt;ROW(B230)))))+1)</f>
+        <f>IF(OR(B230="",COUNTIF($B$6:$B230,B230)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R230)+(($R$6:$R$305=R230)*($B$6:$B$305&lt;B230)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23260,7 +23260,7 @@
         <v/>
       </c>
       <c r="S231">
-        <f>IF(OR(B231="",COUNTIF($B$6:$B231,B231)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R231)+(($R$6:$R$305=R231)*(ROW($B$6:$B$305)&lt;ROW(B231)))))+1)</f>
+        <f>IF(OR(B231="",COUNTIF($B$6:$B231,B231)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R231)+(($R$6:$R$305=R231)*($B$6:$B$305&lt;B231)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23282,7 +23282,7 @@
         <v/>
       </c>
       <c r="S232">
-        <f>IF(OR(B232="",COUNTIF($B$6:$B232,B232)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R232)+(($R$6:$R$305=R232)*(ROW($B$6:$B$305)&lt;ROW(B232)))))+1)</f>
+        <f>IF(OR(B232="",COUNTIF($B$6:$B232,B232)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R232)+(($R$6:$R$305=R232)*($B$6:$B$305&lt;B232)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23304,7 +23304,7 @@
         <v/>
       </c>
       <c r="S233">
-        <f>IF(OR(B233="",COUNTIF($B$6:$B233,B233)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R233)+(($R$6:$R$305=R233)*(ROW($B$6:$B$305)&lt;ROW(B233)))))+1)</f>
+        <f>IF(OR(B233="",COUNTIF($B$6:$B233,B233)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R233)+(($R$6:$R$305=R233)*($B$6:$B$305&lt;B233)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23326,7 +23326,7 @@
         <v/>
       </c>
       <c r="S234">
-        <f>IF(OR(B234="",COUNTIF($B$6:$B234,B234)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R234)+(($R$6:$R$305=R234)*(ROW($B$6:$B$305)&lt;ROW(B234)))))+1)</f>
+        <f>IF(OR(B234="",COUNTIF($B$6:$B234,B234)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R234)+(($R$6:$R$305=R234)*($B$6:$B$305&lt;B234)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23348,7 +23348,7 @@
         <v/>
       </c>
       <c r="S235">
-        <f>IF(OR(B235="",COUNTIF($B$6:$B235,B235)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R235)+(($R$6:$R$305=R235)*(ROW($B$6:$B$305)&lt;ROW(B235)))))+1)</f>
+        <f>IF(OR(B235="",COUNTIF($B$6:$B235,B235)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R235)+(($R$6:$R$305=R235)*($B$6:$B$305&lt;B235)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23370,7 +23370,7 @@
         <v/>
       </c>
       <c r="S236">
-        <f>IF(OR(B236="",COUNTIF($B$6:$B236,B236)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R236)+(($R$6:$R$305=R236)*(ROW($B$6:$B$305)&lt;ROW(B236)))))+1)</f>
+        <f>IF(OR(B236="",COUNTIF($B$6:$B236,B236)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R236)+(($R$6:$R$305=R236)*($B$6:$B$305&lt;B236)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23392,7 +23392,7 @@
         <v/>
       </c>
       <c r="S237">
-        <f>IF(OR(B237="",COUNTIF($B$6:$B237,B237)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R237)+(($R$6:$R$305=R237)*(ROW($B$6:$B$305)&lt;ROW(B237)))))+1)</f>
+        <f>IF(OR(B237="",COUNTIF($B$6:$B237,B237)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R237)+(($R$6:$R$305=R237)*($B$6:$B$305&lt;B237)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23414,7 +23414,7 @@
         <v/>
       </c>
       <c r="S238">
-        <f>IF(OR(B238="",COUNTIF($B$6:$B238,B238)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R238)+(($R$6:$R$305=R238)*(ROW($B$6:$B$305)&lt;ROW(B238)))))+1)</f>
+        <f>IF(OR(B238="",COUNTIF($B$6:$B238,B238)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R238)+(($R$6:$R$305=R238)*($B$6:$B$305&lt;B238)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23436,7 +23436,7 @@
         <v/>
       </c>
       <c r="S239">
-        <f>IF(OR(B239="",COUNTIF($B$6:$B239,B239)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R239)+(($R$6:$R$305=R239)*(ROW($B$6:$B$305)&lt;ROW(B239)))))+1)</f>
+        <f>IF(OR(B239="",COUNTIF($B$6:$B239,B239)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R239)+(($R$6:$R$305=R239)*($B$6:$B$305&lt;B239)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23458,7 +23458,7 @@
         <v/>
       </c>
       <c r="S240">
-        <f>IF(OR(B240="",COUNTIF($B$6:$B240,B240)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R240)+(($R$6:$R$305=R240)*(ROW($B$6:$B$305)&lt;ROW(B240)))))+1)</f>
+        <f>IF(OR(B240="",COUNTIF($B$6:$B240,B240)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R240)+(($R$6:$R$305=R240)*($B$6:$B$305&lt;B240)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23480,7 +23480,7 @@
         <v/>
       </c>
       <c r="S241">
-        <f>IF(OR(B241="",COUNTIF($B$6:$B241,B241)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R241)+(($R$6:$R$305=R241)*(ROW($B$6:$B$305)&lt;ROW(B241)))))+1)</f>
+        <f>IF(OR(B241="",COUNTIF($B$6:$B241,B241)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R241)+(($R$6:$R$305=R241)*($B$6:$B$305&lt;B241)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23502,7 +23502,7 @@
         <v/>
       </c>
       <c r="S242">
-        <f>IF(OR(B242="",COUNTIF($B$6:$B242,B242)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R242)+(($R$6:$R$305=R242)*(ROW($B$6:$B$305)&lt;ROW(B242)))))+1)</f>
+        <f>IF(OR(B242="",COUNTIF($B$6:$B242,B242)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R242)+(($R$6:$R$305=R242)*($B$6:$B$305&lt;B242)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23524,7 +23524,7 @@
         <v/>
       </c>
       <c r="S243">
-        <f>IF(OR(B243="",COUNTIF($B$6:$B243,B243)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R243)+(($R$6:$R$305=R243)*(ROW($B$6:$B$305)&lt;ROW(B243)))))+1)</f>
+        <f>IF(OR(B243="",COUNTIF($B$6:$B243,B243)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R243)+(($R$6:$R$305=R243)*($B$6:$B$305&lt;B243)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23546,7 +23546,7 @@
         <v/>
       </c>
       <c r="S244">
-        <f>IF(OR(B244="",COUNTIF($B$6:$B244,B244)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R244)+(($R$6:$R$305=R244)*(ROW($B$6:$B$305)&lt;ROW(B244)))))+1)</f>
+        <f>IF(OR(B244="",COUNTIF($B$6:$B244,B244)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R244)+(($R$6:$R$305=R244)*($B$6:$B$305&lt;B244)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23568,7 +23568,7 @@
         <v/>
       </c>
       <c r="S245">
-        <f>IF(OR(B245="",COUNTIF($B$6:$B245,B245)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R245)+(($R$6:$R$305=R245)*(ROW($B$6:$B$305)&lt;ROW(B245)))))+1)</f>
+        <f>IF(OR(B245="",COUNTIF($B$6:$B245,B245)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R245)+(($R$6:$R$305=R245)*($B$6:$B$305&lt;B245)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23590,7 +23590,7 @@
         <v/>
       </c>
       <c r="S246">
-        <f>IF(OR(B246="",COUNTIF($B$6:$B246,B246)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R246)+(($R$6:$R$305=R246)*(ROW($B$6:$B$305)&lt;ROW(B246)))))+1)</f>
+        <f>IF(OR(B246="",COUNTIF($B$6:$B246,B246)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R246)+(($R$6:$R$305=R246)*($B$6:$B$305&lt;B246)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23612,7 +23612,7 @@
         <v/>
       </c>
       <c r="S247">
-        <f>IF(OR(B247="",COUNTIF($B$6:$B247,B247)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R247)+(($R$6:$R$305=R247)*(ROW($B$6:$B$305)&lt;ROW(B247)))))+1)</f>
+        <f>IF(OR(B247="",COUNTIF($B$6:$B247,B247)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R247)+(($R$6:$R$305=R247)*($B$6:$B$305&lt;B247)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23634,7 +23634,7 @@
         <v/>
       </c>
       <c r="S248">
-        <f>IF(OR(B248="",COUNTIF($B$6:$B248,B248)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R248)+(($R$6:$R$305=R248)*(ROW($B$6:$B$305)&lt;ROW(B248)))))+1)</f>
+        <f>IF(OR(B248="",COUNTIF($B$6:$B248,B248)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R248)+(($R$6:$R$305=R248)*($B$6:$B$305&lt;B248)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23656,7 +23656,7 @@
         <v/>
       </c>
       <c r="S249">
-        <f>IF(OR(B249="",COUNTIF($B$6:$B249,B249)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R249)+(($R$6:$R$305=R249)*(ROW($B$6:$B$305)&lt;ROW(B249)))))+1)</f>
+        <f>IF(OR(B249="",COUNTIF($B$6:$B249,B249)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R249)+(($R$6:$R$305=R249)*($B$6:$B$305&lt;B249)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23678,7 +23678,7 @@
         <v/>
       </c>
       <c r="S250">
-        <f>IF(OR(B250="",COUNTIF($B$6:$B250,B250)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R250)+(($R$6:$R$305=R250)*(ROW($B$6:$B$305)&lt;ROW(B250)))))+1)</f>
+        <f>IF(OR(B250="",COUNTIF($B$6:$B250,B250)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R250)+(($R$6:$R$305=R250)*($B$6:$B$305&lt;B250)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23700,7 +23700,7 @@
         <v/>
       </c>
       <c r="S251">
-        <f>IF(OR(B251="",COUNTIF($B$6:$B251,B251)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R251)+(($R$6:$R$305=R251)*(ROW($B$6:$B$305)&lt;ROW(B251)))))+1)</f>
+        <f>IF(OR(B251="",COUNTIF($B$6:$B251,B251)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R251)+(($R$6:$R$305=R251)*($B$6:$B$305&lt;B251)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23722,7 +23722,7 @@
         <v/>
       </c>
       <c r="S252">
-        <f>IF(OR(B252="",COUNTIF($B$6:$B252,B252)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R252)+(($R$6:$R$305=R252)*(ROW($B$6:$B$305)&lt;ROW(B252)))))+1)</f>
+        <f>IF(OR(B252="",COUNTIF($B$6:$B252,B252)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R252)+(($R$6:$R$305=R252)*($B$6:$B$305&lt;B252)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23744,7 +23744,7 @@
         <v/>
       </c>
       <c r="S253">
-        <f>IF(OR(B253="",COUNTIF($B$6:$B253,B253)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R253)+(($R$6:$R$305=R253)*(ROW($B$6:$B$305)&lt;ROW(B253)))))+1)</f>
+        <f>IF(OR(B253="",COUNTIF($B$6:$B253,B253)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R253)+(($R$6:$R$305=R253)*($B$6:$B$305&lt;B253)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23766,7 +23766,7 @@
         <v/>
       </c>
       <c r="S254">
-        <f>IF(OR(B254="",COUNTIF($B$6:$B254,B254)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R254)+(($R$6:$R$305=R254)*(ROW($B$6:$B$305)&lt;ROW(B254)))))+1)</f>
+        <f>IF(OR(B254="",COUNTIF($B$6:$B254,B254)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R254)+(($R$6:$R$305=R254)*($B$6:$B$305&lt;B254)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23788,7 +23788,7 @@
         <v/>
       </c>
       <c r="S255">
-        <f>IF(OR(B255="",COUNTIF($B$6:$B255,B255)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R255)+(($R$6:$R$305=R255)*(ROW($B$6:$B$305)&lt;ROW(B255)))))+1)</f>
+        <f>IF(OR(B255="",COUNTIF($B$6:$B255,B255)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R255)+(($R$6:$R$305=R255)*($B$6:$B$305&lt;B255)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23810,7 +23810,7 @@
         <v/>
       </c>
       <c r="S256">
-        <f>IF(OR(B256="",COUNTIF($B$6:$B256,B256)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R256)+(($R$6:$R$305=R256)*(ROW($B$6:$B$305)&lt;ROW(B256)))))+1)</f>
+        <f>IF(OR(B256="",COUNTIF($B$6:$B256,B256)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R256)+(($R$6:$R$305=R256)*($B$6:$B$305&lt;B256)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23832,7 +23832,7 @@
         <v/>
       </c>
       <c r="S257">
-        <f>IF(OR(B257="",COUNTIF($B$6:$B257,B257)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R257)+(($R$6:$R$305=R257)*(ROW($B$6:$B$305)&lt;ROW(B257)))))+1)</f>
+        <f>IF(OR(B257="",COUNTIF($B$6:$B257,B257)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R257)+(($R$6:$R$305=R257)*($B$6:$B$305&lt;B257)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23854,7 +23854,7 @@
         <v/>
       </c>
       <c r="S258">
-        <f>IF(OR(B258="",COUNTIF($B$6:$B258,B258)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R258)+(($R$6:$R$305=R258)*(ROW($B$6:$B$305)&lt;ROW(B258)))))+1)</f>
+        <f>IF(OR(B258="",COUNTIF($B$6:$B258,B258)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R258)+(($R$6:$R$305=R258)*($B$6:$B$305&lt;B258)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23876,7 +23876,7 @@
         <v/>
       </c>
       <c r="S259">
-        <f>IF(OR(B259="",COUNTIF($B$6:$B259,B259)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R259)+(($R$6:$R$305=R259)*(ROW($B$6:$B$305)&lt;ROW(B259)))))+1)</f>
+        <f>IF(OR(B259="",COUNTIF($B$6:$B259,B259)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R259)+(($R$6:$R$305=R259)*($B$6:$B$305&lt;B259)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23898,7 +23898,7 @@
         <v/>
       </c>
       <c r="S260">
-        <f>IF(OR(B260="",COUNTIF($B$6:$B260,B260)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R260)+(($R$6:$R$305=R260)*(ROW($B$6:$B$305)&lt;ROW(B260)))))+1)</f>
+        <f>IF(OR(B260="",COUNTIF($B$6:$B260,B260)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R260)+(($R$6:$R$305=R260)*($B$6:$B$305&lt;B260)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23920,7 +23920,7 @@
         <v/>
       </c>
       <c r="S261">
-        <f>IF(OR(B261="",COUNTIF($B$6:$B261,B261)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R261)+(($R$6:$R$305=R261)*(ROW($B$6:$B$305)&lt;ROW(B261)))))+1)</f>
+        <f>IF(OR(B261="",COUNTIF($B$6:$B261,B261)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R261)+(($R$6:$R$305=R261)*($B$6:$B$305&lt;B261)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23942,7 +23942,7 @@
         <v/>
       </c>
       <c r="S262">
-        <f>IF(OR(B262="",COUNTIF($B$6:$B262,B262)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R262)+(($R$6:$R$305=R262)*(ROW($B$6:$B$305)&lt;ROW(B262)))))+1)</f>
+        <f>IF(OR(B262="",COUNTIF($B$6:$B262,B262)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R262)+(($R$6:$R$305=R262)*($B$6:$B$305&lt;B262)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23964,7 +23964,7 @@
         <v/>
       </c>
       <c r="S263">
-        <f>IF(OR(B263="",COUNTIF($B$6:$B263,B263)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R263)+(($R$6:$R$305=R263)*(ROW($B$6:$B$305)&lt;ROW(B263)))))+1)</f>
+        <f>IF(OR(B263="",COUNTIF($B$6:$B263,B263)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R263)+(($R$6:$R$305=R263)*($B$6:$B$305&lt;B263)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -23986,7 +23986,7 @@
         <v/>
       </c>
       <c r="S264">
-        <f>IF(OR(B264="",COUNTIF($B$6:$B264,B264)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R264)+(($R$6:$R$305=R264)*(ROW($B$6:$B$305)&lt;ROW(B264)))))+1)</f>
+        <f>IF(OR(B264="",COUNTIF($B$6:$B264,B264)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R264)+(($R$6:$R$305=R264)*($B$6:$B$305&lt;B264)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24008,7 +24008,7 @@
         <v/>
       </c>
       <c r="S265">
-        <f>IF(OR(B265="",COUNTIF($B$6:$B265,B265)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R265)+(($R$6:$R$305=R265)*(ROW($B$6:$B$305)&lt;ROW(B265)))))+1)</f>
+        <f>IF(OR(B265="",COUNTIF($B$6:$B265,B265)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R265)+(($R$6:$R$305=R265)*($B$6:$B$305&lt;B265)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24030,7 +24030,7 @@
         <v/>
       </c>
       <c r="S266">
-        <f>IF(OR(B266="",COUNTIF($B$6:$B266,B266)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R266)+(($R$6:$R$305=R266)*(ROW($B$6:$B$305)&lt;ROW(B266)))))+1)</f>
+        <f>IF(OR(B266="",COUNTIF($B$6:$B266,B266)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R266)+(($R$6:$R$305=R266)*($B$6:$B$305&lt;B266)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24052,7 +24052,7 @@
         <v/>
       </c>
       <c r="S267">
-        <f>IF(OR(B267="",COUNTIF($B$6:$B267,B267)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R267)+(($R$6:$R$305=R267)*(ROW($B$6:$B$305)&lt;ROW(B267)))))+1)</f>
+        <f>IF(OR(B267="",COUNTIF($B$6:$B267,B267)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R267)+(($R$6:$R$305=R267)*($B$6:$B$305&lt;B267)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24074,7 +24074,7 @@
         <v/>
       </c>
       <c r="S268">
-        <f>IF(OR(B268="",COUNTIF($B$6:$B268,B268)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R268)+(($R$6:$R$305=R268)*(ROW($B$6:$B$305)&lt;ROW(B268)))))+1)</f>
+        <f>IF(OR(B268="",COUNTIF($B$6:$B268,B268)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R268)+(($R$6:$R$305=R268)*($B$6:$B$305&lt;B268)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24096,7 +24096,7 @@
         <v/>
       </c>
       <c r="S269">
-        <f>IF(OR(B269="",COUNTIF($B$6:$B269,B269)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R269)+(($R$6:$R$305=R269)*(ROW($B$6:$B$305)&lt;ROW(B269)))))+1)</f>
+        <f>IF(OR(B269="",COUNTIF($B$6:$B269,B269)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R269)+(($R$6:$R$305=R269)*($B$6:$B$305&lt;B269)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24118,7 +24118,7 @@
         <v/>
       </c>
       <c r="S270">
-        <f>IF(OR(B270="",COUNTIF($B$6:$B270,B270)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R270)+(($R$6:$R$305=R270)*(ROW($B$6:$B$305)&lt;ROW(B270)))))+1)</f>
+        <f>IF(OR(B270="",COUNTIF($B$6:$B270,B270)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R270)+(($R$6:$R$305=R270)*($B$6:$B$305&lt;B270)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24140,7 +24140,7 @@
         <v/>
       </c>
       <c r="S271">
-        <f>IF(OR(B271="",COUNTIF($B$6:$B271,B271)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R271)+(($R$6:$R$305=R271)*(ROW($B$6:$B$305)&lt;ROW(B271)))))+1)</f>
+        <f>IF(OR(B271="",COUNTIF($B$6:$B271,B271)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R271)+(($R$6:$R$305=R271)*($B$6:$B$305&lt;B271)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24162,7 +24162,7 @@
         <v/>
       </c>
       <c r="S272">
-        <f>IF(OR(B272="",COUNTIF($B$6:$B272,B272)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R272)+(($R$6:$R$305=R272)*(ROW($B$6:$B$305)&lt;ROW(B272)))))+1)</f>
+        <f>IF(OR(B272="",COUNTIF($B$6:$B272,B272)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R272)+(($R$6:$R$305=R272)*($B$6:$B$305&lt;B272)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24184,7 +24184,7 @@
         <v/>
       </c>
       <c r="S273">
-        <f>IF(OR(B273="",COUNTIF($B$6:$B273,B273)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R273)+(($R$6:$R$305=R273)*(ROW($B$6:$B$305)&lt;ROW(B273)))))+1)</f>
+        <f>IF(OR(B273="",COUNTIF($B$6:$B273,B273)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R273)+(($R$6:$R$305=R273)*($B$6:$B$305&lt;B273)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24206,7 +24206,7 @@
         <v/>
       </c>
       <c r="S274">
-        <f>IF(OR(B274="",COUNTIF($B$6:$B274,B274)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R274)+(($R$6:$R$305=R274)*(ROW($B$6:$B$305)&lt;ROW(B274)))))+1)</f>
+        <f>IF(OR(B274="",COUNTIF($B$6:$B274,B274)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R274)+(($R$6:$R$305=R274)*($B$6:$B$305&lt;B274)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24228,7 +24228,7 @@
         <v/>
       </c>
       <c r="S275">
-        <f>IF(OR(B275="",COUNTIF($B$6:$B275,B275)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R275)+(($R$6:$R$305=R275)*(ROW($B$6:$B$305)&lt;ROW(B275)))))+1)</f>
+        <f>IF(OR(B275="",COUNTIF($B$6:$B275,B275)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R275)+(($R$6:$R$305=R275)*($B$6:$B$305&lt;B275)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24250,7 +24250,7 @@
         <v/>
       </c>
       <c r="S276">
-        <f>IF(OR(B276="",COUNTIF($B$6:$B276,B276)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R276)+(($R$6:$R$305=R276)*(ROW($B$6:$B$305)&lt;ROW(B276)))))+1)</f>
+        <f>IF(OR(B276="",COUNTIF($B$6:$B276,B276)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R276)+(($R$6:$R$305=R276)*($B$6:$B$305&lt;B276)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24272,7 +24272,7 @@
         <v/>
       </c>
       <c r="S277">
-        <f>IF(OR(B277="",COUNTIF($B$6:$B277,B277)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R277)+(($R$6:$R$305=R277)*(ROW($B$6:$B$305)&lt;ROW(B277)))))+1)</f>
+        <f>IF(OR(B277="",COUNTIF($B$6:$B277,B277)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R277)+(($R$6:$R$305=R277)*($B$6:$B$305&lt;B277)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24294,7 +24294,7 @@
         <v/>
       </c>
       <c r="S278">
-        <f>IF(OR(B278="",COUNTIF($B$6:$B278,B278)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R278)+(($R$6:$R$305=R278)*(ROW($B$6:$B$305)&lt;ROW(B278)))))+1)</f>
+        <f>IF(OR(B278="",COUNTIF($B$6:$B278,B278)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R278)+(($R$6:$R$305=R278)*($B$6:$B$305&lt;B278)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24316,7 +24316,7 @@
         <v/>
       </c>
       <c r="S279">
-        <f>IF(OR(B279="",COUNTIF($B$6:$B279,B279)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R279)+(($R$6:$R$305=R279)*(ROW($B$6:$B$305)&lt;ROW(B279)))))+1)</f>
+        <f>IF(OR(B279="",COUNTIF($B$6:$B279,B279)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R279)+(($R$6:$R$305=R279)*($B$6:$B$305&lt;B279)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24338,7 +24338,7 @@
         <v/>
       </c>
       <c r="S280">
-        <f>IF(OR(B280="",COUNTIF($B$6:$B280,B280)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R280)+(($R$6:$R$305=R280)*(ROW($B$6:$B$305)&lt;ROW(B280)))))+1)</f>
+        <f>IF(OR(B280="",COUNTIF($B$6:$B280,B280)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R280)+(($R$6:$R$305=R280)*($B$6:$B$305&lt;B280)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24360,7 +24360,7 @@
         <v/>
       </c>
       <c r="S281">
-        <f>IF(OR(B281="",COUNTIF($B$6:$B281,B281)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R281)+(($R$6:$R$305=R281)*(ROW($B$6:$B$305)&lt;ROW(B281)))))+1)</f>
+        <f>IF(OR(B281="",COUNTIF($B$6:$B281,B281)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R281)+(($R$6:$R$305=R281)*($B$6:$B$305&lt;B281)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24382,7 +24382,7 @@
         <v/>
       </c>
       <c r="S282">
-        <f>IF(OR(B282="",COUNTIF($B$6:$B282,B282)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R282)+(($R$6:$R$305=R282)*(ROW($B$6:$B$305)&lt;ROW(B282)))))+1)</f>
+        <f>IF(OR(B282="",COUNTIF($B$6:$B282,B282)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R282)+(($R$6:$R$305=R282)*($B$6:$B$305&lt;B282)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24404,7 +24404,7 @@
         <v/>
       </c>
       <c r="S283">
-        <f>IF(OR(B283="",COUNTIF($B$6:$B283,B283)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R283)+(($R$6:$R$305=R283)*(ROW($B$6:$B$305)&lt;ROW(B283)))))+1)</f>
+        <f>IF(OR(B283="",COUNTIF($B$6:$B283,B283)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R283)+(($R$6:$R$305=R283)*($B$6:$B$305&lt;B283)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24426,7 +24426,7 @@
         <v/>
       </c>
       <c r="S284">
-        <f>IF(OR(B284="",COUNTIF($B$6:$B284,B284)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R284)+(($R$6:$R$305=R284)*(ROW($B$6:$B$305)&lt;ROW(B284)))))+1)</f>
+        <f>IF(OR(B284="",COUNTIF($B$6:$B284,B284)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R284)+(($R$6:$R$305=R284)*($B$6:$B$305&lt;B284)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24448,7 +24448,7 @@
         <v/>
       </c>
       <c r="S285">
-        <f>IF(OR(B285="",COUNTIF($B$6:$B285,B285)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R285)+(($R$6:$R$305=R285)*(ROW($B$6:$B$305)&lt;ROW(B285)))))+1)</f>
+        <f>IF(OR(B285="",COUNTIF($B$6:$B285,B285)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R285)+(($R$6:$R$305=R285)*($B$6:$B$305&lt;B285)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24470,7 +24470,7 @@
         <v/>
       </c>
       <c r="S286">
-        <f>IF(OR(B286="",COUNTIF($B$6:$B286,B286)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R286)+(($R$6:$R$305=R286)*(ROW($B$6:$B$305)&lt;ROW(B286)))))+1)</f>
+        <f>IF(OR(B286="",COUNTIF($B$6:$B286,B286)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R286)+(($R$6:$R$305=R286)*($B$6:$B$305&lt;B286)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24492,7 +24492,7 @@
         <v/>
       </c>
       <c r="S287">
-        <f>IF(OR(B287="",COUNTIF($B$6:$B287,B287)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R287)+(($R$6:$R$305=R287)*(ROW($B$6:$B$305)&lt;ROW(B287)))))+1)</f>
+        <f>IF(OR(B287="",COUNTIF($B$6:$B287,B287)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R287)+(($R$6:$R$305=R287)*($B$6:$B$305&lt;B287)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24514,7 +24514,7 @@
         <v/>
       </c>
       <c r="S288">
-        <f>IF(OR(B288="",COUNTIF($B$6:$B288,B288)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R288)+(($R$6:$R$305=R288)*(ROW($B$6:$B$305)&lt;ROW(B288)))))+1)</f>
+        <f>IF(OR(B288="",COUNTIF($B$6:$B288,B288)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R288)+(($R$6:$R$305=R288)*($B$6:$B$305&lt;B288)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24536,7 +24536,7 @@
         <v/>
       </c>
       <c r="S289">
-        <f>IF(OR(B289="",COUNTIF($B$6:$B289,B289)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R289)+(($R$6:$R$305=R289)*(ROW($B$6:$B$305)&lt;ROW(B289)))))+1)</f>
+        <f>IF(OR(B289="",COUNTIF($B$6:$B289,B289)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R289)+(($R$6:$R$305=R289)*($B$6:$B$305&lt;B289)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24558,7 +24558,7 @@
         <v/>
       </c>
       <c r="S290">
-        <f>IF(OR(B290="",COUNTIF($B$6:$B290,B290)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R290)+(($R$6:$R$305=R290)*(ROW($B$6:$B$305)&lt;ROW(B290)))))+1)</f>
+        <f>IF(OR(B290="",COUNTIF($B$6:$B290,B290)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R290)+(($R$6:$R$305=R290)*($B$6:$B$305&lt;B290)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24580,7 +24580,7 @@
         <v/>
       </c>
       <c r="S291">
-        <f>IF(OR(B291="",COUNTIF($B$6:$B291,B291)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R291)+(($R$6:$R$305=R291)*(ROW($B$6:$B$305)&lt;ROW(B291)))))+1)</f>
+        <f>IF(OR(B291="",COUNTIF($B$6:$B291,B291)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R291)+(($R$6:$R$305=R291)*($B$6:$B$305&lt;B291)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24602,7 +24602,7 @@
         <v/>
       </c>
       <c r="S292">
-        <f>IF(OR(B292="",COUNTIF($B$6:$B292,B292)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R292)+(($R$6:$R$305=R292)*(ROW($B$6:$B$305)&lt;ROW(B292)))))+1)</f>
+        <f>IF(OR(B292="",COUNTIF($B$6:$B292,B292)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R292)+(($R$6:$R$305=R292)*($B$6:$B$305&lt;B292)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24624,7 +24624,7 @@
         <v/>
       </c>
       <c r="S293">
-        <f>IF(OR(B293="",COUNTIF($B$6:$B293,B293)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R293)+(($R$6:$R$305=R293)*(ROW($B$6:$B$305)&lt;ROW(B293)))))+1)</f>
+        <f>IF(OR(B293="",COUNTIF($B$6:$B293,B293)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R293)+(($R$6:$R$305=R293)*($B$6:$B$305&lt;B293)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24646,7 +24646,7 @@
         <v/>
       </c>
       <c r="S294">
-        <f>IF(OR(B294="",COUNTIF($B$6:$B294,B294)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R294)+(($R$6:$R$305=R294)*(ROW($B$6:$B$305)&lt;ROW(B294)))))+1)</f>
+        <f>IF(OR(B294="",COUNTIF($B$6:$B294,B294)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R294)+(($R$6:$R$305=R294)*($B$6:$B$305&lt;B294)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24668,7 +24668,7 @@
         <v/>
       </c>
       <c r="S295">
-        <f>IF(OR(B295="",COUNTIF($B$6:$B295,B295)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R295)+(($R$6:$R$305=R295)*(ROW($B$6:$B$305)&lt;ROW(B295)))))+1)</f>
+        <f>IF(OR(B295="",COUNTIF($B$6:$B295,B295)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R295)+(($R$6:$R$305=R295)*($B$6:$B$305&lt;B295)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24690,7 +24690,7 @@
         <v/>
       </c>
       <c r="S296">
-        <f>IF(OR(B296="",COUNTIF($B$6:$B296,B296)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R296)+(($R$6:$R$305=R296)*(ROW($B$6:$B$305)&lt;ROW(B296)))))+1)</f>
+        <f>IF(OR(B296="",COUNTIF($B$6:$B296,B296)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R296)+(($R$6:$R$305=R296)*($B$6:$B$305&lt;B296)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24712,7 +24712,7 @@
         <v/>
       </c>
       <c r="S297">
-        <f>IF(OR(B297="",COUNTIF($B$6:$B297,B297)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R297)+(($R$6:$R$305=R297)*(ROW($B$6:$B$305)&lt;ROW(B297)))))+1)</f>
+        <f>IF(OR(B297="",COUNTIF($B$6:$B297,B297)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R297)+(($R$6:$R$305=R297)*($B$6:$B$305&lt;B297)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24734,7 +24734,7 @@
         <v/>
       </c>
       <c r="S298">
-        <f>IF(OR(B298="",COUNTIF($B$6:$B298,B298)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R298)+(($R$6:$R$305=R298)*(ROW($B$6:$B$305)&lt;ROW(B298)))))+1)</f>
+        <f>IF(OR(B298="",COUNTIF($B$6:$B298,B298)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R298)+(($R$6:$R$305=R298)*($B$6:$B$305&lt;B298)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24756,7 +24756,7 @@
         <v/>
       </c>
       <c r="S299">
-        <f>IF(OR(B299="",COUNTIF($B$6:$B299,B299)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R299)+(($R$6:$R$305=R299)*(ROW($B$6:$B$305)&lt;ROW(B299)))))+1)</f>
+        <f>IF(OR(B299="",COUNTIF($B$6:$B299,B299)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R299)+(($R$6:$R$305=R299)*($B$6:$B$305&lt;B299)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24778,7 +24778,7 @@
         <v/>
       </c>
       <c r="S300">
-        <f>IF(OR(B300="",COUNTIF($B$6:$B300,B300)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R300)+(($R$6:$R$305=R300)*(ROW($B$6:$B$305)&lt;ROW(B300)))))+1)</f>
+        <f>IF(OR(B300="",COUNTIF($B$6:$B300,B300)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R300)+(($R$6:$R$305=R300)*($B$6:$B$305&lt;B300)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24800,7 +24800,7 @@
         <v/>
       </c>
       <c r="S301">
-        <f>IF(OR(B301="",COUNTIF($B$6:$B301,B301)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R301)+(($R$6:$R$305=R301)*(ROW($B$6:$B$305)&lt;ROW(B301)))))+1)</f>
+        <f>IF(OR(B301="",COUNTIF($B$6:$B301,B301)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R301)+(($R$6:$R$305=R301)*($B$6:$B$305&lt;B301)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24822,7 +24822,7 @@
         <v/>
       </c>
       <c r="S302">
-        <f>IF(OR(B302="",COUNTIF($B$6:$B302,B302)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R302)+(($R$6:$R$305=R302)*(ROW($B$6:$B$305)&lt;ROW(B302)))))+1)</f>
+        <f>IF(OR(B302="",COUNTIF($B$6:$B302,B302)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R302)+(($R$6:$R$305=R302)*($B$6:$B$305&lt;B302)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24844,7 +24844,7 @@
         <v/>
       </c>
       <c r="S303">
-        <f>IF(OR(B303="",COUNTIF($B$6:$B303,B303)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R303)+(($R$6:$R$305=R303)*(ROW($B$6:$B$305)&lt;ROW(B303)))))+1)</f>
+        <f>IF(OR(B303="",COUNTIF($B$6:$B303,B303)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R303)+(($R$6:$R$305=R303)*($B$6:$B$305&lt;B303)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24866,7 +24866,7 @@
         <v/>
       </c>
       <c r="S304">
-        <f>IF(OR(B304="",COUNTIF($B$6:$B304,B304)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R304)+(($R$6:$R$305=R304)*(ROW($B$6:$B$305)&lt;ROW(B304)))))+1)</f>
+        <f>IF(OR(B304="",COUNTIF($B$6:$B304,B304)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R304)+(($R$6:$R$305=R304)*($B$6:$B$305&lt;B304)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>
@@ -24888,7 +24888,7 @@
         <v/>
       </c>
       <c r="S305">
-        <f>IF(OR(B305="",COUNTIF($B$6:$B305,B305)&gt;1),"",SUMPRODUCT((MATCH($B$6:$B$305,$B$6:$B$305,0)=ROW($B$6:$B$305)-ROW($B$5))*($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R305)+(($R$6:$R$305=R305)*(ROW($B$6:$B$305)&lt;ROW(B305)))))+1)</f>
+        <f>IF(OR(B305="",COUNTIF($B$6:$B305,B305)&gt;1),"",ROUND(SUMPRODUCT(($B$6:$B$305&lt;&gt;"")*(($R$6:$R$305&gt;R305)+(($R$6:$R$305=R305)*($B$6:$B$305&lt;B305)))/COUNTIF($B$6:$B$305,$B$6:$B$305)),0)+1)</f>
         <v/>
       </c>
     </row>

</xml_diff>